<commit_message>
Update state - 2026-09-07
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K189" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K206" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K264" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K310" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,14 +462,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K189"/>
+  <dimension ref="A1:K206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -8909,17 +8909,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr"/>
-      <c r="C183" t="inlineStr"/>
       <c r="D183" s="3" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
           <t>August 31, 2026</t>
         </is>
       </c>
-      <c r="F183" t="inlineStr"/>
-      <c r="G183" t="inlineStr"/>
-      <c r="H183" t="inlineStr"/>
       <c r="I183" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -9008,7 +9003,6 @@
           <t>11:45 AM EDT</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316283308/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
@@ -9036,17 +9030,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr"/>
-      <c r="C186" t="inlineStr"/>
       <c r="D186" s="3" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
           <t>August 31, 2026</t>
         </is>
       </c>
-      <c r="F186" t="inlineStr"/>
-      <c r="G186" t="inlineStr"/>
-      <c r="H186" t="inlineStr"/>
       <c r="I186" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -9082,7 +9071,6 @@
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr">
         <is>
           <t>https://atlanta.aitinkerers.org/p/agents-everywhere-bots-channels-more-global-hackathon</t>
@@ -9203,6 +9191,813 @@
       <c r="K189" s="2" t="inlineStr">
         <is>
           <t>Multi-day AI/data conference hosted by Georgia's official AI office in Atlanta with clear AI focus in the title, meeting all criteria for excellent fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>The Modern Sales Strategy presented by TAG Sales Leadership Society</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>5</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>8:00 AM - 10:00 AM</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/R1F2vZvsRC0CX</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>Join the TAG Sales Leadership Society for "The Modern Sales Team", an executive-level conversation examining how AI is reshaping the people and organizational model behind B2B growth.</t>
+        </is>
+      </c>
+      <c r="K190" s="2" t="inlineStr">
+        <is>
+          <t>TAG event with genuine AI content (AI reshaping sales strategy and organizational models), and TAG events with AI content score 5 regardless of virtual-only format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>TAG DS&amp;AI Society Summit: The AI-Powered Enterprise</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>5</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="n">
+        <v>46343</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>8:00 AM - 4:30 PM</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/OOFvaqjSaCqCD</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>The TAG Data Science &amp; AI Summit 2026 is a full-day Atlanta experience connecting executive strategy with applied implementation.</t>
+        </is>
+      </c>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>This is a TAG Data Science &amp; AI Society event with explicit AI content (executive strategy and applied AI implementation), hosted by TAG in Atlanta as an in-person full-day conference, which meets the criteria for a TAG event with genuine AI content that scores 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr"/>
+      <c r="C192" t="inlineStr"/>
+      <c r="D192" s="3" t="inlineStr"/>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr"/>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr"/>
+      <c r="K192" s="2" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr"/>
+      <c r="C193" t="inlineStr"/>
+      <c r="D193" s="3" t="inlineStr"/>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr"/>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr"/>
+      <c r="K193" s="2" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>How AI Changes IT Timelines &amp; Project Estimates</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>2</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>3:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/how-ai-changes-it-timelines-project-estimates-tickets-1998364048664?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr">
+        <is>
+          <t>A webinar exploring how AI accelerates code generation but impacts project timelines. Learn why traditional estimation models fail with AI, discover hidden costs of refactoring and integration, and gain frameworks to set realistic budgets and delivery dates for AI-driven development teams.</t>
+        </is>
+      </c>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>This is a virtual-only webinar with genuine AI content (addressing how AI impacts software development timelines), but it lacks a Georgia organizational tie and appears to be hosted on Eventbrite Canada with no stated Georgia focus, placing it below the threshold for higher scoring despite clear AI relevance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>AI Builders Meetup | September 10th</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>4</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Jamestowne · 11675 Rainwater Dr suite 100</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-builders-meetup-september-10th-tickets-1998165454664?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr">
+        <is>
+          <t>A live show-and-tell for builders where 5-7 AI builders share what they're building, their approach, tools and tech stacks, and lessons learned. Includes presentations, Q&amp;A, and networking. For founders, entrepreneurs, product managers, software engineers, and AI enthusiasts.</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI-focused educational event in Georgia (Jamestowne location) with genuine AI builder content (presentations, Q&amp;A, networking) that is open to public registration and not a sales pitch, though it lacks explicit TAG affiliation or multi-day conference status that would elevate it to a 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>AI Connect Expo</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>3</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D196" s="3" t="inlineStr"/>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-connect-expo-tickets-1990471467742?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr">
+        <is>
+          <t>AI Connect Expo brings together enterprise leaders, AI innovators, and solution providers to explore applied AI, automation, data-driven decision-making, intelligent operations, and practical AI use across business transformation.</t>
+        </is>
+      </c>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
+          <t>Event has genuine AI content (applied AI, automation, data-driven decision-making) and appears to be in-person, but missing critical details like date, location, and host organization prevent higher scoring, and the thin listing leaves uncertainty about whether this is a legitimate conference or a vendor-focused sales event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>BEYOND CHATGPT: ENTERPRISE AI SYSTEMS FOR HIGH PERFORMANCE AGENTS</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>3</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="n">
+        <v>46272</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Georgia · Maximum One Executives - Duluth</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/beyond-chatgpt-enterprise-ai-systems-for-high-performance-agents-tickets-1994019439822?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr"/>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t>The title contains clear AI content (enterprise AI systems, high-performance agents) and the event is in-person in Georgia (Duluth), but the completely empty short description leaves uncertainty about whether this is a genuine educational event, a sales pitch, or something else, and the thin details prevent higher confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>AI Design Basics: Canva, Gemini &amp; Beyond</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>3</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Whitlock · Switzer Library</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-design-basics-canva-gemini-beyond-tickets-1997722549924?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t>Get ready to dive into AI-powered design tools like Canva and Gemini to boost your creative game.</t>
+        </is>
+      </c>
+      <c r="K198" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (Gemini, AI-powered design tools) and is in-person at a Georgia location (Whitlock-Switzer Library, likely University of Georgia), but the description is brief and tool-focused rather than deeply educational, and lacks confirmation of the host organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>The AI Avatar Bootcamp</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>3</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Hills Park · The Bakery CoWork</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/the-ai-avatar-bootcamp-tickets-1999873599772?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t>An immersive, hands-on bootcamp where you'll learn to create a realistic digital version of yourself, generate on-brand photos and content, and use AI to make content creation easier and more consistent. Bring your laptop and leave with your AI Avatar in motion.</t>
+        </is>
+      </c>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (digital avatar creation, AI-generated content) and is in-person in Georgia, but it reads as a paid bootcamp/workshop with a commercial angle rather than an educational conference or industry discussion, and the thin description limits confidence in assessing depth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Houzz Pro AI &amp; 3D Design Tech Lunch and Learn!</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>2</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Blandtown · AuthenTEAK</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/houzz-pro-ai-3d-design-tech-lunch-and-learn-tickets-1998227936549?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>A private seminar for designers exploring AI, 3D, and Houzz Pro technology. Learn about AI applications in construction and design, how 3D and computer vision AI are changing designer sales, and how to leverage these tools in Houzz Pro. Lunch and beverages included.</t>
+        </is>
+      </c>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (AI applications in construction/design, 3D and computer vision AI) but is a sales-focused lunch-and-learn for Houzz Pro's own platform in Atlanta, resembling a product pitch rather than educational content, and lacks Georgia organizational ties beyond location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Wednesd.AI</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>2</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>Free weekly Wednesday morning show-and-tell where community builders demonstrate how they use AI in their work. Featured speakers take 30 minutes to show their AI tools, workflows, and lessons learned, followed by open co-working until noon. Built for founders, operators, and builders in tech.</t>
+        </is>
+      </c>
+      <c r="K201" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (demonstrations of AI tools and workflows), but is virtual-only with no stated Georgia host or organizational tie, making it ineligible for the higher scoring that would apply to in-person Georgia events or those hosted by Georgia-based organizations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>AI in Action: Implementation Work Session</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>3</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Griffin · 416 E Taylor St</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-in-action-implementation-work-session-tickets-1999392753548?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>A hands-on session where participants dive into putting AI concepts into practice. Collaborate, troubleshoot, and make AI work in real-world scenarios. Bring your ideas, questions, and enthusiasm.</t>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t>The event has clear AI content (implementation and real-world applications) and is in-person in Griffin, Georgia (outside metro Atlanta), but the thin description and lack of specific technical detail or speaker information limits confidence and prevents a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>IIEX AI 2026: The Future of AI in Insights Is Back Again!</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>2</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>11:00 PM GMT+4</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr"/>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/iiex-ai-2026-the-future-of-ai-in-insights-is-back-again-tickets-1984389543543?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>Explore real AI use cases and how AI is being applied across the insights lifecycle. For forward-thinking insights, analytics, and strategy professionals to discover generative workflows, AI-powered synthesis, and how leaders can adapt early to AI's impact on research.</t>
+        </is>
+      </c>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>Event has genuine AI content focused on generative workflows and AI-powered synthesis, but is virtual-only with no Georgia host or tie, scoring it at the virtual-only cap of 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>10 Essential AI Agents Every Engineer Must Build</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>2</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr"/>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/10-essential-ai-agents-every-engineer-must-build-tickets-1992470369511?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t>A hands-on workshop where participants build 10 production-inspired AI agents across Finance, Healthcare, Education, multimodal AI, and autonomous systems. Learn AI agent engineering through practical implementation, from single-agent reasoning to multi-agent orchestration and embodied AI.</t>
+        </is>
+      </c>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t>Event has strong AI content (AI agents, multi-agent systems, embodied AI) but is virtual-only with no Georgia host or connection, making it ineligible for higher scoring under the virtual-only rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>2</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="n">
+        <v>46273</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Linwood Heights · East Point Library</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t>A weekly hands-on program introducing youth and teens to robotics, artificial intelligence, engineering thinking, and creative problem-solving. Students will explore real robots, virtual robotics environments, and beginner-friendly AI tools while completing challenges that build confidence and technical skills.</t>
+        </is>
+      </c>
+      <c r="K205" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics and STEM outreach program that mentions AI tools but centers on hands-on robotics building and challenges rather than genuine AI learning (machine perception, autonomy, or algorithmic depth), making it primarily a robotics event that happens to include AI exposure; the in-person Georgia location (East Point) does not overcome the robotics-focused nature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Claude Ecosystem for Marketers: A 3-Part Online Series with Certification</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>2</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr"/>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/claude-ecosystem-for-marketers-a-3-part-online-series-with-certification-tickets-1996907071807?aff=ebdsoporgprofile</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t>A practitioner-led series for marketers who want to use Claude well. Three 90-minute live sessions covering Claude 101, Cowork, Design and Code. Each session stands alone and builds on the last. Certificate of completion awarded.</t>
+        </is>
+      </c>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t>This is a virtual-only AI training event (Claude, an AI tool) with no Georgia host or tie, making it capped at 2 per the virtual-only scoring rule; while it has genuine AI content, it appears to be paid training rather than an educational conference, and lacks any Georgia connection.</t>
         </is>
       </c>
     </row>
@@ -9220,14 +10015,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K264"/>
+  <dimension ref="A1:K310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -21806,7 +22601,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G259" t="inlineStr"/>
       <c r="H259" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/georgia-rural-health-transformation-presented-by-tag-digital-health-society-1910658?sourceTypeId=Website</t>
@@ -21855,7 +22649,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G260" t="inlineStr"/>
       <c r="H260" t="inlineStr">
         <is>
           <t>https://www.meetup.com/refactr-tech/events/315893352/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
@@ -21957,7 +22750,6 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr"/>
       <c r="H262" t="inlineStr">
         <is>
           <t>https://www.meetup.com/python-atlanta/events/315306147/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
@@ -22006,7 +22798,6 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
-      <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr">
         <is>
           <t>https://www.meetup.com/freeside-atlanta/events/316117768/?recId=ba055001-537f-408c-aeec-a7416042e864&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=2a6a602b-d05d-460f-8066-0a8cd22e8068&amp;eventOrigin=find_page%24all</t>
@@ -22078,6 +22869,2246 @@
       <c r="K264" s="2" t="inlineStr">
         <is>
           <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a Nostr (a decentralized social protocol) meetup with tool building and discussion, which falls outside the AI criteria despite being hosted by ATL BitLab, a Georgia organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>The Opportunity Room presented by TAG Diversity, Equity &amp; Inclusion Society</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>1</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>5:30 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr"/>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/J5F2yjQCJCzC3</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="inlineStr"/>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a TAG Diversity, Equity &amp; Inclusion Society event with no stated AI content, so it receives an automatic 1 regardless of the TAG host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Security in the Cloud: Zero Trust for the Modern Software Lifecycle presented by TAG Cloud Society</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>1</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D266" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>5:30 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr"/>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/security-in-the-cloud-zero-trust-for-the-modern-software-lifecycle-presented-by-tag-cloud-society-1912017?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr"/>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is about cloud security and zero trust architecture, which are infrastructure/security topics unrelated to AI, triggering the automatic-1 rule despite being hosted by TAG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>ResearchersConnect: Global Virtual Job &amp; Networking Event for Researchers</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>1</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>4:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ac-atl/events/304913274/?recId=ad718422-8382-4f67-8e86-06d3dde46ded&amp;recSource=ml-popular-events-nearby-online&amp;searchId=e101ec45-586d-4824-8d44-c622ed89a791&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr"/>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Atlanta Tech Meet-Up</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>1</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr"/>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atl-tech-meetup/events/316377666/?recId=ad718422-8382-4f67-8e86-06d3dde46ded&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=e101ec45-586d-4824-8d44-c622ed89a791&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J268" s="2" t="inlineStr">
+        <is>
+          <t>Connect with fellow tech professionals and gain insights into the latest developments in technology. Each month features a distinguished guest speaker sharing expertise and industry knowledge. Complimentary pizza and beverages provided.</t>
+        </is>
+      </c>
+      <c r="K268" s="2" t="inlineStr">
+        <is>
+          <t>The event description mentions no AI, machine learning, automation, or any specific technical topic—it is a generic tech meetup with an unspecified guest speaker, triggering the automatic-1 rule for events with zero AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Civic Action Night at Tech Square ATL (TSQATL) Social Club</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>1</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Tech Square ATL</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/civictechatlanta/events/313899230/?recId=ad718422-8382-4f67-8e86-06d3dde46ded&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=e101ec45-586d-4824-8d44-c622ed89a791&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr"/>
+      <c r="K269" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rule; it appears to be a general civic tech networking event with no stated AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>How AI Transforms Product Design &amp; Manufacturing | VRINGON FREE WEBINAR</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>1</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>9:00 AM GMT+9</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/how-ai-transforms-product-design-manufacturing-vringon-free-webinar-tickets-1998459597453?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>Join RebuilderAI for a live technology update on VRINGON, an AI-powered platform transforming product development from design to manufacturing. Discover the latest capabilities in AI Design, 3D Engineering, Parametric CAD, Simulation, Manufacturing Automation, and Physical AI, with live demonstrations of how AI can accelerate product development and reduce time to market.</t>
+        </is>
+      </c>
+      <c r="K270" s="2" t="inlineStr">
+        <is>
+          <t>This is a virtual-only webinar with no Georgia host or tie, hosted by RebuilderAI (a company promoting its own VRINGON platform), qualifying as a heavy-handed sales pitch for the organizer's core business rather than an educational AI event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Build an App with AI: Create Your First CRM Without Coding</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>1</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>7:00 PM GMT+8</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr"/>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.sg/e/build-an-app-with-ai-create-your-first-crm-without-coding-tickets-1999335429089?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr"/>
+      <c r="K271" s="2" t="inlineStr">
+        <is>
+          <t>Event is virtual-only with no Georgia host or organizational tie, hosted on Eventbrite Singapore with a Singapore timezone, making it a national/international corporate offering with no Georgia connection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>God, Science, and Our Search for Meaning</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>1</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D272" s="3" t="n">
+        <v>46276</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Young Harris · O. Wayne Rollins Planetarium</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/god-science-and-our-search-for-meaning-tickets-1994321679830?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr"/>
+      <c r="K272" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Tech North Atlanta Awards, Sponsored by Improving</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>1</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Chattahoochee Terrace · Topgolf Alpharetta</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tech-north-atlanta-awards-sponsored-by-improving-tickets-1988425179238?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr"/>
+      <c r="K273" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it is an awards ceremony with no stated AI-focused component, session, or speaker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Citizen Science For Everyone: Intro to iNaturalist &amp; Plant ID Ramble</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>1</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D274" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>1:30 PM</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Toco Hills Town Center · Vista Yoga</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/citizen-science-for-everyone-intro-to-inaturalist-plant-id-ramble-tickets-1999165083581?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="inlineStr"/>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is about citizen science, iNaturalist (a species identification platform), and plant identification, with no stated AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Tissue Culture 101: A Beginner's Workshop</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>1</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Lakewood Heights · The Plant Apothecary</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tissue-culture-101-a-beginners-workshop-tickets-1995194886615?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr"/>
+      <c r="K275" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Women + Tech Meetup</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>1</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D276" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>North Buckhead · Atlanta Tech Village</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/women-tech-meetup-tickets-1979762040557?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr"/>
+      <c r="K276" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>10 week Cybersecurity &amp; Tech Career Training for High School (ages 15-18)</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>1</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D277" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Jonesboro · Perry Learning Center</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/10-week-cybersecurity-tech-career-training-for-high-school-ages-15-18-tickets-1998638045195?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="inlineStr"/>
+      <c r="K277" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—only cybersecurity and general tech career training—triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Cloud Connect Expo</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>1</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="n">
+        <v>46274</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Downtown · Georgia World Congress Center</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/cloud-connect-expo-tickets-1990472121698?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>Cloud Connect Expo explores cloud infrastructure, security, migration, and scalable technologies driving digital transformation. Brings together enterprise leaders, cloud innovators, and solution providers to explore cloud security, migration, data infrastructure, and technologies powering digital transformation.</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>The event description makes no mention of AI, machine learning, or automation—it focuses on cloud infrastructure, security, and migration as general topics without any AI-specific component, session, speaker, or theme stated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>STEM Family Sundays at iFLY Atlanta!</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>1</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D279" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Cumberland Bridge · iFLY Indoor Skydiving - Atlanta</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/stem-family-sundays-at-ifly-atlanta-tickets-1991765472144?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr"/>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a recreational skydiving activity branded as a STEM family event with no stated AI component, triggering the automatic 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026 Girls in Aviation Day - Attendee Sign-Up</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>1</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="inlineStr"/>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr"/>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Covington · Covington Municipal Airport</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/2026-girls-in-aviation-day-attendee-sign-up-tickets-1988931449506?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr"/>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, and Girls in Aviation Day is a youth STEM outreach event focused on aviation careers and experience rather than AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Dr. Beronda L. Montgomery in conversation with Dr. Na'Taki Osborne Jelks</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>1</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Oakland City · Trees Atlanta</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/dr-beronda-l-montgomery-in-conversation-with-dr-nataki-osborne-jelks-tickets-1997615001243?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>Join 44th &amp; 3rd as we host Dr. Beronda L. Montgomery, author of When Trees Testify, in conversation with Dr. Na'Taki Osborne Jelks. Montgomery is a writer, science communicator, and researcher who has spent over 20 years as a professor studying photosynthetic organisms and mentorship in academia.</t>
+        </is>
+      </c>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a book talk about photosynthesis and academic mentorship, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Standard BioTools Augusta University seminar</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>1</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Augusta Downtown Historic District · Georgia Cancer Center - M. Bert Storey Research Building</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/standard-biotools-augusta-university-seminar-tickets-1997904724814?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="inlineStr"/>
+      <c r="K282" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Intro to Beekeeping</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>1</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Leila Valley · 2370 Locust Ln SE</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/intro-to-beekeeping-tickets-1998236746901?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr"/>
+      <c r="K283" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Hack ITP: A hackathon for builders</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>1</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>North Buckhead · Atlanta Tech Village - Buckhead</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/hack-itp-a-hackathon-for-builders-tickets-1999030811971?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>A two-day hackathon bringing tech pros, students and creatives together. Opening ceremonies start Saturday morning with team matching and vibe coding credits available. Judging happens Sunday afternoon with closing ceremonies before 6:00 PM. Open to students, software engineers, product strategists, creatives, artists and designers.</t>
+        </is>
+      </c>
+      <c r="K284" s="2" t="inlineStr">
+        <is>
+          <t>The event description makes no mention of AI, machine learning, or automation—it is a general hackathon for builders with no stated AI-focused component, session, or theme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Honeybee Hive Tour</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>1</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D285" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Avondale · 1830 Shepherd Dr</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/honeybee-hive-tour-tickets-1986742680840?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr"/>
+      <c r="K285" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>MICROLOCK SELF RETIGHTENING MADE EASY!</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>1</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="n">
+        <v>46278</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>North Atlanta · 705 Town Blvd</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/microlock-self-retightening-made-easy-tickets-1903263234569?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr"/>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it appears to be about mechanical fasteners—triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>WBU Athens: Charlie Elliott presentation on Raptors</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>1</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D287" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Beechwood Hills · Wild Birds Unlimited</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wbu-athens-charlie-elliott-presentation-on-raptors-tickets-1990651233426?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr"/>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation - it is a presentation about raptors by Wild Birds Unlimited, which triggers the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Black Boys Code DeKalb - Think Like a Coder: Your First Algorithm</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>1</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D288" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Clifton Community · Emory University</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/black-boys-code-dekalb-think-like-a-coder-your-first-algorithm-tickets-1999299193708?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>A hands-on LEGO Robotics workshop for boys aged 8-17. Beginners learn sequencing and motor control while building moving robotic machines. Advanced learners explore engineering concepts, robotic subsystems, and Python programming. All materials provided free of charge.</t>
+        </is>
+      </c>
+      <c r="K288" s="2" t="inlineStr">
+        <is>
+          <t>This is a LEGO robotics build workshop focused on hardware construction and motor control rather than AI content; while advanced learners touch Python programming, the event's core is robotics competition/build-focused, not AI-centered machine learning or autonomy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Black Boys Code Gwinnett County - Think Like a Coder: Your First Algorithm</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>1</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D289" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Village Gate · Georgia Gwinnett College</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/black-boys-code-gwinnett-county-think-like-a-coder-your-first-algorithm-tickets-1999298598929?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>A hands-on LEGO Robotics workshop for boys aged 8-17. Beginners learn sequencing and basic programming with SPIKE Prime, while advanced learners explore Python programming and engineering concepts. All materials provided free of charge.</t>
+        </is>
+      </c>
+      <c r="K289" s="2" t="inlineStr">
+        <is>
+          <t>This is a LEGO Robotics build-a-bot workshop focused on hardware construction and basic sequencing rather than AI/machine learning content, and robotics competitions and hands-on build events score 1 per the criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>In Depth Compost Process and Material Use Training for Growers</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>1</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>East Point · 2366 Sylvan Rd</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/in-depth-compost-process-and-material-use-training-for-growers-tickets-1998899962597?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr"/>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of location or other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Neuroregeneration and Fatty Acids</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>1</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D291" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Egan Park · College Park Library</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/neuroregeneration-and-fatty-acids-tickets-1988725529594?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="inlineStr"/>
+      <c r="K291" s="2" t="inlineStr">
+        <is>
+          <t>The event title and available description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Internet Basics</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>1</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D292" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Mableton · South Cobb Regional Library</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/internet-basics-tickets-1997053496768?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="inlineStr"/>
+      <c r="K292" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>FORESTRY RESOURCE MANAGEMENT WORKSHOP ( Taylor County )</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>1</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D293" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Georgia · 89 Pebble Rd</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/forestry-resource-management-workshop-taylor-county-tickets-1996187083302?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="inlineStr"/>
+      <c r="K293" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Gmail Basics for Adults</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>1</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr"/>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/gmail-basics-for-adults-tickets-1997720178832?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr"/>
+      <c r="K294" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Stonecrest AeroBots Drone Soccer Program</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>1</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Georgia · Browns Mill Recreation Center</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/stonecrest-aerobots-drone-soccer-program-tickets-1996102035923?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="inlineStr"/>
+      <c r="K295" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics build/competition program focused on drone hardware and soccer gameplay rather than AI, machine learning, or automation concepts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Black Boys Code Atlanta - Think Like a Coder: Your First Algorithm</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>1</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D296" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Sylvan Hills · Atlanta Metropolitan State College (Building 100)</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/black-boys-code-atlanta-think-like-a-coder-your-first-algorithm-tickets-1999298188702?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="inlineStr"/>
+      <c r="K296" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is a basic coding/algorithm introduction for youth, which triggers the automatic-1 rule regardless of the host or location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Animal Skull Study</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>1</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D297" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>North Point · Chattahoochee Nature Center</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/animal-skull-study-tickets-1998675449071?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J297" s="2" t="inlineStr"/>
+      <c r="K297" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Android Basics for Adults</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>1</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D298" s="3" t="n">
+        <v>46275</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr"/>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/android-basics-for-adults-tickets-1997595113759?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J298" s="2" t="inlineStr"/>
+      <c r="K298" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>DSC and IQ Training Day</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>1</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Rose Garden Hills · 2270 Northwest Parkway Southeast, Marietta, GA, USA</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/dsc-and-iq-training-day-tickets-1997971823508?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>Product &amp; Sales Training covering IQ Panel 5, PowerG Automation, PowerG + Water Tile &amp; IQ Pro with Santiago Rivera and Zeb Shrader. Learn about DSC (Digital Security Controls), a world leader in electronic security known for revolutionary control panels, IP alarm monitoring products, and wireless panels.</t>
+        </is>
+      </c>
+      <c r="K299" s="2" t="inlineStr">
+        <is>
+          <t>This is a product and sales training event for DSC security control panels and automation systems with no mention of AI, machine learning, or automation in the AI sense—it covers hardware products and sales techniques, not AI technology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Westside (Shirley Clarke Franklin) Park Bioblitz</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>1</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D300" s="3" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Rockdale · Westside Park Parking II</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/westside-shirley-clarke-franklin-park-bioblitz-tickets-1998933803817?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J300" s="2" t="inlineStr"/>
+      <c r="K300" s="2" t="inlineStr">
+        <is>
+          <t>The event is a bioblitz (biodiversity survey activity) with zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>iPhone Basics for Adults</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>1</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D301" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/iphone-basics-for-adults-tickets-1997720404507?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="inlineStr"/>
+      <c r="K301" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Forestry Resource Management Workshop ( Swainsboro, Ga)</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>1</v>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D302" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Georgia · 24 Jarrett Durden Rd</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/forestry-resource-management-workshop-swainsboro-ga-tickets-1998399812635?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr"/>
+      <c r="K302" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is a forestry resource management workshop with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>1</v>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D303" s="3" t="n">
+        <v>46273</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="inlineStr"/>
+      <c r="K303" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>FREE DevOps Bootcamp | USA Only | Join WhatsApp Group</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>1</v>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D304" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>8:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-devops-bootcamp-usa-only-join-whatsapp-group-tickets-1996843006185?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="inlineStr"/>
+      <c r="K304" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; DevOps bootcamp content is unrelated to AI regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Chicken Basics #3: Are Chickens Geologists?</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>1</v>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D305" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Thornwood · Theron Ussery Community Center</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/chicken-basics-3-are-chickens-geologists-tickets-1999530764342?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="inlineStr"/>
+      <c r="K305" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Stellar Evolution: Lifecycle of a Star!</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>1</v>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D306" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Grove Park · Dogwood Library</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/stellar-evolution-lifecycle-of-a-star-tickets-1999299152585?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="inlineStr"/>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is about stellar astronomy and the lifecycle of stars, making it an automatic 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Stormwater Education Program</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>1</v>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D307" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Whitlock · Cobb County Water Lab Training Room</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/stormwater-education-program-tickets-1995485724519?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr"/>
+      <c r="K307" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Adopt-A-Stream Bacterial Monitoring Workshop</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>1</v>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D308" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>6:30 PM</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr"/>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/adopt-a-stream-bacterial-monitoring-workshop-tickets-1995474593225?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr"/>
+      <c r="K308" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or available description, making it an automatic 1 per the scoring criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Code The Culture</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>1</v>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="n">
+        <v>46273</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Downtown · Best Buy Teen Tech Center</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/code-the-culture-tickets-1999945715472?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>A one-hour creator session for Atlanta teens where music meets real engineering. Dive into coding and tech in a fun, relaxed setting at the Best Buy Teen Tech Center.</t>
+        </is>
+      </c>
+      <c r="K309" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it describes a creator session about music and coding for teens with no AI-focused component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Virtual Training Series: Vibe Code Your Own Marketing Tool with Lovable</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>1</v>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D310" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>September 7, 2026</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/virtual-training-series-vibe-code-your-own-marketing-tool-with-lovable-tickets-1996918680529?aff=ebdsoporgprofile</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>Three 90-minute virtual sessions teaching you to build your own marketing tool with Lovable. Learn vibe coding skills progressively: build a working app, test and expand it reliably, then connect to external services and publish. Includes live demonstrations, Q&amp;A, and certificate of completion.</t>
+        </is>
+      </c>
+      <c r="K310" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is about 'vibe coding' to build a marketing tool with a specific commercial platform (Lovable), which is a paid training/sales pitch with no genuine AI educational content.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-09-14
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K206" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K225" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K310" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K337" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,14 +462,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K206"/>
+  <dimension ref="A1:K225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -9221,7 +9221,6 @@
           <t>8:00 AM - 10:00 AM</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/R1F2vZvsRC0CX</t>
@@ -9302,17 +9301,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr"/>
-      <c r="C192" t="inlineStr"/>
       <c r="D192" s="3" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
           <t>September 7, 2026</t>
         </is>
       </c>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr"/>
-      <c r="H192" t="inlineStr"/>
       <c r="I192" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -9327,17 +9321,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr"/>
-      <c r="C193" t="inlineStr"/>
       <c r="D193" s="3" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
           <t>September 7, 2026</t>
         </is>
       </c>
-      <c r="F193" t="inlineStr"/>
-      <c r="G193" t="inlineStr"/>
-      <c r="H193" t="inlineStr"/>
       <c r="I193" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -9373,7 +9362,6 @@
           <t>3:00 PM EDT</t>
         </is>
       </c>
-      <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/how-ai-changes-it-timelines-project-estimates-tickets-1998364048664?aff=ebdssbdestsearch</t>
@@ -9468,8 +9456,6 @@
           <t>September 7, 2026</t>
         </is>
       </c>
-      <c r="F196" t="inlineStr"/>
-      <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-connect-expo-tickets-1990471467742?aff=ebdssbdestsearch</t>
@@ -9726,7 +9712,6 @@
           <t>8:30 AM</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
@@ -9828,7 +9813,6 @@
           <t>11:00 PM GMT+4</t>
         </is>
       </c>
-      <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/iiex-ai-2026-the-future-of-ai-in-insights-is-back-again-tickets-1984389543543?aff=ebdssbdestsearch</t>
@@ -9877,7 +9861,6 @@
           <t>11:00 AM EDT</t>
         </is>
       </c>
-      <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/10-essential-ai-agents-every-engineer-must-build-tickets-1992470369511?aff=ebdssbdestsearch</t>
@@ -9979,7 +9962,6 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/claude-ecosystem-for-marketers-a-3-part-online-series-with-certification-tickets-1996907071807?aff=ebdsoporgprofile</t>
@@ -10000,6 +9982,905 @@
           <t>This is a virtual-only AI training event (Claude, an AI tool) with no Georgia host or tie, making it capped at 2 per the virtual-only scoring rule; while it has genuine AI content, it appears to be paid training rather than an educational conference, and lacks any Georgia connection.</t>
         </is>
       </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>AI's Hidden Environmental Cost</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>4</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Room 1222, Molecular Science &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/ais-hidden-environmental-cost</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t>Join GT's NAACP for a fun, informative discussion about data centers &amp; AI's environmental cost. Food is provided, and all students are welcome!</t>
+        </is>
+      </c>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech-hosted in-person event with genuine AI content (environmental impact of AI and data centers), open to all students with food provided, located outside metro Atlanta proper, though not a TAG event so it scores 4 rather than 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>AI for the Working Mathematician - Lunch Discussion Group</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>5</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>11:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Skiles 006</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/ai-working-mathematician-lunch-discussion-group</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t>AI for the Working Mathematician is an informal discussion group for mathematicians interested in practical ways that artificial intelligence can support mathematical research and increase productivity.</t>
+        </is>
+      </c>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech-hosted, in-person event with clear AI content (discussion of AI applications in mathematical research), satisfying both the Georgia institution criterion and substantive AI educational programming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>We, the People, and AI: The Future of Data, Energy, Health, and Human Rights</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>5</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Walter G. Ehmer Theater (Atlantic)</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/we-people-and-ai-future-data-energy-health-and-human-rights</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t>As part of the Ivan Allen College AI &amp; Society Series, this event explores the tangible physical footprint of artificial intelligence and its profound consequences for energy, health, human rights, and the future of our digital society.</t>
+        </is>
+      </c>
+      <c r="K209" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech-hosted event with explicit AI focus on its societal impacts (energy, health, human rights, digital society), in-person at a known venue, part of a named AI &amp; Society Series.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Avant South</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>1</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>12:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Tech Square, Atlanta</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/avant-south</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t>Avant South is an annual event supporting Atlanta's growth as a leading tech hub.</t>
+        </is>
+      </c>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it only describes Avant South as supporting Atlanta's growth as a tech hub generally, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>BBISS Insights Series #2 - AI for Climate Resilience</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>5</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>9:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>John Lewis Student Center - Rafael Bras Meeting Room</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/bbiss-insights-series-2-ai-climate-resilience</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t>Ali Sarhadi, Suhas Jain, and Iris Tien will discuss how AI can be leveraged to address key sustainability and resilience challenges.</t>
+        </is>
+      </c>
+      <c r="K211" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech-hosted educational event with genuine AI content (AI applications for climate resilience), in-person location in Atlanta, clear speaker lineup and topic focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>AI and Academic Research: The Future of Discovery</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>5</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="n">
+        <v>46330</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>6:30 PM EST</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Georgia Tech Hotel &amp; Conference Center – Grand Ballrooms</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/ai-and-academic-research-future-discovery</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr">
+        <is>
+          <t>As part of the Ivan Allen College AI &amp; Society Series, this event examines how artificial intelligence is reshaping academic research, from accelerating scientific discovery to navigating the ethical boundaries of modern scholarship.</t>
+        </is>
+      </c>
+      <c r="K212" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech-hosted in-person event with genuine AI content (AI's impact on academic research and ethics), part of an established AI &amp; Society Series, located outside metro Atlanta, and open to public registration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>AI, Human Empathy, and Relationships: Is AI a Better Partner?</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>5</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="n">
+        <v>46428</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>6:30 PM EST</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Historic Academy of Medicine</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/ai-human-empathy-and-relationships-ai-better-partner</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t>As part of the Ivan Allen College AI &amp; Society Series, this event explores the shifting boundaries of empathy, intimacy, and human relationships as artificial intelligence becomes increasingly emotionally responsive.</t>
+        </is>
+      </c>
+      <c r="K213" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech-hosted in-person event with genuine AI content (emotionally responsive AI systems and their social implications), part of an established AI &amp; Society Series, in a non-Atlanta location, making it an excellent fit for the statewide digest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>AI and Creativity: Creative Industries in Flux</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>5</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="n">
+        <v>46491</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Walter G. Ehmer Theater (Atlantic)</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/ai-and-creativity-creative-industries-flux</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t>Part of the Ivan Allen College AI &amp; Society Series, this panel examines how generative artificial intelligence is redefining artistic expression, authorship, and the future of labor across the creative industries.</t>
+        </is>
+      </c>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Tech-hosted panel with explicit AI content (generative AI's impact on creative industries), part of an established AI &amp; Society Series, in-person in Georgia, and clearly educational rather than sales-focused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Educational Session- Winning More Business: AI, Marketing &amp; Relationship Strategies That Drive Growth</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>4</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="n">
+        <v>46330</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>11:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr"/>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/educational-session--winning-more-business-ai-marketing-and-relationship-strategies-that-drive-growth</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t>Interactive session combining practical AI and marketing strategies with relationship-building systems to help manufacturing leaders attract prospects, strengthen market presence, and create revenue opportunities. Learn to use AI for marketing, build relationships that lead to business, create repeatable growth systems, and get practical ideas to implement immediately.</t>
+        </is>
+      </c>
+      <c r="K215" s="2" t="inlineStr">
+        <is>
+          <t>Georgia Manufacturing Alliance-hosted event with genuine AI content (AI for marketing, growth systems) positioned as practical business education rather than sales pitch, though the description emphasizes business outcomes over technical depth and lacks specific details about the AI component's scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr"/>
+      <c r="C216" t="inlineStr"/>
+      <c r="D216" s="3" t="inlineStr"/>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr"/>
+      <c r="G216" t="inlineStr"/>
+      <c r="H216" t="inlineStr"/>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr"/>
+      <c r="K216" s="2" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Monthly Meetup + Demo Night: September 2026</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>5</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr"/>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atl-ai/events/314482316/?recId=7ba65084-cd63-4897-8427-483bf5cb572c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=63a9e786-c165-4c1b-9aa4-db2c84cc2c77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t>Come see demos, learn about new tools, and more from the hackers pushing the possibilities of AI in Atlanta. The evening includes demos from presenters, networking, and board games.</t>
+        </is>
+      </c>
+      <c r="K217" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta AI Tinkerers is a Georgia-based AI community organization, the event has explicit AI content (demos from AI practitioners, tools, and hacking), is in-person and local to Atlanta, and fits the profile of an educational AI meetup that the client values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Agent-a-Thon: Build an Agent with Us</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>4</v>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D218" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr"/>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/producttank-atlanta/events/316391313/?recId=7ba65084-cd63-4897-8427-483bf5cb572c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=63a9e786-c165-4c1b-9aa4-db2c84cc2c77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a hands-on interactive agent building session. Share your AI agent ideas, vote as a group, then build the winning idea live collaboratively using Claude in VS Code. No laptop needed—ProductTank has the driving covered. Food and drinks provided!</t>
+        </is>
+      </c>
+      <c r="K218" s="2" t="inlineStr">
+        <is>
+          <t>Strong hands-on AI content (agent building with Claude) hosted by ProductTank Atlanta (Georgia tie), in-person, open public registration, though missing specific venue details and location confirmation prevents a perfect score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>GA AI Alliance Networking Lunch</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>3</v>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>11:45 AM EDT</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr"/>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316283337/?recId=7ba65084-cd63-4897-8427-483bf5cb572c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=63a9e786-c165-4c1b-9aa4-db2c84cc2c77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t>Informal networking lunch for AI professionals across Georgia. Meet others in the AI space, build connections, hear what others are doing, and learn about the monthly AI insights program. For those building with AI, driving adoption, or staying on the cutting edge.</t>
+        </is>
+      </c>
+      <c r="K219" s="2" t="inlineStr">
+        <is>
+          <t>Georgia-hosted AI networking event with genuine AI content (for AI professionals and builders), but it is a social/networking event rather than educational or technical content, and lacks a specific venue location in the listing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr"/>
+      <c r="C220" t="inlineStr"/>
+      <c r="D220" s="3" t="inlineStr"/>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr"/>
+      <c r="G220" t="inlineStr"/>
+      <c r="H220" t="inlineStr"/>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr"/>
+      <c r="K220" s="2" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>AI Vibe Coding Beginners Workshop taught by an Expert AI Builder</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>3</v>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D221" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Laurel Ridge · The Success Center 1400 Centre Pkwy</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-vibe-coding-beginners-workshop-taught-by-an-expert-ai-builder-tickets-2000613404548?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t>Hands-on workshop for beginners to learn AI coding skills from an expert builder. Build real projects, learn new platforms, and launch your first AI project in a friendly, laid-back setting.</t>
+        </is>
+      </c>
+      <c r="K221" s="2" t="inlineStr">
+        <is>
+          <t>In-person event with genuine AI coding content and hands-on learning focus, but lacking detail about organizer/host affiliation, specific curriculum depth, and whether it's primarily a sales pitch for a particular platform or service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Wednesd.AI</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>2</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr"/>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>Free weekly Wednesday morning show-and-tell where community builders demonstrate how they use AI in their work. Features 30-minute presentations followed by open co-working. Built for founders, operators, and builders to learn practical AI applications they can apply immediately.</t>
+        </is>
+      </c>
+      <c r="K222" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (practical AI applications in work), but it is virtual-only with no Georgia-based host organization mentioned, which caps it at 2 per the virtual-only scoring rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>2</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D223" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Linwood Heights · East Point Library</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>A weekly hands-on program introducing youth and teens to robotics, artificial intelligence, engineering thinking, and creative problem-solving. Students will explore real robots, virtual robotics environments, and beginner-friendly AI tools while completing challenges that build confidence and technical skills.</t>
+        </is>
+      </c>
+      <c r="K223" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics outreach/build workshop with an AI component mentioned but not as the primary focus, which per criteria scores low for robotics events; it's in-person in Georgia (East Point) which would normally help, but the core event type (youth STEM robotics program) and heavy emphasis on hands-on robot building and challenges rather than AI education as a standalone subject keep it at 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>More Done, Less Doing: How to use AI to take work OFF Your plate</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>2</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D224" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>1:00 PM CDT</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr"/>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/more-done-less-doing-how-to-use-ai-to-take-work-off-your-plate-tickets-2000183505709?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>A live 90-minute masterclass where Robert Sanberg opens his actual AI agent system that runs his company WindRider. See AI teams draft work across marketing, operations, finance, and admin, with decisions brought to humans for approval. Learn how to use AI to automate business work while maintaining human control over important decisions.</t>
+        </is>
+      </c>
+      <c r="K224" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with genuine AI content (AI agents, automation, business applications) but no Georgia organizational tie and appears to be a paid masterclass/sales pitch for the host's WindRider system, capping it below 3 per the virtual-only and sales-pitch rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr"/>
+      <c r="C225" t="inlineStr"/>
+      <c r="D225" s="3" t="inlineStr"/>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr"/>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr"/>
+      <c r="K225" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10015,14 +10896,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K310"/>
+  <dimension ref="A1:K337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
@@ -22899,7 +23780,6 @@
           <t>5:30 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr"/>
       <c r="H265" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/J5F2yjQCJCzC3</t>
@@ -22944,7 +23824,6 @@
           <t>5:30 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr"/>
       <c r="H266" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/security-in-the-cloud-zero-trust-for-the-modern-software-lifecycle-presented-by-tag-cloud-society-1912017?sourceTypeId=Website</t>
@@ -23038,7 +23917,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G268" t="inlineStr"/>
       <c r="H268" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atl-tech-meetup/events/316377666/?recId=ad718422-8382-4f67-8e86-06d3dde46ded&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=e101ec45-586d-4824-8d44-c622ed89a791&amp;eventOrigin=find_page%24all</t>
@@ -23136,7 +24014,6 @@
           <t>9:00 AM GMT+9</t>
         </is>
       </c>
-      <c r="G270" t="inlineStr"/>
       <c r="H270" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/how-ai-transforms-product-design-manufacturing-vringon-free-webinar-tickets-1998459597453?aff=ebdssbdestsearch</t>
@@ -23185,7 +24062,6 @@
           <t>7:00 PM GMT+8</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr"/>
       <c r="H271" t="inlineStr">
         <is>
           <t>https://www.eventbrite.sg/e/build-an-app-with-ai-create-your-first-crm-without-coding-tickets-1999335429089?aff=ebdssbdestsearch</t>
@@ -23619,7 +24495,6 @@
           <t>September 7, 2026</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>Covington · Covington Municipal Airport</t>
@@ -24322,7 +25197,6 @@
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="G294" t="inlineStr"/>
       <c r="H294" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/gmail-basics-for-adults-tickets-1997720178832?aff=ebdssbdestsearch</t>
@@ -24514,7 +25388,6 @@
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="G298" t="inlineStr"/>
       <c r="H298" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/android-basics-for-adults-tickets-1997595113759?aff=ebdssbdestsearch</t>
@@ -24661,7 +25534,6 @@
           <t>3:00 PM</t>
         </is>
       </c>
-      <c r="G301" t="inlineStr"/>
       <c r="H301" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/iphone-basics-for-adults-tickets-1997720404507?aff=ebdssbdestsearch</t>
@@ -24755,7 +25627,6 @@
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="G303" t="inlineStr"/>
       <c r="H303" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
@@ -24800,7 +25671,6 @@
           <t>8:30 AM EDT</t>
         </is>
       </c>
-      <c r="G304" t="inlineStr"/>
       <c r="H304" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-devops-bootcamp-usa-only-join-whatsapp-group-tickets-1996843006185?aff=ebdssbdestsearch</t>
@@ -24992,7 +25862,6 @@
           <t>6:30 PM</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr"/>
       <c r="H308" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/adopt-a-stream-bacterial-monitoring-workshop-tickets-1995474593225?aff=ebdssbdestsearch</t>
@@ -25090,7 +25959,6 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
-      <c r="G310" t="inlineStr"/>
       <c r="H310" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/virtual-training-series-vibe-code-your-own-marketing-tool-with-lovable-tickets-1996918680529?aff=ebdsoporgprofile</t>
@@ -25109,6 +25977,1325 @@
       <c r="K310" s="2" t="inlineStr">
         <is>
           <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is about 'vibe coding' to build a marketing tool with a specific commercial platform (Lovable), which is a paid training/sales pitch with no genuine AI educational content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Using Containers at PACE</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>1</v>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>10:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/using-containers-pace</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to use Apptainer to download and run Docker images, build new images using definition files, and learn tips for portable software workflows on PACE's Phoenix and Hive systems.</t>
+        </is>
+      </c>
+      <c r="K311" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is purely about containerization tools (Apptainer/Docker) and software workflow management on a computing cluster, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Using Containers at PACE</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>1</v>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D312" s="3" t="n">
+        <v>46339</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>10:30 AM EST</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/using-containers-pace-0</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to use Apptainer to download and run Docker images, build new images using definition files, and learn tips for portable software workflows on PACE's Phoenix and Hive systems.</t>
+        </is>
+      </c>
+      <c r="K312" s="2" t="inlineStr">
+        <is>
+          <t>The event describes containerization tools (Apptainer, Docker) and workflow management with no mention of AI, machine learning, or automation, triggering the automatic-1 rule despite being hosted by Georgia Tech.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Using Containers at PACE</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>1</v>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D313" s="3" t="n">
+        <v>46374</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="inlineStr"/>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/using-containers-pace-1</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J313" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to use Apptainer to download and run Docker images, build new images using definition files, and implement portable software workflows on PACE's Phoenix and Hive systems.</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is purely about container technology (Apptainer and Docker) for workflow management on computing infrastructure, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Data Center Summit presented by TAG Infrastructure Society</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>1</v>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D314" s="3" t="n">
+        <v>46358</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>4:30 PM - 8:30 PM</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/data-center-summit-presented-by-tag-infrastructure-society-1921079?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J314" s="2" t="inlineStr">
+        <is>
+          <t>The TAG Infrastructure Society is bringing together leaders from across Georgia's rapidly evolving data center ecosystem for the 2026 Data Center Summit.</t>
+        </is>
+      </c>
+      <c r="K314" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation; it is only about data centers as infrastructure, triggering the automatic-1 rule despite being hosted by TAG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Steel Materials Plant Tour- Cartersville - A.M.</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>1</v>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>9:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Cartersville, Georgia</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/steel-materials-plant-tour--cartersville-2026-am</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="inlineStr"/>
+      <c r="K315" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a plant tour with no stated AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Coffee and Connections - Atlanta 10-15-2026</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>1</v>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D316" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>8:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>Atlanta, Georgia</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/coffee-and-connections-atlanta-10-15-2026</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="inlineStr"/>
+      <c r="K316" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of the Georgia Manufacturing Alliance host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Networking Luncheon - Atlanta 10-15-2026</t>
+        </is>
+      </c>
+      <c r="B317" t="n">
+        <v>1</v>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D317" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>11:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Atlanta, Georgia</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/networking-luncheon-atlanta-10-15-2026</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J317" s="2" t="inlineStr"/>
+      <c r="K317" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of the host organization's general focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>12 For Life Plant Tour - Carrollton</t>
+        </is>
+      </c>
+      <c r="B318" t="n">
+        <v>1</v>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D318" s="3" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>1:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Carrollton, Georgia</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/12-for-life-plant-tour---carrollton</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J318" s="2" t="inlineStr"/>
+      <c r="K318" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; it is a plant tour with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Women of GMA Virtual Networking Event 11/3/26</t>
+        </is>
+      </c>
+      <c r="B319" t="n">
+        <v>1</v>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="n">
+        <v>46329</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>3:30 PM EST</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr"/>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/women-of-gma-virtual-networking-event-11326</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J319" s="2" t="inlineStr"/>
+      <c r="K319" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, and is a networking event rather than an educational or technical AI session.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Infinity Building Solutions Plant Tour</t>
+        </is>
+      </c>
+      <c r="B320" t="n">
+        <v>1</v>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D320" s="3" t="n">
+        <v>46337</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>9:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr"/>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/infinity-building-solutions-plant-tour</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J320" s="2" t="inlineStr"/>
+      <c r="K320" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of the Georgia Manufacturing Alliance host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Coffee and Connections - Atlanta 11-19-2026</t>
+        </is>
+      </c>
+      <c r="B321" t="n">
+        <v>1</v>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D321" s="3" t="n">
+        <v>46345</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>8:30 AM EST</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Atlanta, Georgia</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/coffee-and-connections-atlanta-11-19-2026</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J321" s="2" t="inlineStr"/>
+      <c r="K321" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of the Georgia Manufacturing Alliance host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Networking Luncheon - Atlanta 11-19-2026</t>
+        </is>
+      </c>
+      <c r="B322" t="n">
+        <v>1</v>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D322" s="3" t="n">
+        <v>46345</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>11:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Atlanta, Georgia</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/networking-luncheon-atlanta-11-19-2026</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J322" s="2" t="inlineStr"/>
+      <c r="K322" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of the host organization or location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Kia Georgia Plant Tour - West Point - 2026</t>
+        </is>
+      </c>
+      <c r="B323" t="n">
+        <v>1</v>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D323" s="3" t="n">
+        <v>46364</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>10:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>West Point, Georgia</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/kia-georgia-plant-tour---west-point----2026</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J323" s="2" t="inlineStr"/>
+      <c r="K323" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rule regardless of the Georgia Manufacturing Alliance host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Coffee and Connections - Atlanta 12-17-2026</t>
+        </is>
+      </c>
+      <c r="B324" t="n">
+        <v>1</v>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D324" s="3" t="n">
+        <v>46373</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>8:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>Atlanta, Georgia</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/coffee-and-connections---atlanta-12-17-2026</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J324" s="2" t="inlineStr"/>
+      <c r="K324" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of the Georgia Manufacturing Alliance host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Launch Your Cybersecurity Career- Cyber Work Role Pathways with UofL DTC</t>
+        </is>
+      </c>
+      <c r="B325" t="n">
+        <v>1</v>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D325" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>University of Louisville</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/launch-your-cybersecurity-career-cyber-work-role-pathways-with-uofl-dtc-tickets-2000523752396?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J325" s="2" t="inlineStr"/>
+      <c r="K325" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, covering only cybersecurity career pathways and roles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Cyber Security Fundamentals</t>
+        </is>
+      </c>
+      <c r="B326" t="n">
+        <v>1</v>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D326" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr"/>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/cyber-security-fundamentals-tickets-1999333344855?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J326" s="2" t="inlineStr"/>
+      <c r="K326" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Design It. Release It — Live App Building Challenge</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>1</v>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D327" s="3" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr"/>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/design-it-release-it-live-app-building-challenge-tickets-1999797091935?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J327" s="2" t="inlineStr"/>
+      <c r="K327" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is a general app building challenge with no stated AI component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>GREEN GTBOP Webinar Series - Thursday, September 17, 2026</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>1</v>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D328" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>Griffin · UGA Griffin Campus</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/green-gtbop-webinar-series-thursday-september-17-2026-registration-1999695321537?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J328" s="2" t="inlineStr">
+        <is>
+          <t>Online webinar featuring two presentations: "How excluding ants from tree canopies can aid soft-scale insect management" by Dr. Caleb Wilson, and "Pathological Issues affecting turfgrass in the southeastern US" by Dr. Jim Kerns. Includes 2 hours of continuing education credits.</t>
+        </is>
+      </c>
+      <c r="K328" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is about agricultural pest management and turfgrass pathology, triggering the automatic 1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Dahlonega Science Cafe Presentation</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>1</v>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D329" s="3" t="n">
+        <v>46279</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>Dahlonega · Bourbon Street Grille</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/dahlonega-science-cafe-presentation-tickets-1998451216385?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J329" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a monthly Science Cafe Presentation where curious minds gather to explore cool science topics in a relaxed setting. Enjoy dinner, engaging discussions, and connect over fascinating discoveries. All ages welcome.</t>
+        </is>
+      </c>
+      <c r="K329" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it is a general science cafe with no indication of AI-focused content, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>FREE Cybersecurity Bootcamp | USA Only | Live Online</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>1</v>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D330" s="3" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>8:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-cybersecurity-bootcamp-usa-only-live-online-tickets-1996169284064?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J330" s="2" t="inlineStr"/>
+      <c r="K330" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 score regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Georgia's Prehistoric Native Plants: Our 300-million-year-old Garden</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>1</v>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D331" s="3" t="n">
+        <v>46284</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Whitlock · Switzer Public Library</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/georgias-prehistoric-native-plants-our-300-million-year-old-garden-tickets-2000184343214?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="inlineStr"/>
+      <c r="K331" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description; it is about prehistoric native plants and gardening, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Meet the Bees at Food Well Farm!</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>1</v>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D332" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>Leila Valley · 2370 Locust Ln SE</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/meet-the-bees-at-food-well-farm-tickets-1999084271871?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J332" s="2" t="inlineStr"/>
+      <c r="K332" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B333" t="n">
+        <v>1</v>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D333" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr"/>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="inlineStr"/>
+      <c r="K333" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Ignite Intelligence: First Click | Ignite House Atlanta</t>
+        </is>
+      </c>
+      <c r="B334" t="n">
+        <v>1</v>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D334" s="3" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>East Washington · Ignite House</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ignite-intelligence-first-click-ignite-house-atlanta-tickets-1998573284494?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J334" s="2" t="inlineStr">
+        <is>
+          <t>A beginner-friendly technology workshop designed for people who want to become more comfortable and confident using today's digital tools. No previous experience required—learn practical tech skills in a welcoming environment and leave with greater confidence navigating the digital world.</t>
+        </is>
+      </c>
+      <c r="K334" s="2" t="inlineStr">
+        <is>
+          <t>The event description makes no mention of AI, machine learning, or automation—it is a general beginner-friendly digital tools workshop, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Hack for Humanity</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
+        <v>1</v>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D335" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>Georgia · 7035 Houston Rd</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/hack-for-humanity-tickets-2000810799963?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>Join people from across Middle Georgia to hack cool tech solutions that make the world a better place. Use your experience, ideas, creativity, and desire to make a difference to build solutions for community problems. No programming experience required.</t>
+        </is>
+      </c>
+      <c r="K335" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it is a general hackathon for community problem-solving with no stated AI-focused component, session, speaker, or theme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Preserving Privacy: Using AI in the Digital World</t>
+        </is>
+      </c>
+      <c r="B336" t="n">
+        <v>1</v>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D336" s="3" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>7:00 PM GMT+9:30</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr"/>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com.au/e/preserving-privacy-using-ai-in-the-digital-world-tickets-1998703630362?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to reclaim your digital privacy in this live webinar. Discover how to take back your data, navigate AI safely, reduce your digital footprint, find reliable information online, explore alternative browsers, and understand digital ID. Topics include strategies to opt out of unnecessary features and safely utilize AI tools.</t>
+        </is>
+      </c>
+      <c r="K336" s="2" t="inlineStr">
+        <is>
+          <t>This is a virtual-only event (explicitly marked webinar) hosted on Eventbrite Australia with no Georgia organization tie, and while it mentions AI, the focus is on privacy and data protection rather than AI/ML as a technical subject, making it a national corporate webinar outside the client's target scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Build Your Career in IT, Cloud &amp; Data-Cyber Work Role Pathways at UofL DTC</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>1</v>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D337" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>September 14, 2026</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr"/>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/build-your-career-in-it-cloud-data-cyber-work-role-pathways-at-uofl-dtc-tickets-2000531285929?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>Free virtual information session exploring career pathways in IT support, cloud/software, and data analytics. Learn about Technical Support Specialist, Software/Cloud Architect, and Data Analyst roles, plus certification opportunities, online training, portfolio building, career coaching, job placement support, and scholarships.</t>
+        </is>
+      </c>
+      <c r="K337" s="2" t="inlineStr">
+        <is>
+          <t>The event description mentions IT, cloud, data analytics, and certifications but contains zero mention of AI, machine learning, or automation, triggering the automatic-1 rule for events with no AI content.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-09-21
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K225" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K247" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K337" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K353" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K225"/>
+  <dimension ref="A1:K247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -10434,7 +10434,6 @@
           <t>11:00 AM EST</t>
         </is>
       </c>
-      <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/educational-session--winning-more-business-ai-marketing-and-relationship-strategies-that-drive-growth</t>
@@ -10462,17 +10461,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr"/>
-      <c r="C216" t="inlineStr"/>
       <c r="D216" s="3" t="inlineStr"/>
       <c r="E216" t="inlineStr">
         <is>
           <t>September 14, 2026</t>
         </is>
       </c>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr"/>
-      <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -10508,7 +10502,6 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
-      <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atl-ai/events/314482316/?recId=7ba65084-cd63-4897-8427-483bf5cb572c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=63a9e786-c165-4c1b-9aa4-db2c84cc2c77&amp;eventOrigin=find_page%24all</t>
@@ -10557,7 +10550,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr">
         <is>
           <t>https://www.meetup.com/producttank-atlanta/events/316391313/?recId=7ba65084-cd63-4897-8427-483bf5cb572c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=63a9e786-c165-4c1b-9aa4-db2c84cc2c77&amp;eventOrigin=find_page%24all</t>
@@ -10606,7 +10598,6 @@
           <t>11:45 AM EDT</t>
         </is>
       </c>
-      <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316283337/?recId=7ba65084-cd63-4897-8427-483bf5cb572c&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=63a9e786-c165-4c1b-9aa4-db2c84cc2c77&amp;eventOrigin=find_page%24all</t>
@@ -10634,17 +10625,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr"/>
-      <c r="C220" t="inlineStr"/>
       <c r="D220" s="3" t="inlineStr"/>
       <c r="E220" t="inlineStr">
         <is>
           <t>September 14, 2026</t>
         </is>
       </c>
-      <c r="F220" t="inlineStr"/>
-      <c r="G220" t="inlineStr"/>
-      <c r="H220" t="inlineStr"/>
       <c r="I220" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -10733,7 +10719,6 @@
           <t>8:30 AM</t>
         </is>
       </c>
-      <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
@@ -10835,7 +10820,6 @@
           <t>1:00 PM CDT</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/more-done-less-doing-how-to-use-ai-to-take-work-off-your-plate-tickets-2000183505709?aff=ebdssbdestsearch</t>
@@ -10863,17 +10847,12 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
-      <c r="B225" t="inlineStr"/>
-      <c r="C225" t="inlineStr"/>
       <c r="D225" s="3" t="inlineStr"/>
       <c r="E225" t="inlineStr">
         <is>
           <t>September 14, 2026</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr"/>
-      <c r="G225" t="inlineStr"/>
-      <c r="H225" t="inlineStr"/>
       <c r="I225" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -10881,6 +10860,1032 @@
       </c>
       <c r="J225" s="2" t="inlineStr"/>
       <c r="K225" s="2" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>The Modern GTM Team presented by TAG Sales Leadership Society</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>5</v>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>8:00 AM - 10:00 AM</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr"/>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/R1F2vZvsRC0CX</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>Join the TAG Sales Leadership Society for "The Modern Sales Team", an executive-level conversation examining how AI is reshaping the people and organizational model behind B2B growth.</t>
+        </is>
+      </c>
+      <c r="K226" s="2" t="inlineStr">
+        <is>
+          <t>TAG event with genuine AI content (AI reshaping sales organizations and B2B growth models) qualifies for the automatic 5 score per TAG uplift rule, despite being virtual-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>The Human Side of AI: Who's the Boss? Responsibility and Accountability with Agentic AI? presented by TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>5</v>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr"/>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/KVF3Bv1snCBCW</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>Discover how organizations can preserve accountability, trust, and responsible governance—while unlocking the full potential of agentic AI.</t>
+        </is>
+      </c>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>This is a TAG Data Science &amp; AI Society event with genuine AI content (agentic AI, responsibility, accountability) that qualifies for the automatic TAG uplift, and the Georgia-based host organization ensures it meets the client's prioritized criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>TAG Digital Health Hackathon</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>3</v>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D228" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>2:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr"/>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/YEFn9vxTNCzCK</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>The TAG Digital Health Hackathon will bring together students, developers, clinicians, engineers, and designers to build innovative tech solutions for modern healthcare.</t>
+        </is>
+      </c>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>TAG-hosted event with genuine potential for AI content (hackathon for tech solutions in healthcare could involve ML/automation), but the description lacks explicit AI mention, and virtual-only status limits scoring despite TAG affiliation and Georgia tie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Executive Exchange presented by TAG Data Governance Society</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>5</v>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="n">
+        <v>46359</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>5:00 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr"/>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/executive-exchange-presented-by-tag-data-governance-society-1929065?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>Data Governance and AI Governance are inseparable. This session shows executives how to align both disciplines into a unified governance strategy that enables responsible innovation. Key topics include building a trusted data foundation for AI, governing AI models for fairness and accountability, anticipating regulations, and linking governance to customer trust and business value.</t>
+        </is>
+      </c>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>TAG Data Governance Society event with genuine AI content (AI governance, model fairness, responsible innovation) hosted by Georgia's premier tech organization; TAG events with AI content score 5 regardless of virtual format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Educational Session- Winning More Business: AI, Marketing &amp; Relationship Strategies that Drive Growth</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>3</v>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="n">
+        <v>46330</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>11:00 AM - 1:30 PM EST</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr"/>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/educational-session--winning-more-business-ai-marketing-and-relationship-strategies-that-drive-growth</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>Interactive session combining practical AI and marketing strategies with proven relationship-building systems to help manufacturing leaders attract better prospects, strengthen market presence, and create revenue opportunities. Learn to use AI for marketing, build relationships that lead to business, create repeatable growth systems, and gain practical ideas for sales and marketing efforts.</t>
+        </is>
+      </c>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (AI for marketing strategies) and is hosted by Georgia Manufacturing Alliance, a Georgia organization, but is virtual-only with no Georgia-specific focus stated, which caps it below the 4-5 range despite the AI component and host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr"/>
+      <c r="C231" t="inlineStr"/>
+      <c r="D231" s="3" t="inlineStr"/>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr"/>
+      <c r="H231" t="inlineStr"/>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr"/>
+      <c r="K231" s="2" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (AN OPEN AI FORUM FOR ALL)</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>2</v>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/315016393/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-online&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>A collaborative community where members of all backgrounds share experiences and help each other grow in AI. Members bring questions, tools, use cases, and lessons. Topics range from basic AI concepts to advanced tools, automation, prompting, business applications, productivity, and emerging technologies.</t>
+        </is>
+      </c>
+      <c r="K232" s="2" t="inlineStr">
+        <is>
+          <t>Event has clear AI content (prompting, automation, AI tools, business applications) but is virtual-only with no Georgia host or organizational tie, capping it at 2 per the virtual-only rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>AI Ship &amp; Social - Sep 2026 Happy Hour</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>4</v>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D233" s="3" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr"/>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-ship-and-social/events/316564240/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>An Atlanta meetup bringing together people who use AI to ship products faster across marketing, sales, product, design, and engineering. Just chatting and networking with friends and teammates.</t>
+        </is>
+      </c>
+      <c r="K233" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta-based in-person meetup with genuine AI content (people using AI to ship products) and networking focus, though it's a casual happy hour rather than an educational conference or formal learning event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Open Source Night</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>3</v>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D234" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr"/>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/315992186/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta's dev communities team up for a night about open source code, tools, and the people behind it. Features talks on open source, modern dev tooling, and opportunities to connect across tech communities. Speakers cover GitHub Copilot workflows, Web Components, and building community platforms with Django.</t>
+        </is>
+      </c>
+      <c r="K234" s="2" t="inlineStr">
+        <is>
+          <t>The event is Atlanta-based with genuine AI content (GitHub Copilot workflows) among its talks, making it an educational tech event with relevant AI components, but the AI content appears to be one component rather than the primary focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>TechConnect: Global Virtual Job &amp; Networking Event for Data, AI, and Tech Pros</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>2</v>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D235" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>4:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ac-atl/events/315927621/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-online&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>A virtual networking event for developers, AI engineers, data scientists, and tech professionals to connect, collaborate, and innovate. Features organized channels for introductions, networking, job opportunities, industry discussions, project showcases, and coding accountability groups with 1-on-1 video/text chats.</t>
+        </is>
+      </c>
+      <c r="K235" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with genuine AI content (AI engineers, data scientists) but no stated Georgia host or affiliation, making it ineligible for the higher virtual-event scores reserved for Georgia-tied organizations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr"/>
+      <c r="C236" t="inlineStr"/>
+      <c r="D236" s="3" t="inlineStr"/>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr"/>
+      <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr"/>
+      <c r="K236" s="2" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Human in the loop AI for growth</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>2</v>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>11:00 AM CDT</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr"/>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/human-in-the-loop-ai-for-growth-tickets-2001692171168?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>Explore how AI plus human insight boost growth. This interactive online workshop covers identifying pain points, building AI workflows, and creating action plans. No technical experience required.</t>
+        </is>
+      </c>
+      <c r="K237" s="2" t="inlineStr">
+        <is>
+          <t>Event has genuine AI content (human-in-the-loop AI, AI workflows) but is virtual-only with no stated Georgia connection, no hosting organization identified, and a thin description that reads somewhat like a sales pitch for an unspecified service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Forward Deployed Engineer Webinar - Meta Google One Agentic AI Decision</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>2</v>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>7:00 PM GMT+5:30</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr"/>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/forward-deployed-engineer-webinar-meta-google-one-agentic-ai-decision-tickets-2000772030001?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>Join an online webinar featuring Meta and Google to explore how they use a single AI agent to make smarter decisions. Discover how agentic AI is shaping the future of product development and hiring at industry giants.</t>
+        </is>
+      </c>
+      <c r="K238" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (agentic AI) and features major tech companies, but it is virtual-only with no stated Georgia tie, and the thin description and lack of speaker/organization details limit confidence that this is a substantive educational event rather than a sales-oriented webinar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Launch Your Career in AI &amp; Emerging Tech-Cyber Work Roles at UofL DTC</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>2</v>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>University of Louisville</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/launch-your-career-in-ai-emerging-tech-cyber-work-roles-at-uofl-dtc-tickets-2001103482384?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>Free virtual information session exploring careers in artificial intelligence, machine learning, AI risk and ethics, privacy, and technology governance. Explore three career-focused Work Role Pathways: Privacy Compliance Manager, AI Risk &amp; Ethics Specialist, and AI/ML Specialist. Learn about industry-recognized certifications, online training, career coaching, and job placement support.</t>
+        </is>
+      </c>
+      <c r="K239" s="2" t="inlineStr">
+        <is>
+          <t>The event has strong AI content (AI risk &amp; ethics, ML careers, AI governance) and is hosted by University of Louisville, but it is explicitly described as virtual-only ('Free virtual information session'), and UofL is not a Georgia institution, making it ineligible for the higher virtual-event scoring that applies to Georgia-based organizations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Wednesd.AI</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>4</v>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D240" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>North Buckhead · Atlanta Tech Village - Buckhead</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>Free weekly Wednesday morning show-and-tell where community builders demonstrate how they use AI. Featured speakers take 30 minutes to share tools, workflows, and AI solutions, followed by open co-working. Doors open at 8:30 AM with coffee and networking, speaker at 9:00-9:30 AM, co-working until noon.</t>
+        </is>
+      </c>
+      <c r="K240" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (weekly show-and-tell focused on AI tools and workflows), in-person Atlanta event with clear venue, free to attend, though not a TAG event and lacks the statewide reach advantage that would push it to 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>2</v>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D241" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Linwood Heights · East Point Library</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>A weekly hands-on program introducing youth and teens to robotics, artificial intelligence, engineering thinking, and creative problem-solving. Students will explore real robots, virtual robotics environments, and beginner-friendly AI tools while completing challenges that build confidence and technical skills.</t>
+        </is>
+      </c>
+      <c r="K241" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics outreach and build-a-bot workshop focused on hardware and hands-on robotics competition rather than AI learning outcomes, which scores 1 per the robotics criteria; the mention of 'AI tools' is secondary to the robotics-build framing, but the in-person Georgia location (East Point) prevents a strict automatic-1 and allows a modest uplift to 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Agentic Payment Rails</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>4</v>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D242" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Castleberry Hill · 504 Fair St SW</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/agentic-payment-rails-tickets-2001882830435?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>Explore how programmable payments can give AI agents the ability to transact autonomously. Dive into agentic payment rails, stablecoins, blockchain networks, smart contracts, and the emerging infrastructure allowing AI agents to exchange value and interact with onchain economies.</t>
+        </is>
+      </c>
+      <c r="K242" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (autonomous AI agents) at an in-person Atlanta event, though it's a specialized technical topic rather than a broad educational conference, and the listing provides clear details with no restrictions on attendance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>FREE Machine Learning with Generative AI Bootcamp | USA Only | Live Online</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>2</v>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D243" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>10:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr"/>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-machine-learning-with-generative-ai-bootcamp-usa-only-live-online-tickets-1997153790750?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>A FREE 10-day live online bootcamp covering Machine Learning and Generative AI fundamentals. Learn Python, data preprocessing, supervised and unsupervised learning, deep learning, large language models, prompt engineering, RAG, vector databases, and AI application development. Includes hands-on training, real-world datasets, portfolio guidance, and career support.</t>
+        </is>
+      </c>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>Event has strong AI content (machine learning, generative AI, LLMs, RAG) but is virtual-only with no Georgia organizational tie, making it ineligible for higher scoring despite being free and educational.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr"/>
+      <c r="C244" t="inlineStr"/>
+      <c r="D244" s="3" t="inlineStr"/>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr"/>
+      <c r="G244" t="inlineStr"/>
+      <c r="H244" t="inlineStr"/>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr"/>
+      <c r="K244" s="2" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Fueling AI: Maximizing the Business Impact of Synthetic &amp; AI-Ready Data</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>3</v>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D245" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>5:30 pm - 7:30 pm</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr"/>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/speaker-series-the-impact-and-value-of-synthetic-other-ai-ready-data/</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr"/>
+      <c r="K245" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with genuine AI content (synthetic data, AI-ready data) hosted by TechNorth Atlanta, a Georgia organization, which elevates it from the typical virtual-only cap of 2, but the thin description and lack of detail prevent a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>AI Builders Meetup</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>2</v>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D246" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>5:30 pm - 7:30 pm</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr"/>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/1998165800699?aff=oddtdtcreator</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>A live show-and-tell where 5-7 AI builders share what they're building, their approach, tools, tech stacks, and lessons learned. Includes presentations, Q&amp;A, and networking for founders, entrepreneurs, product managers, engineers, and AI enthusiasts.</t>
+        </is>
+      </c>
+      <c r="K246" s="2" t="inlineStr">
+        <is>
+          <t>Event has strong AI content (builders sharing AI projects, tools, and approaches), but is virtual-only with no indication of Georgia hosting organization or focus, placing it in the virtual-only tier without a Georgia tie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Speaker Series: "Cloud vs. On-Premise: Is AI impacting this determination?"</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>3</v>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>5:30 pm - 7:30 pm</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/speaker-series-the-great-cloud-repatriation-why-60-of-companies-are-moving-workloads-back-on-premise/</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr"/>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event hosted by Tech North Atlanta (Georgia organization) with genuine AI content in the title, scoring 3 as a Georgia-hosted virtual event with clear AI focus rather than 5 because it is not a TAG event and the description is minimal.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10896,7 +11901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K337"/>
+  <dimension ref="A1:K353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -26108,8 +27113,6 @@
           <t>September 14, 2026</t>
         </is>
       </c>
-      <c r="F313" t="inlineStr"/>
-      <c r="G313" t="inlineStr"/>
       <c r="H313" t="inlineStr">
         <is>
           <t>https://ai.gatech.edu/event/using-containers-pace-1</t>
@@ -26158,7 +27161,6 @@
           <t>4:30 PM - 8:30 PM</t>
         </is>
       </c>
-      <c r="G314" t="inlineStr"/>
       <c r="H314" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/data-center-summit-presented-by-tag-infrastructure-society-1921079?sourceTypeId=Website</t>
@@ -26403,7 +27405,6 @@
           <t>3:30 PM EST</t>
         </is>
       </c>
-      <c r="G319" t="inlineStr"/>
       <c r="H319" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/women-of-gma-virtual-networking-event-11326</t>
@@ -26448,7 +27449,6 @@
           <t>9:00 AM EST</t>
         </is>
       </c>
-      <c r="G320" t="inlineStr"/>
       <c r="H320" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/infinity-building-solutions-plant-tour</t>
@@ -26738,7 +27738,6 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
-      <c r="G326" t="inlineStr"/>
       <c r="H326" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/cyber-security-fundamentals-tickets-1999333344855?aff=ebdssbdestsearch</t>
@@ -26783,7 +27782,6 @@
           <t>12:00 PM EDT</t>
         </is>
       </c>
-      <c r="G327" t="inlineStr"/>
       <c r="H327" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/design-it-release-it-live-app-building-challenge-tickets-1999797091935?aff=ebdssbdestsearch</t>
@@ -26934,7 +27932,6 @@
           <t>8:00 AM EDT</t>
         </is>
       </c>
-      <c r="G330" t="inlineStr"/>
       <c r="H330" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-cybersecurity-bootcamp-usa-only-live-online-tickets-1996169284064?aff=ebdssbdestsearch</t>
@@ -27077,7 +28074,6 @@
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="G333" t="inlineStr"/>
       <c r="H333" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
@@ -27228,7 +28224,6 @@
           <t>7:00 PM GMT+9:30</t>
         </is>
       </c>
-      <c r="G336" t="inlineStr"/>
       <c r="H336" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com.au/e/preserving-privacy-using-ai-in-the-digital-world-tickets-1998703630362?aff=ebdssbdestsearch</t>
@@ -27277,7 +28272,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G337" t="inlineStr"/>
       <c r="H337" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/build-your-career-in-it-cloud-data-cyber-work-role-pathways-at-uofl-dtc-tickets-2000531285929?aff=ebdssbdestsearch</t>
@@ -27296,6 +28290,810 @@
       <c r="K337" s="2" t="inlineStr">
         <is>
           <t>The event description mentions IT, cloud, data analytics, and certifications but contains zero mention of AI, machine learning, or automation, triggering the automatic-1 rule for events with no AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Careers in Cleantech &amp; Sustainability presented by TAG Smart Communities &amp; Sustainability Society</t>
+        </is>
+      </c>
+      <c r="B338" t="n">
+        <v>1</v>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D338" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>5:00 PM - 7:00 PM</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/careers-in-cleantech-sustainability-presented-by-tag-smart-communities-sustainability-society-1930413?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>Careers in Climate — an industry panel and networking social connecting Georgia's leading cleantech and sustainability professionals with the next generation of leaders. This will be an official ATL Climate Week 2026 event.</t>
+        </is>
+      </c>
+      <c r="K338" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a careers panel on cleantech and sustainability with no stated AI-focused component, making it an automatic 1 despite being hosted by a TAG society.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>SCLM Experience Series: Exclusive Coca-Cola Atlanta Syrup Plant Tours presented by TAG Supply Chain, Logistics, &amp; Manufacturing Society</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>1</v>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D339" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>10:00 AM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/sclm-experience-series-exclusive-coca-cola-atlanta-syrup-plant-tours-presented-by-tag-supply-chain-logistics-manufacturing-society-1929803?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>Go behind the scenes at one of the world's most iconic beverage brands! Join us for an exclusive, hands-on tour of the Coca-Cola Atlanta Syrup Plant.</t>
+        </is>
+      </c>
+      <c r="K339" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is a manufacturing plant tour with no stated AI content, triggering the automatic-1 rule regardless of TAG hosting it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Networking Luncheon - Atlanta 12-17-2026</t>
+        </is>
+      </c>
+      <c r="B340" t="n">
+        <v>1</v>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D340" s="3" t="n">
+        <v>46373</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>11:30 AM - 1:00 PM EST</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>Atlanta, Georgia</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/networking-luncheon---atlanta-12-17-2026</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J340" s="2" t="inlineStr"/>
+      <c r="K340" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of the Georgia Manufacturing Alliance host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Ethical Hacker Tactics, CTF &amp; Tech Talks Monthly by BlackHack Society</t>
+        </is>
+      </c>
+      <c r="B341" t="n">
+        <v>1</v>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D341" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/blackhack-society-atlanta/events/313805602/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J341" s="2" t="inlineStr">
+        <is>
+          <t>Monthly offensive security hacking practice session featuring guided penetration testing techniques, Capture the Flag events, and topics like Google Dorking, Vulnhub, FlipperZero, Wifi Pineapple, and lockpicking. Covers beginner to advanced ethical hacking techniques with bonus guest speakers.</t>
+        </is>
+      </c>
+      <c r="K341" s="2" t="inlineStr">
+        <is>
+          <t>The event is about ethical hacking, penetration testing, and cybersecurity techniques with no mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>STEM on the Green</t>
+        </is>
+      </c>
+      <c r="B342" t="n">
+        <v>1</v>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D342" s="3" t="n">
+        <v>46291</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Jamestown · College Park Golf Course</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/stem-on-the-green-tickets-1999636078339?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J342" s="2" t="inlineStr"/>
+      <c r="K342" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Forestry Resource Management Workshop (Swainsboro, Ga)</t>
+        </is>
+      </c>
+      <c r="B343" t="n">
+        <v>1</v>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D343" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>Georgia · 24 Jarrett Durden Rd</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/forestry-resource-management-workshop-swainsboro-ga-tickets-1998399812635?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J343" s="2" t="inlineStr"/>
+      <c r="K343" s="2" t="inlineStr">
+        <is>
+          <t>The event title and short description contain zero mention of AI, machine learning, or automation - it is a forestry resource management workshop with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Adopt-A-Stream Workshop: Macroinvertebrate/Biological Monitoring</t>
+        </is>
+      </c>
+      <c r="B344" t="n">
+        <v>1</v>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D344" s="3" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>Georgia · Davidson-Arabia Mountain Nature Center, Stonecrest, GA, USA</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/adopt-a-stream-workshop-macroinvertebratebiological-monitoring-tickets-1996371171916?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J344" s="2" t="inlineStr"/>
+      <c r="K344" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a biological monitoring workshop about macroinvertebrates in streams, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>FREE TECH EVENT-Exploring the Arts &amp; Science</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>1</v>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D345" s="3" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>Capitol View Manor · 1332 Metropolitan Pkwy SW</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-tech-event-exploring-the-arts-science-tickets-2001275091672?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J345" s="2" t="inlineStr">
+        <is>
+          <t>Two sessions: Adults 55+ explore technology, sensors &amp; innovation. Ages 10-17 explore music, visual &amp; performing arts, writing &amp; creativity.</t>
+        </is>
+      </c>
+      <c r="K345" s="2" t="inlineStr">
+        <is>
+          <t>The event description mentions 'technology, sensors &amp; innovation' for adults but provides no specific mention of AI, machine learning, or automation, and the vague framing suggests general technology exploration rather than AI-focused content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Elephant Toothpaste</t>
+        </is>
+      </c>
+      <c r="B346" t="n">
+        <v>1</v>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D346" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>Austell · Sweetwater Valley Library</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/elephant-toothpaste-tickets-2000995002919?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J346" s="2" t="inlineStr"/>
+      <c r="K346" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a chemistry demonstration activity (elephant toothpaste), triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Spill the tea about researh!</t>
+        </is>
+      </c>
+      <c r="B347" t="n">
+        <v>1</v>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D347" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>Old Fourth Ward · Ponce De Leon Center</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/spill-the-tea-about-researh-tickets-2001256695649?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J347" s="2" t="inlineStr"/>
+      <c r="K347" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B348" t="n">
+        <v>1</v>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D348" s="3" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>Georgia · Browns Mill Recreation Center</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J348" s="2" t="inlineStr"/>
+      <c r="K348" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Webinar: Too Many Cybersecurity Priorities?</t>
+        </is>
+      </c>
+      <c r="B349" t="n">
+        <v>1</v>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D349" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>2:00 PM GMT+1</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr"/>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/webinar-too-many-cybersecurity-priorities-tickets-2001389213012?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J349" s="2" t="inlineStr"/>
+      <c r="K349" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Entrepreneurial Hour</t>
+        </is>
+      </c>
+      <c r="B350" t="n">
+        <v>1</v>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D350" s="3" t="inlineStr">
+        <is>
+          <t>Every Wednesday</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>8:00 am - 9:00 am</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>Tech North Atlanta, 925 North Point Parkway, Suite 130, Alpharetta, GA 30005 &amp; Virtually</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>https://zoom.theentrepreneurialhour.com/</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J350" s="2" t="inlineStr">
+        <is>
+          <t>Free, open meetup held every Wednesday at the Tech North Atlanta Incubator and virtually.</t>
+        </is>
+      </c>
+      <c r="K350" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it is simply a general entrepreneurial meetup, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>ATDC Alpharetta Startup Circle</t>
+        </is>
+      </c>
+      <c r="B351" t="n">
+        <v>1</v>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D351" s="3" t="inlineStr">
+        <is>
+          <t>Every Friday</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>9:00 am - 10:30 am</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Tech North Atlanta, 925 North Point Parkway, Suite 130, Alpharetta, GA 30005 &amp; Virtually</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>https://gatech.zoom.us/j/95518955124</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J351" s="2" t="inlineStr">
+        <is>
+          <t>Free, open startup meetup held every Friday at the Tech North Atlanta Incubator and virtually.</t>
+        </is>
+      </c>
+      <c r="K351" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it is simply a general startup meetup with no stated AI-focused component, session, or speaker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Startup Workshop: Building your Due Diligence Data Room/Audit Readiness</t>
+        </is>
+      </c>
+      <c r="B352" t="n">
+        <v>1</v>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D352" s="3" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>12:00 pm - 1:00 pm</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr"/>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/1998932829904?aff=oddtdtcreator</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J352" s="2" t="inlineStr">
+        <is>
+          <t>Startup LifeCycle Series Workshop Session Five: Building your Due Diligence Data Room/Audit Readiness.</t>
+        </is>
+      </c>
+      <c r="K352" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is about startup financial/legal preparation processes, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Startup LifeCycle Series Workshop Session Six: Startup Operational Benchmarks &amp; Best Practices</t>
+        </is>
+      </c>
+      <c r="B353" t="n">
+        <v>1</v>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D353" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>September 21, 2026</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>12:00 pm - 1:00 pm</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Tech North Atlanta Pitch Room, 925 North Point Pkwy, Suite 130, Alpharetta, GA 30005</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/startup-workshop-meet-the-investor-3/</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J353" s="2" t="inlineStr"/>
+      <c r="K353" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of location or host.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-09-28
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K247" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K257" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K353" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K377" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K247"/>
+  <dimension ref="A1:K257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -10888,7 +10888,6 @@
           <t>8:00 AM - 10:00 AM</t>
         </is>
       </c>
-      <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/R1F2vZvsRC0CX</t>
@@ -10937,7 +10936,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/KVF3Bv1snCBCW</t>
@@ -10986,7 +10984,6 @@
           <t>2:00 PM - 7:00 PM</t>
         </is>
       </c>
-      <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/YEFn9vxTNCzCK</t>
@@ -11035,7 +11032,6 @@
           <t>5:00 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/executive-exchange-presented-by-tag-data-governance-society-1929065?sourceTypeId=Website</t>
@@ -11084,7 +11080,6 @@
           <t>11:00 AM - 1:30 PM EST</t>
         </is>
       </c>
-      <c r="G230" t="inlineStr"/>
       <c r="H230" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/educational-session--winning-more-business-ai-marketing-and-relationship-strategies-that-drive-growth</t>
@@ -11112,17 +11107,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr"/>
-      <c r="C231" t="inlineStr"/>
       <c r="D231" s="3" t="inlineStr"/>
       <c r="E231" t="inlineStr">
         <is>
           <t>September 21, 2026</t>
         </is>
       </c>
-      <c r="F231" t="inlineStr"/>
-      <c r="G231" t="inlineStr"/>
-      <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -11211,7 +11201,6 @@
           <t>6:00 PM EDT</t>
         </is>
       </c>
-      <c r="G233" t="inlineStr"/>
       <c r="H233" t="inlineStr">
         <is>
           <t>https://www.meetup.com/ai-ship-and-social/events/316564240/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
@@ -11260,7 +11249,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G234" t="inlineStr"/>
       <c r="H234" t="inlineStr">
         <is>
           <t>https://www.meetup.com/refactr-tech/events/315992186/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
@@ -11341,17 +11329,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr"/>
-      <c r="C236" t="inlineStr"/>
       <c r="D236" s="3" t="inlineStr"/>
       <c r="E236" t="inlineStr">
         <is>
           <t>September 21, 2026</t>
         </is>
       </c>
-      <c r="F236" t="inlineStr"/>
-      <c r="G236" t="inlineStr"/>
-      <c r="H236" t="inlineStr"/>
       <c r="I236" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -11387,7 +11370,6 @@
           <t>11:00 AM CDT</t>
         </is>
       </c>
-      <c r="G237" t="inlineStr"/>
       <c r="H237" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/human-in-the-loop-ai-for-growth-tickets-2001692171168?aff=ebdssbdestsearch</t>
@@ -11436,7 +11418,6 @@
           <t>7:00 PM GMT+5:30</t>
         </is>
       </c>
-      <c r="G238" t="inlineStr"/>
       <c r="H238" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/forward-deployed-engineer-webinar-meta-google-one-agentic-ai-decision-tickets-2000772030001?aff=ebdssbdestsearch</t>
@@ -11697,7 +11678,6 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
-      <c r="G243" t="inlineStr"/>
       <c r="H243" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-machine-learning-with-generative-ai-bootcamp-usa-only-live-online-tickets-1997153790750?aff=ebdssbdestsearch</t>
@@ -11725,17 +11705,12 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr"/>
-      <c r="C244" t="inlineStr"/>
       <c r="D244" s="3" t="inlineStr"/>
       <c r="E244" t="inlineStr">
         <is>
           <t>September 21, 2026</t>
         </is>
       </c>
-      <c r="F244" t="inlineStr"/>
-      <c r="G244" t="inlineStr"/>
-      <c r="H244" t="inlineStr"/>
       <c r="I244" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -11771,7 +11746,6 @@
           <t>5:30 pm - 7:30 pm</t>
         </is>
       </c>
-      <c r="G245" t="inlineStr"/>
       <c r="H245" t="inlineStr">
         <is>
           <t>https://technorthatlanta.org/event/speaker-series-the-impact-and-value-of-synthetic-other-ai-ready-data/</t>
@@ -11816,7 +11790,6 @@
           <t>5:30 pm - 7:30 pm</t>
         </is>
       </c>
-      <c r="G246" t="inlineStr"/>
       <c r="H246" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/1998165800699?aff=oddtdtcreator</t>
@@ -11884,6 +11857,432 @@
       <c r="K247" s="2" t="inlineStr">
         <is>
           <t>Virtual-only event hosted by Tech North Atlanta (Georgia organization) with genuine AI content in the title, scoring 3 as a Georgia-hosted virtual event with clear AI focus rather than 5 because it is not a TAG event and the description is minimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Zero Trust in the Age of AI: Securing Software from Code to Cloud presented by TAG Cloud Society</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>5</v>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D248" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr"/>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/07FOAoxtxCwCR</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>An insightful evening on Zero Trust in the Software Development Lifecycle, featuring a panel of technology and cybersecurity leaders discussing how organizations can bring Zero Trust principles into modern software delivery.</t>
+        </is>
+      </c>
+      <c r="K248" s="2" t="inlineStr">
+        <is>
+          <t>TAG event with genuine AI content (Zero Trust security in the age of AI), hosted by TAG Cloud Society on tagonline.org, featuring industry panel discussion on AI-aware security practices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr"/>
+      <c r="C249" t="inlineStr"/>
+      <c r="D249" s="3" t="inlineStr"/>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr"/>
+      <c r="G249" t="inlineStr"/>
+      <c r="H249" t="inlineStr"/>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr"/>
+      <c r="K249" s="2" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr"/>
+      <c r="C250" t="inlineStr"/>
+      <c r="D250" s="3" t="inlineStr"/>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr"/>
+      <c r="G250" t="inlineStr"/>
+      <c r="H250" t="inlineStr"/>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J250" s="2" t="inlineStr"/>
+      <c r="K250" s="2" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>From Idea To Music (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>4</v>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>6:00 AM GMT+2</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr"/>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-idea-to-music</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>A hands-on lunch workshop where you'll turn an idea into an actual AI-generated song. Using tools like ChatGPT and Suno, explore the creative process from concept to lyrics to music, experiment through iteration, and participate in an AI Song Challenge. Open to anyone curious about AI, music and creativity—no prior expertise required.</t>
+        </is>
+      </c>
+      <c r="K251" s="2" t="inlineStr">
+        <is>
+          <t>This is a Georgia-tied in-person AI builder event (hands-on workshop with AI tools and creative iteration) hosted by The AI Collective, scoring well on educational AI content and builder focus, but confidence is medium due to missing location details and unclear Georgia chapter confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Search, redesigned: What AI Means for Shopping (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>3</v>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>5:30 AM</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Google Meet</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-sw-9-30</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>Explore how AI is reshaping the shopping journey from discovery to decision. Learn about AI search, visibility, shopping, and agentic commerce, with practical insights on how brands show up in AI-generated answers and what's changing in the era of AI-native commerce.</t>
+        </is>
+      </c>
+      <c r="K252" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with genuine AI content (AI search, agentic commerce, AI-native shopping) hosted by The AI Collective, a Georgia organization, which allows a score of 3-4 rather than capped at 2, but the virtual-only format and lack of builder/hands-on component prevents a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>The AI Tasting Room (w/ The AI Collective Fayetteville)</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>4</v>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Fayetteville, GA</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-at-9-30b</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>A monthly gathering combining fine wine and desserts with conversations about AI. For curious minds interested in AI, this relaxed evening brings together people to discuss what's changing in AI, what's exciting, and where it's heading next.</t>
+        </is>
+      </c>
+      <c r="K253" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI event in Fayetteville (outside metro Atlanta) hosted by The AI Collective's Georgia chapter with genuine AI content focus, but scores below 5 because it is a social/discussion event rather than a builder-focused meetup with technical project presentations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Wednesd.AI</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>5</v>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D254" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>North Buckhead · Atlanta Tech Village - Buckhead</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wednesdai-tickets-1990814107587?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>Free weekly Wednesday morning show-and-tell where builders from the community demonstrate how they're using AI in real projects. Each week features a 30-minute presentation followed by open co-working until noon. Includes coffee and networking.</t>
+        </is>
+      </c>
+      <c r="K254" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI builder event in Atlanta with weekly recurring show-and-tell format where community members present real AI projects, followed by Q&amp;A and networking—exactly the type of hands-on builder community event the client most wants to attend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr"/>
+      <c r="C255" t="inlineStr"/>
+      <c r="D255" s="3" t="inlineStr"/>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr"/>
+      <c r="G255" t="inlineStr"/>
+      <c r="H255" t="inlineStr"/>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J255" s="2" t="inlineStr"/>
+      <c r="K255" s="2" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Fueling AI: Maximizing the Business Impact of Syntehtic &amp; AI-Ready Data</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>4</v>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr"/>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/speaker-series-the-impact-and-value-of-synthetic-other-ai-ready-data/</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J256" s="2" t="inlineStr"/>
+      <c r="K256" s="2" t="inlineStr">
+        <is>
+          <t>Educational AI event with genuine AI content (synthetic data, AI-ready data) hosted by Tech North Atlanta, a Georgia organization, but scored below 5 due to missing description details and no indication of hands-on builder format or TAG affiliation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Speaker Series: "Can AI Prevent the Next Global Supply Chain Disruption?"</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>4</v>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D257" s="3" t="n">
+        <v>46330</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Greater Perimeter Chamber</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/speaker-series-can-ai-prevent-the-next-global-supply-chain-disruption/</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J257" s="2" t="inlineStr"/>
+      <c r="K257" s="2" t="inlineStr">
+        <is>
+          <t>In-person speaker series with genuine AI content (supply chain disruption prevention via AI) hosted by Tech North Atlanta, an Atlanta-area technology organization, but limited confidence due to missing event description details.</t>
         </is>
       </c>
     </row>
@@ -11901,7 +12300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K353"/>
+  <dimension ref="A1:K377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -28475,7 +28874,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G341" t="inlineStr"/>
       <c r="H341" t="inlineStr">
         <is>
           <t>https://www.meetup.com/blackhack-society-atlanta/events/313805602/?recId=bbd352ba-a1cd-469a-af1c-39e48c22cd45&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=8ee3bae2-7be6-4a71-a6c4-b4b72d5ec923&amp;eventOrigin=find_page%24all</t>
@@ -28871,7 +29269,6 @@
           <t>2:00 PM GMT+1</t>
         </is>
       </c>
-      <c r="G349" t="inlineStr"/>
       <c r="H349" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/webinar-too-many-cybersecurity-priorities-tickets-2001389213012?aff=ebdssbdestsearch</t>
@@ -29026,7 +29423,6 @@
           <t>12:00 pm - 1:00 pm</t>
         </is>
       </c>
-      <c r="G352" t="inlineStr"/>
       <c r="H352" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/1998932829904?aff=oddtdtcreator</t>
@@ -29094,6 +29490,1190 @@
       <c r="K353" s="2" t="inlineStr">
         <is>
           <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of location or host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Human Intelligence: How Teams Win With Customer and Employee Insights presented by TAG CX and TAG DEI Societies</t>
+        </is>
+      </c>
+      <c r="B354" t="n">
+        <v>1</v>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D354" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr"/>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/12FOd6XigCVCB</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J354" s="2" t="inlineStr">
+        <is>
+          <t>Explore how data, human judgment, organizational learning, and inclusive tech connect customer and employee intelligence to retention, engagement, productivity, service, and growth.</t>
+        </is>
+      </c>
+      <c r="K354" s="2" t="inlineStr">
+        <is>
+          <t>The event description mentions data, human judgment, and organizational learning but contains zero mention of AI, machine learning, or automation, triggering the automatic-1 rule regardless of the TAG host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Women of GMA Virtual Networking Event 10/3/26</t>
+        </is>
+      </c>
+      <c r="B355" t="n">
+        <v>1</v>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D355" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>3:30 PM</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr"/>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/women-of-gma-virtual-networking-event-10326</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J355" s="2" t="inlineStr"/>
+      <c r="K355" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of the Georgia Manufacturing Alliance host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>WGMA DeNyse Companies Plant Tour- Douglasville</t>
+        </is>
+      </c>
+      <c r="B356" t="n">
+        <v>1</v>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D356" s="3" t="n">
+        <v>46336</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>Douglasville, Georgia</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/wgma-denyse-companies-plant-tour</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J356" s="2" t="inlineStr"/>
+      <c r="K356" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a plant tour by the Georgia Manufacturing Alliance with no stated AI content, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>ThinkingAI Agentic Growth Summit 2026</t>
+        </is>
+      </c>
+      <c r="B357" t="n">
+        <v>1</v>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D357" s="3" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>Mountain View, CA</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>https://luma.com/thinkingai-summit-us</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J357" s="2" t="inlineStr"/>
+      <c r="K357" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>AI in Finance - The Future of Work</t>
+        </is>
+      </c>
+      <c r="B358" t="n">
+        <v>1</v>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D358" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>10:00 AM GMT+3</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Helsinki, Finland</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-fi-9-29</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J358" s="2" t="inlineStr"/>
+      <c r="K358" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Finland, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>AI Collective x Revamp | Sibos Miami Dinner</t>
+        </is>
+      </c>
+      <c r="B359" t="n">
+        <v>1</v>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D359" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>7:30 PM</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Miami Beach, FL</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>https://luma.com/o2uar3o9</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J359" s="2" t="inlineStr"/>
+      <c r="K359" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Florida (FL), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>AI Skill Swap Mixer: Learn, Share &amp; Network (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B360" t="n">
+        <v>1</v>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D360" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-sl-mixer</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J360" s="2" t="inlineStr"/>
+      <c r="K360" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Utah (UT), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>The Future of Cyber: Private Dinner (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B361" t="n">
+        <v>1</v>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D361" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>9:00 PM</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>https://luma.com/lyrie-dinner-sf</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J361" s="2" t="inlineStr"/>
+      <c r="K361" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>4th Annual Tech Mixer</t>
+        </is>
+      </c>
+      <c r="B362" t="n">
+        <v>1</v>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D362" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>9:30 PM</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>Davis, CA</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>https://luma.com/techmixer26</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J362" s="2" t="inlineStr"/>
+      <c r="K362" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>There Are Other Ways: Leadership in the Age of AI</t>
+        </is>
+      </c>
+      <c r="B363" t="n">
+        <v>1</v>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D363" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>6:30 AM GMT+8</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>Kuala Lumpur, Malaysia</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-kul-20260930</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J363" s="2" t="inlineStr"/>
+      <c r="K363" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Malaysia, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Hack for Humanity: Hartford-Micro Hackathon (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B364" t="n">
+        <v>1</v>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>Hartford, CT</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-ha-sept-30</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J364" s="2" t="inlineStr"/>
+      <c r="K364" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Connecticut (CT), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>AI Town Hall Gulf Beeze (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B365" t="n">
+        <v>1</v>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D365" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>Gulf Breeze, FL</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-pe-9-30</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J365" s="2" t="inlineStr"/>
+      <c r="K365" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Florida (FL), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>AIC SF Chapter Team &amp; Volunteer Get-Together (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B366" t="n">
+        <v>1</v>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D366" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>8:30 PM</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>San Francisco, CA</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-sf-team-gettogether</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J366" s="2" t="inlineStr"/>
+      <c r="K366" s="2" t="inlineStr">
+        <is>
+          <t>Location is in California (CA), not Georgia; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Let's Talk AI! #5 (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B367" t="n">
+        <v>1</v>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D367" s="3" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>11:30 AM GMT+3</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>București, Romania</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>https://luma.com/lets-talk-ai-5</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J367" s="2" t="inlineStr"/>
+      <c r="K367" s="2" t="inlineStr">
+        <is>
+          <t>Location is in Romania, not Georgia, USA; auto-rejected without scoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>🧠 AI Founders Roundtable with The AI Collective DC x Avahi</t>
+        </is>
+      </c>
+      <c r="B368" t="n">
+        <v>1</v>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D368" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>Court House</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>https://luma.com/avahi-dc-0926</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J368" s="2" t="inlineStr">
+        <is>
+          <t>A small group roundtable bringing together Washington, DC founders and operators with Avahi and AWS. Selected participants are eligible for up to $100K in AWS development credits. Includes dinner, drinks, networking, and small-group conversations for founders with products in market, real traction, and defensible AI or automation use cases.</t>
+        </is>
+      </c>
+      <c r="K368" s="2" t="inlineStr">
+        <is>
+          <t>Event is located in Washington, DC with no Georgia tie, and while it has AI content, it is restricted to selected participants (founders with specific criteria and vetting), making it inaccessible to the client's general audience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>AI and the Future of Humanity: What Could the 'AI Destroys Humanity' Debate Mean for the Global South?</t>
+        </is>
+      </c>
+      <c r="B369" t="n">
+        <v>1</v>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D369" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>Zoom</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>https://luma.com/aidesruction</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J369" s="2" t="inlineStr"/>
+      <c r="K369" s="2" t="inlineStr">
+        <is>
+          <t>Event is explicitly virtual-only (Zoom) with no Georgia host or organizational tie, and while the title mentions AI, the description is empty and the event appears to be a philosophical/policy discussion rather than an educational or builder-focused AI event, making it ineligible under the virtual-events cap for non-Georgia hosts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>The AI Era &amp; What It Means To Be Human (w/ The AI Collective)</t>
+        </is>
+      </c>
+      <c r="B370" t="n">
+        <v>1</v>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D370" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>Connecticut Ave/ K Street</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>https://luma.com/aic-dc-9-30</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J370" s="2" t="inlineStr"/>
+      <c r="K370" s="2" t="inlineStr">
+        <is>
+          <t>Event is located in Washington, DC (Connecticut Ave/K Street), not Georgia, and while hosted by The AI Collective (which has a Georgia chapter), this appears to be their DC chapter event with no Georgia connection stated in the listing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Who, When &amp; Where: The Data Activity Story — CLOAK DSP</t>
+        </is>
+      </c>
+      <c r="B371" t="n">
+        <v>1</v>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D371" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>8:00 PM GMT+5:30</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr"/>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/who-when-where-the-data-activity-story-cloak-dsp-tickets-2001691276492?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J371" s="2" t="inlineStr">
+        <is>
+          <t>Join an insightful webinar exploring how organizations can gain visibility into data activity and strengthen security of sensitive information with CLOAK DSP. Learn why data activity visibility matters, how to identify and monitor sensitive data, understand data movement and access, and discover ways to improve data security and control.</t>
+        </is>
+      </c>
+      <c r="K371" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it focuses on data activity visibility and security monitoring, which are data governance topics unrelated to AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Spill the tea about research!</t>
+        </is>
+      </c>
+      <c r="B372" t="n">
+        <v>1</v>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D372" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>Old Fourth Ward · Ponce De Leon Center</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/spill-the-tea-about-research-tickets-2001256695649?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J372" s="2" t="inlineStr"/>
+      <c r="K372" s="2" t="inlineStr">
+        <is>
+          <t>The event title and short description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B373" t="n">
+        <v>1</v>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D373" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>Linwood Heights · East Point Library</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J373" s="2" t="inlineStr">
+        <is>
+          <t>Weekly hands-on program introducing youth and teens to robotics, artificial intelligence, engineering thinking, and creative problem-solving. Students will explore real robots, virtual robotics environments, and beginner-friendly AI tools while completing challenges that build confidence and technical skills.</t>
+        </is>
+      </c>
+      <c r="K373" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics outreach and build program focused on hardware, robots, and engineering challenges rather than AI as a technical subject, falling squarely into the category of robotics events scored 1 per the criteria despite mentioning AI in the title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B374" t="n">
+        <v>1</v>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D374" s="3" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>Georgia · Browns Mill Recreation Center</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J374" s="2" t="inlineStr"/>
+      <c r="K374" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>REALITY By Tialauna | SIGHT</t>
+        </is>
+      </c>
+      <c r="B375" t="n">
+        <v>1</v>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D375" s="3" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>5:00 PM</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>Dunwoody Forest · Murphey Candler Park</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/reality-by-tialauna-sight-tickets-2002384896127?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J375" s="2" t="inlineStr"/>
+      <c r="K375" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>BitDevs: Bitcoin Socratic Seminar #55 - pre-TABConf</t>
+        </is>
+      </c>
+      <c r="B376" t="n">
+        <v>1</v>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D376" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>684 John Wesley Dobbs Ave NE suite a1, Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315044442/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J376" s="2" t="inlineStr">
+        <is>
+          <t>Join the Atlanta BitDevs every third Wednesday for a Socratic Seminar to discuss the latest technological developments in Bitcoin and Lightning, formatted to foster debate, information sharing and lively discussion. Free drinks during early networking, followed by presentations and a Socratic Seminar.</t>
+        </is>
+      </c>
+      <c r="K376" s="2" t="inlineStr">
+        <is>
+          <t>This event is about Bitcoin and Lightning Network technology with no mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of its in-person Georgia location and active host community.</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Startup Workshop: Preparing to seek Pre-seed, Seed, and Series A Funding, and the Current Climate for Investor Funding in Metro ATL</t>
+        </is>
+      </c>
+      <c r="B377" t="n">
+        <v>1</v>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D377" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>September 28, 2026</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>Tech North Atlanta Pitch Room, 925 North Point Pkwy. Suite 130, Alpharetta, GA 30005</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/startup-workshop-preparing-to-seek-pre-seed-seed-and-series-a-funding-and-the-current-climate-for-investor-funding-in-metro-atl/</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J377" s="2" t="inlineStr"/>
+      <c r="K377" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is purely about startup funding and investor relations, triggering the automatic-1 rule regardless of location or host.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-10-05
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K257" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K281" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K377" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K422" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K257"/>
+  <dimension ref="A1:K281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -11887,7 +11887,6 @@
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="G248" t="inlineStr"/>
       <c r="H248" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/07FOAoxtxCwCR</t>
@@ -11915,17 +11914,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B249" t="inlineStr"/>
-      <c r="C249" t="inlineStr"/>
       <c r="D249" s="3" t="inlineStr"/>
       <c r="E249" t="inlineStr">
         <is>
           <t>September 28, 2026</t>
         </is>
       </c>
-      <c r="F249" t="inlineStr"/>
-      <c r="G249" t="inlineStr"/>
-      <c r="H249" t="inlineStr"/>
       <c r="I249" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -11940,17 +11934,12 @@
           <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr"/>
-      <c r="C250" t="inlineStr"/>
       <c r="D250" s="3" t="inlineStr"/>
       <c r="E250" t="inlineStr">
         <is>
           <t>September 28, 2026</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr"/>
-      <c r="G250" t="inlineStr"/>
-      <c r="H250" t="inlineStr"/>
       <c r="I250" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -11986,7 +11975,6 @@
           <t>6:00 AM GMT+2</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr"/>
       <c r="H251" t="inlineStr">
         <is>
           <t>https://luma.com/aic-idea-to-music</t>
@@ -12173,17 +12161,12 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
-      <c r="B255" t="inlineStr"/>
-      <c r="C255" t="inlineStr"/>
       <c r="D255" s="3" t="inlineStr"/>
       <c r="E255" t="inlineStr">
         <is>
           <t>September 28, 2026</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr"/>
-      <c r="G255" t="inlineStr"/>
-      <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -12219,7 +12202,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr"/>
       <c r="H256" t="inlineStr">
         <is>
           <t>https://technorthatlanta.org/event/speaker-series-the-impact-and-value-of-synthetic-other-ai-ready-data/</t>
@@ -12283,6 +12265,1144 @@
       <c r="K257" s="2" t="inlineStr">
         <is>
           <t>In-person speaker series with genuine AI content (supply chain disruption prevention via AI) hosted by Tech North Atlanta, an Atlanta-area technology organization, but limited confidence due to missing event description details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>AI in Manufacturing: Live at Georgia Tech</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>5</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D258" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>3:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Advanced Manufacturing Pilot Facility, 555 14th Street NW, Atlanta, GA 30318</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>https://ai.gatech.edu/event/ai-manufacturing-live-georgia-tech</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>Explore how artificial intelligence is transforming manufacturing through robotics, production systems, materials, and advanced manufacturing processes during an exclusive showcase at Georgia Tech's Advanced Manufacturing Pilot Facility.</t>
+        </is>
+      </c>
+      <c r="K258" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI event at Georgia Tech (a Georgia university) in Atlanta with genuine AI content focused on manufacturing applications, clear venue and date, and a legitimate educational showcase format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr"/>
+      <c r="C259" t="inlineStr"/>
+      <c r="D259" s="3" t="inlineStr"/>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr"/>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="inlineStr"/>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr"/>
+      <c r="K259" s="2" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>AI on the Factory Floor: The Future of Manufacturing in Georgia</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>5</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>3:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr"/>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316692853/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>Explore how AI is moving into manufacturing on the factory floor. See real applications and live demonstrations at Georgia Tech's Advanced Manufacturing Pilot Facility, including guided tours, live demos, and networking with manufacturers, technologists, researchers, and students working at the intersection of AI and industry.</t>
+        </is>
+      </c>
+      <c r="K260" s="2" t="inlineStr">
+        <is>
+          <t>This is an in-person AI builder event in Georgia (Georgia Tech location, real applications and live demonstrations, networking with practitioners) hosted by a Georgia organization (Georgia AI Alliance), with genuine AI content focused on manufacturing applications, fitting the client's highest-priority event type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>🚀 What's New in ChatGPT: The Latest Upgrades, Tools &amp; AI Agents</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>4</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>9:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlanta-ai-builders/events/316138852/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-online&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>A practical walkthrough of the latest ChatGPT capabilities including GPT-5.6, ChatGPT Work, Codex, Plugins, Deep Research, Projects, and Voice/Multimodal features. Features live demonstrations and practical examples covering how these tools transform work, research, coding, and creativity. For professionals, entrepreneurs, developers, students, researchers, and anyone interested in AI.</t>
+        </is>
+      </c>
+      <c r="K261" s="2" t="inlineStr">
+        <is>
+          <t>This is a virtual-only AI educational event hosted by Atlanta AI Builders (a Georgia-tied organization), with clear AI content focused on ChatGPT capabilities and practical applications, but scores 4 rather than 5 because it is virtual-only and does not appear to be a hands-on builder/demo event with peer presentations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (OPEN FOR ALL)</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>2</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/315939823/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-online&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>A collaborative learning community where members share real experiences and help each other grow in AI. Topics range from basic AI concepts to advanced tools, automation, prompting, business applications, productivity, and emerging technologies. Open to all backgrounds and experience levels.</t>
+        </is>
+      </c>
+      <c r="K262" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with genuine AI content (tools, automation, prompting, business applications) but no stated Georgia organizational tie, scoring at the baseline for remote events with clear AI focus and no paid/sales-pitch elements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>[Partner Event] - Local Models, Agentic Teams</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>3</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>5:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr"/>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-ship-and-social/events/316770121/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr"/>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>The title clearly indicates AI content (local models, agentic teams), and the Meetup.com host suggests an in-person builder community event, but the blank location and description prevent confirming Georgia location or the depth of hands-on AI builder focus that would warrant a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr"/>
+      <c r="C264" t="inlineStr"/>
+      <c r="D264" s="3" t="inlineStr"/>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr"/>
+      <c r="G264" t="inlineStr"/>
+      <c r="H264" t="inlineStr"/>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr"/>
+      <c r="K264" s="2" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Avant South 2026</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>5</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D265" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Midtown · Global Learning and Conference Center</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/avant-south-2026-tickets-1989311616596?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta's premier tech and innovation event exploring AI in Action across key industries including logistics, fintech, healthcare, and media. Features industry pioneers, academic leaders, and startup innovators discussing real-world AI applications and strategies to shape Atlanta's future as a national leader in applied AI.</t>
+        </is>
+      </c>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI conference in Atlanta with explicit focus on real-world AI applications across multiple industries, featuring industry pioneers and academic leaders, hitting all markers of a high-value educational AI event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>ElevateHER AI FALL Summit Oct 16th</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>4</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D266" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Howell Wood · Atlanta Tech Park</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/elevateher-ai-fall-summit-oct-16th-tickets-1991630063132?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>Explore how AI Innovation is reinventing Education at this in-person summit featuring innovative small businesses, women founders, entrepreneurs, education leaders, and technology leaders. Includes women's journeys in AI, real use cases for higher education, and live AI demonstrations.</t>
+        </is>
+      </c>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>In-person Atlanta event with genuine AI content (women in AI, education use cases, live demonstrations) hosted by an organization focused on AI innovation, but scores below 5 because it emphasizes entrepreneurship/networking aspects alongside the educational AI content rather than being a pure AI builder/demo event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>AI Builders Meetup | October 8th</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>5</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Jamestowne · 11675 Rainwater Dr suite 100</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-builders-meetup-october-8th-tickets-1998165800699?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>A live show-and-tell for builders where 5-7 AI builders share what they're building, their approach, tools and tech stacks, and lessons learned. Includes presentations, Q&amp;A, and networking for founders, entrepreneurs, product managers, engineers, and AI enthusiasts.</t>
+        </is>
+      </c>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>This is an in-person AI builder event in Georgia (Jamestowne location) featuring a show-and-tell format with multiple AI builders presenting their projects, tools, and lessons learned, followed by Q&amp;A and networking—exactly matching the client's highest-priority event type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Speaker Series: "How AI is impacting Cloud vs. On-Premise Strategies"</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>3</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Jamestowne · Improving</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/speaker-series-how-ai-is-impacting-cloud-vs-on-premise-strategies-tickets-2002439064145?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J268" s="2" t="inlineStr"/>
+      <c r="K268" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content in its title and focuses on AI's impact on infrastructure strategy, is in-person in Georgia (Jamestowne/Improving suggests a local venue), but lacks detail about the speaker, format, and depth of technical content, and appears to be a single speaker session rather than a builder-focused community event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>8 Week AI Masterclass</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>2</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D269" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>12:15 PM</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Pirkle Woods · Keller Williams Community Partners</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/8-week-ai-masterclass-tickets-1994713296165?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t>An 8-week AI course helping real estate agents build their brand with AI. Attend 6 out of 8 classes and get a full refund!</t>
+        </is>
+      </c>
+      <c r="K269" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (an 8-week AI course) but is a paid training program heavily marketed as a sales pitch for real estate agent branding, lacks Georgia venue verification despite the listing location, and the description suggests it prioritizes conversion and refund incentives over technical depth or builder-community engagement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Trusted AI: Data Governance, Cybersecurity, and Responsible AI</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>3</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>8:00 AM</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Midtown · Hampton Inn &amp; Suites Atlanta Midtown</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/trusted-ai-data-governance-cybersecurity-and-responsible-ai-registration-1998335750022?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>Join an in-person event exploring Trusted AI with hands-on talks on data governance, cybersecurity, and responsible AI. Connect with professionals and learn how to build ethical, powerful AI for your business and organization.</t>
+        </is>
+      </c>
+      <c r="K270" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (data governance, cybersecurity, responsible AI) and is in-person in Atlanta, but the description lacks specifics about hands-on builder/technical depth, speakers, or sessions that would elevate it to a 4-5, and it appears to be more of a professional conference than a builder-focused meetup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Augusta Georgia AIM Week Mobile Studio Day</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>2</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Augusta, Georgia</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/augusta-georgia-aim-week-mobile-studio-day-tickets-2002228326824?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>Please sign up for a mobile studio tour slot</t>
+        </is>
+      </c>
+      <c r="K271" s="2" t="inlineStr">
+        <is>
+          <t>Event is in Augusta, Georgia (outside Atlanta, which is favorable), but the description is too vague to confirm genuine AI content—'mobile studio tour' could refer to AIM Week's AI/ML focus or could be unrelated hardware/facility tours, and without clarity on what the studio demonstrates or teaches, the AI content cannot be verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026 Annual Torrance Lecture: PO-SHEN LOH (Carnegie Mellon, Mathematician)</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>4</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D272" s="3" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Stonemill Run · UGA Chapel</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/2026-annual-torrance-lecture-po-shen-loh-carnegie-mellon-mathematician-tickets-2000999110204?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>World-renowned mathematician Po-Shen Loh delivers a lecture titled "Building a Thought Full World: Creativity + Love of Humanity," discussing how AI and technology are affecting society, the importance of human connection and creativity, and his innovations in education combining math, actors, and live-streaming.</t>
+        </is>
+      </c>
+      <c r="K272" s="2" t="inlineStr">
+        <is>
+          <t>In-person educational AI event at UGA (Georgia university) with a renowned speaker discussing AI's societal impact, human connection, and AI-informed educational innovation, though it is a single lecture rather than a builder-focused meetup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>AI Made Simple: Understand. Explore. Apply. For Real Life</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>3</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D273" s="3" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Arrowind · Woodland Grove Townhomes</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-made-simple-understand-explore-apply-for-real-life-tickets-2001395814758?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>A free, beginner-friendly community workshop to understand AI in plain language, explore commonly used AI tools like ChatGPT and Claude, and discover practical applications for work, business, and daily life. Includes a live AI demonstration. No tech background required.</t>
+        </is>
+      </c>
+      <c r="K273" s="2" t="inlineStr">
+        <is>
+          <t>This is a legitimate beginner-friendly AI educational event with clear AI content (ChatGPT, Claude, practical applications) and an in-person format in Georgia, but it scores 3 rather than higher because it appears to be a one-time community workshop rather than a builder/networking event, the location (Arrowind townhomes) suggests a small local venue rather than an established organization, and the listing provides minimal detail about the host organization or speaker expertise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Where is AI in 2026 and Where is it Going?</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>3</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D274" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Germany · Rabun County Public Library</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/where-is-ai-in-2026-and-where-is-it-going-tickets-2002586897318?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="inlineStr">
+        <is>
+          <t>This workshop will explore where AI may be in the next 1-5 years and what that means for daily life for all of us.</t>
+        </is>
+      </c>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>Educational AI event with genuine AI content held in-person in rural Georgia (Rabun County), outside metro Atlanta, but limited by a brief description that suggests a general exploration rather than a technical builder or deep-dive format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>AI-Powered Blueprint: From Your Course Idea to Market Domination</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>2</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>10:00 AM PDT</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-powered-blueprint-from-your-course-idea-to-market-domination-tickets-2001867032182?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to leverage AI to pick the right topic, validate your idea, and launch a successful online course. Discover how to use AI to find your perfect topic, understand your ideal audience, and ensure your course stands out in today's digital world.</t>
+        </is>
+      </c>
+      <c r="K275" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (using AI to validate course ideas and find topics), but lacks a location statement despite is_in_person:true, has no Georgia tie, and reads as a sales-oriented course-launching workshop rather than a technical AI builder event or educational conference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>AI Compliance in Business and Technology</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>3</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D276" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>11:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr"/>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-compliance-in-business-and-technology-tickets-2002541859609?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to ensure AI compliance in your business. This webinar breaks down six documented AI incidents, explains which US and EU regulations apply to your company, and provides a 90-day governance plan to account for and comply with all AI systems using a simple spreadsheet approach.</t>
+        </is>
+      </c>
+      <c r="K276" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (AI compliance, regulations, governance) and educational value, but the listing describes it as a webinar despite is_in_person being set to true, making it virtual-only with no stated Georgia host or affiliation, which caps it at 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>How to Build an AI Agent: A Live Hands-On Workshop</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>3</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D277" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>11:00 AM CDT</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr"/>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/how-to-build-an-ai-agent-a-live-hands-on-workshop-tickets-2002852151701?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="inlineStr">
+        <is>
+          <t>Learn to build an AI agent that does real work for your business in this hands-on workshop. Discover how to set up human-in-the-loop AI where the AI drafts and you approve, covering task selection, step-by-step setup, approval workflows, and practical prompts you can use immediately.</t>
+        </is>
+      </c>
+      <c r="K277" s="2" t="inlineStr">
+        <is>
+          <t>This is a genuine hands-on AI builder workshop with strong practical content on AI agents and human-in-the-loop systems, but the missing location and no confirmed Georgia tie prevent a higher score despite the excellent workshop format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Start Your Machine Learning &amp; AI Engineering Career | Free 3-Hour Training</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>2</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr"/>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr"/>
+      <c r="G278" t="inlineStr"/>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/start-your-machine-learning-ai-engineering-career-free-3-hour-training-tickets-2001696889280?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>A free 3-hour live online training covering Machine Learning fundamentals (Pandas, regression, decision trees, model evaluation, feature engineering) and AI Engineering concepts (LLMs, tokenization, embeddings, LLM APIs, tool calling, AI agents), plus a career roadmap. Designed for U.S.-based students, recent graduates, and beginners with no prior ML/AI experience required.</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>Event has strong AI/ML educational content and is free, but is explicitly virtual-only ('live online training'), lacks any Georgia organizational tie or focus, and has no location or date information provided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr"/>
+      <c r="C279" t="inlineStr"/>
+      <c r="D279" s="3" t="inlineStr"/>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr"/>
+      <c r="G279" t="inlineStr"/>
+      <c r="H279" t="inlineStr"/>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr"/>
+      <c r="K279" s="2" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Speaker Series: How AI is Impacting Cloud vs. On-Premise Strategies</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>3</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D280" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr"/>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/speaker-series-the-great-cloud-repatriation-why-60-of-companies-are-moving-workloads-back-on-premise/</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr"/>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>The event has AI content in its title and appears to be hosted by Tech North Atlanta (a Georgia organization), but the missing description and vague framing make it difficult to assess whether this is a substantive AI discussion or a vendor pitch; it reads as an educational speaker series rather than a hands-on builder event, and without location details confirmed as in-person, confidence is moderate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>AI Builders Meetup</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>5</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D281" s="3" t="n">
+        <v>46336</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr"/>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/1998165850849?aff=oddtdtcreator</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>A live show-and-tell for builders where 5-7 AI builders share what they're building, their approach, tools, tech stacks, and lessons learned. For founders, entrepreneurs, product managers, software engineers, and AI enthusiasts.</t>
+        </is>
+      </c>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>This is an in-person AI builder meetup in Georgia (hosted by Atlanta AI Tinkerers based on the event format and Eventbrite link pattern) featuring live demos and technical talks from builders on their tools, tech stacks, and lessons learned—exactly the type of hands-on community event the client most wants to attend.</t>
         </is>
       </c>
     </row>
@@ -12300,7 +13420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K377"/>
+  <dimension ref="A1:K422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -29520,7 +30640,6 @@
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="G354" t="inlineStr"/>
       <c r="H354" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/12FOd6XigCVCB</t>
@@ -29569,7 +30688,6 @@
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="G355" t="inlineStr"/>
       <c r="H355" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/women-of-gma-virtual-networking-event-10326</t>
@@ -30353,7 +31471,6 @@
           <t>8:00 PM GMT+5:30</t>
         </is>
       </c>
-      <c r="G371" t="inlineStr"/>
       <c r="H371" t="inlineStr">
         <is>
           <t>https://www.eventbrite.ca/e/who-when-where-the-data-activity-story-cloak-dsp-tickets-2001691276492?aff=ebdssbdestsearch</t>
@@ -30674,6 +31791,2215 @@
       <c r="K377" s="2" t="inlineStr">
         <is>
           <t>The event title and description contain zero mention of AI, machine learning, or automation—it is purely about startup funding and investor relations, triggering the automatic-1 rule regardless of location or host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Honoring Those Who Served: Veterans Day Luncheon &amp; Panel presented by TAG Infrastructure Society</t>
+        </is>
+      </c>
+      <c r="B378" t="n">
+        <v>1</v>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D378" s="3" t="n">
+        <v>46331</v>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>11:30 AM</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr"/>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/ZRFWY64HgCeC2</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J378" s="2" t="inlineStr"/>
+      <c r="K378" s="2" t="inlineStr">
+        <is>
+          <t>The event title and available description contain zero mention of AI, machine learning, or automation - it is a Veterans Day luncheon and panel with no stated AI component, triggering the automatic-1 rule regardless of the TAG host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Change Tracking in SQL Server 2025: Exploring Change Event Streaming vs CDC</t>
+        </is>
+      </c>
+      <c r="B379" t="n">
+        <v>1</v>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D379" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>12:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/dba-fundamentals-group/events/315588802/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-online&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J379" s="2" t="inlineStr"/>
+      <c r="K379" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is about SQL Server database change tracking features, which is a standard database administration topic unrelated to AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Cybersecurity n' Chill Networking Monthly Meetup by BlackHack Society</t>
+        </is>
+      </c>
+      <c r="B380" t="n">
+        <v>1</v>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D380" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr"/>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/blackhack-society-atlanta/events/314101555/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J380" s="2" t="inlineStr"/>
+      <c r="K380" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a cybersecurity networking meetup with no stated AI component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Open House!</t>
+        </is>
+      </c>
+      <c r="B381" t="n">
+        <v>1</v>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D381" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>7:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr"/>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/freeside-atlanta/events/312398748/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J381" s="2" t="inlineStr">
+        <is>
+          <t>Join Freeside Atlanta for an open house where engineers, programmers, inventors, and artists collaborate. A quick meeting introduces everyone and updates on projects and equipment, followed by an informal open house to chat, tour the space, and see cool equipment.</t>
+        </is>
+      </c>
+      <c r="K381" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation; it is a general makerspace open house with no AI-specific component, session, speaker, or theme stated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>AI Mastery With Armand Morin</t>
+        </is>
+      </c>
+      <c r="B382" t="n">
+        <v>1</v>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D382" s="3" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>10:00 AM PDT</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr"/>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-mastery-with-armand-morin-tickets-2002955088588?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t>Learn directly from Armand Morin in this online event covering AI skills and insider tips. Whether you're a beginner or looking to sharpen your skills, gain hands-on insights on AI in a fun and interactive experience.</t>
+        </is>
+      </c>
+      <c r="K382" s="2" t="inlineStr">
+        <is>
+          <t>The event is described as 'online' in the short description, making it virtual-only, and there is no Georgia host or organization indicated to qualify it under the Georgia-focused virtual event exception, nor any indication this is a TAG event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Start Your Cybersecurity Career| Free 3-Hour Live Training &amp; Career Roadmap</t>
+        </is>
+      </c>
+      <c r="B383" t="n">
+        <v>1</v>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>10:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr"/>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/start-your-cybersecurity-career-free-3-hour-live-training-career-roadmap-tickets-2001641954970?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J383" s="2" t="inlineStr"/>
+      <c r="K383" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a cybersecurity career training event with no stated AI component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Info Session-10 Cyber Work Role Pathways + Job Placement Assistance</t>
+        </is>
+      </c>
+      <c r="B384" t="n">
+        <v>1</v>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D384" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>University of Louisville</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/info-session-10-cyber-work-role-pathways-job-placement-assistance-tickets-2002433211640?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J384" s="2" t="inlineStr"/>
+      <c r="K384" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is about cybersecurity career pathways and job placement, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>BSidesAugusta 2026</t>
+        </is>
+      </c>
+      <c r="B385" t="n">
+        <v>1</v>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D385" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>7:45 AM</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>Greene Street Historic District · Georgia Cyber Innovation &amp; Training Center</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/bsidesaugusta-2026-tickets-1996239645517?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J385" s="2" t="inlineStr"/>
+      <c r="K385" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; BSides is a cybersecurity conference with no stated AI-specific component in this listing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>American Modelica and FMI Conference 2026</t>
+        </is>
+      </c>
+      <c r="B386" t="n">
+        <v>1</v>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D386" s="3" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>Georgia Tech · 275 Ferst Dr NW</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/american-modelica-and-fmi-conference-2026-tickets-1982451921062?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J386" s="2" t="inlineStr"/>
+      <c r="K386" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description; Modelica and FMI are simulation and model-exchange standards with no inherent AI component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Security Onion Conference (SOC) 2026</t>
+        </is>
+      </c>
+      <c r="B387" t="n">
+        <v>1</v>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D387" s="3" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>8:00 AM</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>Greene Street Historic District · Georgia Cyber Innovation and Training Center (aka Georgia Cyber Center)</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/security-onion-conference-soc-2026-tickets-1993478356427?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J387" s="2" t="inlineStr">
+        <is>
+          <t>The twelfth annual Security Onion Conference featuring community members giving talks about tools and techniques for network and host visibility, intrusion detection, log management, and case management. Meet with other members of the community, enjoy presentations about Security Onion and blue team topics, and learn valuable security skills.</t>
+        </is>
+      </c>
+      <c r="K387" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains no mention of AI, machine learning, or automation—it focuses on Security Onion tools for network visibility, intrusion detection, and log management, which are cybersecurity infrastructure topics rather than AI/ML content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Women + Tech Meetup</t>
+        </is>
+      </c>
+      <c r="B388" t="n">
+        <v>1</v>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D388" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>North Buckhead · Atlanta Tech Village</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/women-tech-meetup-tickets-1979762040557?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J388" s="2" t="inlineStr"/>
+      <c r="K388" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Music of the Spheres II: An Immersive Experience with Live Choral Music</t>
+        </is>
+      </c>
+      <c r="B389" t="n">
+        <v>1</v>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D389" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>11:30 AM</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>Young Harris · O. Wayne Rollins Planetarium</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/music-of-the-spheres-ii-an-immersive-experience-with-live-choral-music-tickets-1998988461299?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J389" s="2" t="inlineStr"/>
+      <c r="K389" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description; it is an immersive choral music experience at a planetarium with no stated AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Fall '26 Voice and Conversations on the Net</t>
+        </is>
+      </c>
+      <c r="B390" t="n">
+        <v>1</v>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D390" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>Whispering Pines · Sandy Springs Performing Arts Center</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/fall-26-voice-and-conversations-on-the-net-tickets-1986769647498?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J390" s="2" t="inlineStr"/>
+      <c r="K390" s="2" t="inlineStr">
+        <is>
+          <t>The event title and empty description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Security Onion Fundamentals for Analysts &amp; Admins Oct 2026 @BSidesAugusta</t>
+        </is>
+      </c>
+      <c r="B391" t="n">
+        <v>1</v>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D391" s="3" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>8:00 AM</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>Greene Street Historic District · Georgia Cyber Center Hull McKnight Building</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/security-onion-fundamentals-for-analysts-admins-oct-2026-bsidesaugusta-registration-1988783011524?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J391" s="2" t="inlineStr"/>
+      <c r="K391" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is about cybersecurity tools (Security Onion) and network analysis, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Global CISO Forum 2026</t>
+        </is>
+      </c>
+      <c r="B392" t="n">
+        <v>1</v>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D392" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>8:00 AM</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>Downtown · Westin Peachtree Plaza</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/global-ciso-forum-2026-tickets-1999809692624?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t>An invite-only, closed-door gathering of CISOs and security leaders for trusted peer discussions on the most pressing issues in information security. Features closed-door sessions, interactive discussions, and curated roundtables designed for C-suite and senior security executives to exchange lessons learned and forward-looking strategies.</t>
+        </is>
+      </c>
+      <c r="K392" s="2" t="inlineStr">
+        <is>
+          <t>Event is restricted to an invite-only, closed-door gathering for CISOs and security leaders only, with no public registration path available, making it inaccessible to the client's audience regardless of its security focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>PMP Certification Training in Atlanta, GA | PMI Exam Prep</t>
+        </is>
+      </c>
+      <c r="B393" t="n">
+        <v>1</v>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D393" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>Downtown · 260 Peachtree St suite 2200</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/pmp-certification-training-in-atlanta-ga-pmi-exam-prep-tickets-1973135226578?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J393" s="2" t="inlineStr"/>
+      <c r="K393" s="2" t="inlineStr">
+        <is>
+          <t>The event is PMP certification training with no mention of AI, machine learning, or automation in the title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>PMP Certification Training in Augusta, GA | PMI Exam Prep</t>
+        </is>
+      </c>
+      <c r="B394" t="n">
+        <v>1</v>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D394" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>Greene Street Historic District · 823 Broad St</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/pmp-certification-training-in-augusta-ga-pmi-exam-prep-tickets-1973124928777?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J394" s="2" t="inlineStr"/>
+      <c r="K394" s="2" t="inlineStr">
+        <is>
+          <t>The event is PMP certification training with no mention of AI, machine learning, or automation in the title or description, triggering the automatic 1 rating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>The Super Science Day of the Girl 2026</t>
+        </is>
+      </c>
+      <c r="B395" t="n">
+        <v>1</v>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D395" s="3" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>Downtown · First Congregational Church, UCC</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/the-super-science-day-of-the-girl-2026-tickets-1997717796707?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J395" s="2" t="inlineStr"/>
+      <c r="K395" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>MICROLOCK SELF RETIGHTENING MADE EASY!</t>
+        </is>
+      </c>
+      <c r="B396" t="n">
+        <v>1</v>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D396" s="3" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>North Atlanta · 705 Town Blvd</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/microlock-self-retightening-made-easy-tickets-1903263234569?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J396" s="2" t="inlineStr"/>
+      <c r="K396" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is about microlock self-retightening hardware—triggering the automatic 1 regardless of location or other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Building High-Performing Teams: A 1-Day Course in Atlanta</t>
+        </is>
+      </c>
+      <c r="B397" t="n">
+        <v>1</v>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D397" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Downtown · Regus - Atlanta - 260 Peachtree</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.sg/e/building-high-performing-teams-a-1-day-course-in-atlanta-tickets-2002257229272?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J397" s="2" t="inlineStr"/>
+      <c r="K397" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is about building high-performing teams, which is a management/HR topic, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026 VWR Fall Research Festival &amp; Vendor Show at Emory</t>
+        </is>
+      </c>
+      <c r="B398" t="n">
+        <v>1</v>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D398" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Clifton Community · 605 Asbury Cir</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/2026-vwr-fall-research-festival-vendor-show-at-emory-tickets-1999707841986?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J398" s="2" t="inlineStr"/>
+      <c r="K398" s="2" t="inlineStr">
+        <is>
+          <t>The event description is empty with no mention of AI, machine learning, or automation, triggering the automatic-1 rule; it appears to be a general research festival and vendor show rather than an AI-focused event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Launch Your Cybersecurity Career- Cyber Work Role Pathways with UofL DTC</t>
+        </is>
+      </c>
+      <c r="B399" t="n">
+        <v>1</v>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D399" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr"/>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/launch-your-cybersecurity-career-cyber-work-role-pathways-with-uofl-dtc-tickets-2002439958821?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J399" s="2" t="inlineStr"/>
+      <c r="K399" s="2" t="inlineStr">
+        <is>
+          <t>The event title and available details make no mention of AI, machine learning, or automation—it is a cybersecurity career pathways event, which triggers the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Plant. Eat. Repeat. at Astro-Fain Community Garden</t>
+        </is>
+      </c>
+      <c r="B400" t="n">
+        <v>1</v>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D400" s="3" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>Adamsville · Astro-Fain Community Garden</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/plant-eat-repeat-at-astro-fain-community-garden-tickets-2000184360265?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J400" s="2" t="inlineStr"/>
+      <c r="K400" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Plant. Eat. Repeat. at North Cobb Regional Library Community Garden</t>
+        </is>
+      </c>
+      <c r="B401" t="n">
+        <v>1</v>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D401" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>Lakeview Heights · North Cobb Regional Library Community Garden</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/plant-eat-repeat-at-north-cobb-regional-library-community-garden-tickets-2000190271947?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J401" s="2" t="inlineStr"/>
+      <c r="K401" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a community garden event about planting and eating—triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Plant. Eat. Repeat. at Community Garden of Jonesboro</t>
+        </is>
+      </c>
+      <c r="B402" t="n">
+        <v>1</v>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D402" s="3" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Jonesboro · Community Garden of Jonesboro</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/plant-eat-repeat-at-community-garden-of-jonesboro-tickets-2000189362226?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J402" s="2" t="inlineStr"/>
+      <c r="K402" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule regardless of location or other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Vermicomposting with Cobb Extension</t>
+        </is>
+      </c>
+      <c r="B403" t="n">
+        <v>1</v>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D403" s="3" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Whitlock · Switzer Library</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/vermicomposting-with-cobb-extension-tickets-2001635782508?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J403" s="2" t="inlineStr"/>
+      <c r="K403" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Cyber Safety for Gamers Workshop</t>
+        </is>
+      </c>
+      <c r="B404" t="n">
+        <v>1</v>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D404" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Abbey Hill · Alpha Esports and Technology</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/cyber-safety-for-gamers-workshop-tickets-2002920251389?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J404" s="2" t="inlineStr"/>
+      <c r="K404" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation—it is about cyber safety for gamers, which is a cybersecurity topic unrelated to AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Plant. Eat. Repeat. at EMBARC Community Youth Farm</t>
+        </is>
+      </c>
+      <c r="B405" t="n">
+        <v>1</v>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D405" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Georgia · E.M.B.A.R.C. Community Youth Farm</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/plant-eat-repeat-at-embarc-community-youth-farm-tickets-2000187561841?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J405" s="2" t="inlineStr"/>
+      <c r="K405" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, and appears to be about community gardening and food cultivation rather than any AI-related topic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Visiting the Jekyll Island Banding Station with Sue Killeen</t>
+        </is>
+      </c>
+      <c r="B406" t="n">
+        <v>1</v>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>8:00 AM</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Georgia · 100 St Andrews Dr</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/visiting-the-jekyll-island-banding-station-with-sue-killeen-tickets-1998964187696?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J406" s="2" t="inlineStr"/>
+      <c r="K406" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description; it is about bird banding at Jekyll Island, which is entirely unrelated to the client's focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>The Value of Cover Crops Workshop</t>
+        </is>
+      </c>
+      <c r="B407" t="n">
+        <v>1</v>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D407" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>Blandtown · Souper Jenny's Farm</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/the-value-of-cover-crops-workshop-tickets-1999090680038?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J407" s="2" t="inlineStr"/>
+      <c r="K407" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>BigFix Connect - Atlanta Area User Group</t>
+        </is>
+      </c>
+      <c r="B408" t="n">
+        <v>1</v>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D408" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>North Buckhead · Maggiano's Little Italy</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/bigfix-connect-atlanta-area-user-group-tickets-2000508948116?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J408" s="2" t="inlineStr"/>
+      <c r="K408" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a BigFix user group meeting where BigFix is enterprise systems management software with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B409" t="n">
+        <v>1</v>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D409" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Georgia · Browns Mill Recreation Center</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J409" s="2" t="inlineStr"/>
+      <c r="K409" s="2" t="inlineStr">
+        <is>
+          <t>The event title and empty description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule regardless of location or host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B410" t="n">
+        <v>1</v>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D410" s="3" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>Linwood Heights · East Point Library</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J410" s="2" t="inlineStr"/>
+      <c r="K410" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics outreach and build program focused on hardware and hands-on STEM activities rather than AI concepts like machine perception, autonomy, or reinforcement learning, fitting the automatic-1 category for robotics events centered on the build rather than AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Dahlonega Science Cafe Presentation</t>
+        </is>
+      </c>
+      <c r="B411" t="n">
+        <v>1</v>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D411" s="3" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>Dahlonega · Bourbon Street Grille</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/dahlonega-science-cafe-presentation-tickets-2002838128758?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J411" s="2" t="inlineStr">
+        <is>
+          <t>Join us for our monthly Science Cafe Presentation where curious minds gather to explore cool science topics in a relaxed setting. Grab a seat, bring your questions, and enjoy engaging discussions while you enjoy dinner at Bourbon Street Grille.</t>
+        </is>
+      </c>
+      <c r="K411" s="2" t="inlineStr">
+        <is>
+          <t>The event description mentions only a general 'cool science topics' monthly presentation with no specific mention of AI, machine learning, automation, or any AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Experience STEMM the AIM Way!</t>
+        </is>
+      </c>
+      <c r="B412" t="n">
+        <v>1</v>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D412" s="3" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>Lindbergh/Morosgo · 2450 Piedmont Rd NE</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/experience-stemm-the-aim-way-tickets-2002749607990?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J412" s="2" t="inlineStr"/>
+      <c r="K412" s="2" t="inlineStr">
+        <is>
+          <t>The event title and short description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Watershed Education Workshop</t>
+        </is>
+      </c>
+      <c r="B413" t="n">
+        <v>1</v>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D413" s="3" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>7:00 PM</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>Whitlock · Cobb County Water Lab Training Room</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/watershed-education-workshop-tickets-1990881992633?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J413" s="2" t="inlineStr"/>
+      <c r="K413" s="2" t="inlineStr">
+        <is>
+          <t>The event title and available description contain zero mention of AI, machine learning, or automation; it is a watershed/water education workshop with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>WBU Athens Bat Presentation with Ranger Auggie of Hard Labor Creek</t>
+        </is>
+      </c>
+      <c r="B414" t="n">
+        <v>1</v>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D414" s="3" t="n">
+        <v>46320</v>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>3:30 PM</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>Beechwood Hills · Wild Birds Unlimited</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/wbu-athens-bat-presentation-with-ranger-auggie-of-hard-labor-creek-tickets-1999421962914?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J414" s="2" t="inlineStr"/>
+      <c r="K414" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a bat presentation by a park ranger at a Wild Birds Unlimited location in Athens, Georgia, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Start Your DevOps Career | Free 3-Hour Live Training &amp; Career Roadmap</t>
+        </is>
+      </c>
+      <c r="B415" t="n">
+        <v>1</v>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D415" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>10:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr"/>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/start-your-devops-career-free-3-hour-live-training-career-roadmap-tickets-2001700803989?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J415" s="2" t="inlineStr"/>
+      <c r="K415" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is about DevOps career training, which is unrelated to AI, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Tokenized Collectibles</t>
+        </is>
+      </c>
+      <c r="B416" t="n">
+        <v>1</v>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D416" s="3" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>Castleberry Hill · 504 Fair St SW</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tokenized-collectibles-tickets-2002920765928?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J416" s="2" t="inlineStr"/>
+      <c r="K416" s="2" t="inlineStr">
+        <is>
+          <t>The event title and empty description contain zero mention of AI, machine learning, or automation; 'tokenized collectibles' refers to blockchain/NFT technology with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Black Boys Code DeKalb - Sequencing Robots in Motion</t>
+        </is>
+      </c>
+      <c r="B417" t="n">
+        <v>1</v>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D417" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>Clifton Community · Emory University</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/black-boys-code-dekalb-sequencing-robots-in-motion-tickets-2002918723820?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J417" s="2" t="inlineStr">
+        <is>
+          <t>A hands-on LEGO Robotics workshop for boys aged 8-17 where students build and program robots using LEGO SPIKE Prime. Beginners learn loops and create a driving robot, while advanced learners use Python to work with variables, gear ratios, and drivetrain calibration. All materials provided.</t>
+        </is>
+      </c>
+      <c r="K417" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics build-and-workshop event focused on LEGO hardware and basic programming instruction rather than AI, machine learning, or autonomy, which falls under the robotics-competition category that scores 1 regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Black Boys Code Toronto - Build the Web</t>
+        </is>
+      </c>
+      <c r="B418" t="n">
+        <v>1</v>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D418" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>Georgia · TBD</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/black-boys-code-toronto-build-the-web-tickets-2002921342653?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J418" s="2" t="inlineStr"/>
+      <c r="K418" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; it is a youth coding workshop with no stated AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Black Boys Code Gwinnett County - Sequencing Robots in Motion</t>
+        </is>
+      </c>
+      <c r="B419" t="n">
+        <v>1</v>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D419" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>Georgia · Gwinnett Technical College</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/black-boys-code-gwinnett-county-sequencing-robots-in-motion-tickets-2002918694733?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J419" s="2" t="inlineStr">
+        <is>
+          <t>A hands-on LEGO Robotics workshop for boys aged 8-17 where students build and program robots using LEGO SPIKE Prime. Beginners learn loops and create a driving robot, while advanced learners use Python to work with variables, gear ratios, and drivetrain calibration. All materials provided.</t>
+        </is>
+      </c>
+      <c r="K419" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics build-and-program workshop focused on LEGO hardware construction and basic programming sequencing, not on AI, machine learning, or autonomy—it falls squarely into the robotics-hardware-and-build category that scores 1 per the criteria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Black Boys Code Atlanta - Sequencing Robots in Motion</t>
+        </is>
+      </c>
+      <c r="B420" t="n">
+        <v>1</v>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D420" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>Sylvan Hills · Atlanta Metropolitan State College (Building 100)</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.ca/e/black-boys-code-atlanta-sequencing-robots-in-motion-tickets-2002918623520?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J420" s="2" t="inlineStr">
+        <is>
+          <t>An exciting hands-on LEGO Robotics workshop for boys aged 8-17. Students build and program LEGO SPIKE Prime robots, learning coding concepts like loops, variables, and Python. Beginners create driving robots, while advanced learners work with calibrated drivetrains and real-world engineering calculations. All materials provided.</t>
+        </is>
+      </c>
+      <c r="K420" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics build-and-compete workshop focused on LEGO hardware construction and basic coding instruction, not on AI/machine learning/autonomy, which triggers the automatic-1 rule for robotics events about the build rather than AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>🍖 BitDevs: Bitcoin Socratic Seminar #55 - pre-TABConf BBQ</t>
+        </is>
+      </c>
+      <c r="B421" t="n">
+        <v>1</v>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D421" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>6:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>684 John Wesley Dobbs Ave NE suite a1, Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/315044442/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J421" s="2" t="inlineStr">
+        <is>
+          <t>Kick off TABConf week with Atlanta BitDevs Socratic Seminar #55 + BBQ at ATL BitLab. Dig into the latest developments in Bitcoin and Lightning with the local BitDevs crew and fellow conference-goers. HODLBarbarian and Jesse are cooking up a home-cooked BBQ feast right at the Lab. Come early to eat BBQ (6:00–7:00 PM), then join the Socratic Seminar (7:15–9:00 PM). Get a meal ticket separately.</t>
+        </is>
+      </c>
+      <c r="K421" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a Bitcoin and Lightning Network discussion seminar with a BBQ social component, which triggers the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Startup Workshop: The Current Climate for Investor Funding, Pre-Seed Through Series A</t>
+        </is>
+      </c>
+      <c r="B422" t="n">
+        <v>1</v>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D422" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>October 5, 2026</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr"/>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/2002457508312?aff=oddtdtcreator</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J422" s="2" t="inlineStr"/>
+      <c r="K422" s="2" t="inlineStr">
+        <is>
+          <t>The event title and available details make no mention of AI, machine learning, or automation, triggering the automatic-1 rule for events with zero AI content.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-10-12
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K281" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K293" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K422" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K433" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K281"/>
+  <dimension ref="A1:K293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -12327,17 +12327,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B259" t="inlineStr"/>
-      <c r="C259" t="inlineStr"/>
       <c r="D259" s="3" t="inlineStr"/>
       <c r="E259" t="inlineStr">
         <is>
           <t>October 5, 2026</t>
         </is>
       </c>
-      <c r="F259" t="inlineStr"/>
-      <c r="G259" t="inlineStr"/>
-      <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -12373,7 +12368,6 @@
           <t>3:00 PM EDT</t>
         </is>
       </c>
-      <c r="G260" t="inlineStr"/>
       <c r="H260" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/316692853/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
@@ -12528,7 +12522,6 @@
           <t>5:00 PM EDT</t>
         </is>
       </c>
-      <c r="G263" t="inlineStr"/>
       <c r="H263" t="inlineStr">
         <is>
           <t>https://www.meetup.com/ai-ship-and-social/events/316770121/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
@@ -12552,17 +12545,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr"/>
-      <c r="C264" t="inlineStr"/>
       <c r="D264" s="3" t="inlineStr"/>
       <c r="E264" t="inlineStr">
         <is>
           <t>October 5, 2026</t>
         </is>
       </c>
-      <c r="F264" t="inlineStr"/>
-      <c r="G264" t="inlineStr"/>
-      <c r="H264" t="inlineStr"/>
       <c r="I264" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -13124,7 +13112,6 @@
           <t>10:00 AM PDT</t>
         </is>
       </c>
-      <c r="G275" t="inlineStr"/>
       <c r="H275" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-powered-blueprint-from-your-course-idea-to-market-domination-tickets-2001867032182?aff=ebdssbdestsearch</t>
@@ -13173,7 +13160,6 @@
           <t>11:00 AM EDT</t>
         </is>
       </c>
-      <c r="G276" t="inlineStr"/>
       <c r="H276" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-compliance-in-business-and-technology-tickets-2002541859609?aff=ebdssbdestsearch</t>
@@ -13222,7 +13208,6 @@
           <t>11:00 AM CDT</t>
         </is>
       </c>
-      <c r="G277" t="inlineStr"/>
       <c r="H277" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/how-to-build-an-ai-agent-a-live-hands-on-workshop-tickets-2002852151701?aff=ebdssbdestsearch</t>
@@ -13264,8 +13249,6 @@
           <t>October 5, 2026</t>
         </is>
       </c>
-      <c r="F278" t="inlineStr"/>
-      <c r="G278" t="inlineStr"/>
       <c r="H278" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/start-your-machine-learning-ai-engineering-career-free-3-hour-training-tickets-2001696889280?aff=ebdssbdestsearch</t>
@@ -13293,17 +13276,12 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr"/>
-      <c r="C279" t="inlineStr"/>
       <c r="D279" s="3" t="inlineStr"/>
       <c r="E279" t="inlineStr">
         <is>
           <t>October 5, 2026</t>
         </is>
       </c>
-      <c r="F279" t="inlineStr"/>
-      <c r="G279" t="inlineStr"/>
-      <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -13339,7 +13317,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G280" t="inlineStr"/>
       <c r="H280" t="inlineStr">
         <is>
           <t>https://technorthatlanta.org/event/speaker-series-the-great-cloud-repatriation-why-60-of-companies-are-moving-workloads-back-on-premise/</t>
@@ -13384,7 +13361,6 @@
           <t>5:30 PM - 7:30 PM</t>
         </is>
       </c>
-      <c r="G281" t="inlineStr"/>
       <c r="H281" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/1998165850849?aff=oddtdtcreator</t>
@@ -13405,6 +13381,510 @@
           <t>This is an in-person AI builder meetup in Georgia (hosted by Atlanta AI Tinkerers based on the event format and Eventbrite link pattern) featuring live demos and technical talks from builders on their tools, tech stacks, and lessons learned—exactly the type of hands-on community event the client most wants to attend.</t>
         </is>
       </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Beyond Connected: Powering the Future of AI, IoT, and the Intelligent Edge presented by TAG Cloud Society</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>5</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="n">
+        <v>46366</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>5:15 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr"/>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/dxFKQdzfoC0Cv</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="inlineStr">
+        <is>
+          <t>An executive panel exploring how leading organizations are transforming connected devices into intelligent, business-driven ecosystems.</t>
+        </is>
+      </c>
+      <c r="K282" s="2" t="inlineStr">
+        <is>
+          <t>TAG Cloud Society event with genuine AI content (intelligent edge, AI-driven ecosystems) hosted by TAG, Georgia's premier tech organization, scoring the automatic 5 for TAG events with clear AI components.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr"/>
+      <c r="C283" t="inlineStr"/>
+      <c r="D283" s="3" t="inlineStr"/>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr"/>
+      <c r="G283" t="inlineStr"/>
+      <c r="H283" t="inlineStr"/>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr"/>
+      <c r="K283" s="2" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr"/>
+      <c r="C284" t="inlineStr"/>
+      <c r="D284" s="3" t="inlineStr"/>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr"/>
+      <c r="G284" t="inlineStr"/>
+      <c r="H284" t="inlineStr"/>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr"/>
+      <c r="K284" s="2" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr"/>
+      <c r="C285" t="inlineStr"/>
+      <c r="D285" s="3" t="inlineStr"/>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr"/>
+      <c r="G285" t="inlineStr"/>
+      <c r="H285" t="inlineStr"/>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr"/>
+      <c r="K285" s="2" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>AI Builders Global Conference 2026</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>2</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D286" s="3" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>9:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr"/>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-builders-global-conference-2026-tickets-2002917814099?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>A 3-day virtual conference bringing together 12,000+ AI executives, engineers, founders, and investors from 130+ countries. Features 200+ sessions across 8 tracks, 10+ workshops, an AI Startup Pitch Competition with cash prizes, and investor networking with 1:1 matchmaking. Includes Chief in AI Summit, Startups and Investors Summit, and AI Engineering Day.</t>
+        </is>
+      </c>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>This is a virtual-only conference (stated explicitly as 'virtual conference' in the description) with no Georgia host or organizational tie, making it ineligible for the higher scoring that would apply to in-person Georgia events or Georgia-hosted virtual events, despite strong AI content and multi-day format.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>AI can build your EDC, but it can't shape your culture</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>3</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D287" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>10:00 AM CDT</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr"/>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-can-build-your-edc-but-it-cant-shape-your-culture-tickets-2003032338645?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>A practical look at how organizations can introduce AI into clinical data management. Explore how AI can enhance data management, reshape workflows, and what's needed for responsible AI adoption including people, processes, and governance.</t>
+        </is>
+      </c>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content focused on clinical data management and responsible AI adoption, but lacks a specified location, has no clear Georgia tie, and the thin description and missing venue details create uncertainty about the event's format and accessibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>MENTORSHOP: Using Claude AI to Build a SaaS Site in about a Week</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>2</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D288" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>12:00 PM PDT</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr"/>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/mentorshop-using-claude-ai-to-build-a-saas-site-in-about-a-week-tickets-2003024863286?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to build a SaaS business using Claude AI in about a week. This workshop covers using Claude AI to code solutions, making code maintainable, accepting payments, and web hosting/security. Perfect for entrepreneurs, out-of-work tech professionals, established businesses, non-profits, and those needing to prototype an MVP quickly.</t>
+        </is>
+      </c>
+      <c r="K288" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (Claude AI for SaaS development) but is virtual-only (PDT timezone, no location provided, 12 PM start suggests online format) with no Georgia organizational tie, scoring it at the virtual-without-Georgia-connection cap of 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Unlock The Power of AI (Level Up with AI Pt. 2)</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>4</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D289" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Villa Rica · Kingdom Dominion Church</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/unlock-the-power-of-ai-level-up-with-ai-pt-2-tickets-2003030365744?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>A FREE, hands-on workshop for all ages to discover how AI can make everyday life easier, spark creativity, and help you work smarter. Features live demonstrations of practical AI tools, simple ways to use AI at work/school/home/business/ministry, safety tips, and a live Q&amp;A. No experience required.</t>
+        </is>
+      </c>
+      <c r="K289" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI educational workshop in Villa Rica (outside metro Atlanta) with genuine hands-on AI content, free admission, and no closed-audience restrictions, scoring well for statewide reach and practical AI builder focus despite being hosted by a church rather than a traditional tech organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>BuildIt! Digital: AI Afternoon (Office Hours)</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>3</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D290" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Deerfield · 1111 Chastain Rd NW</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/buildit-digital-ai-afternoon-office-hours-tickets-2003064546981?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>Join BuildIt! Digital for practical tips and hands-on guidance on using AI in daily business operations. Drop in with AI strategist Laila Harrison to discuss workflow challenges, explore AI tools, and learn where AI could help your business.</t>
+        </is>
+      </c>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>The event has clear AI content (AI tools, AI strategy discussion) and is in-person in Georgia (Deerfield/Chastain Rd area), but it's an office-hours/drop-in format rather than a builder-focused community event with project presentations, and the host organization BuildIt! Digital is not a recognized Georgia institution, preventing a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Agentic AI for FP&amp;A: Forecasting, Variance Analysis &amp; Decision Support</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>3</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D291" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>9:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr"/>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/agentic-ai-for-fpa-forecasting-variance-analysis-decision-support-tickets-2001140331601?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="inlineStr">
+        <is>
+          <t>A 3.5-hour live, hands-on workshop teaching Finance professionals how to build agentic AI workflows for FP&amp;A tasks including forecasting, variance analysis, scenario planning, and decision support. Learn to design AI-enabled workflows that diagnose variances, challenge assumptions, generate scenarios, and produce management commentary—no coding experience required.</t>
+        </is>
+      </c>
+      <c r="K291" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (agentic AI workflows) and is hands-on/educational, but lacks a confirmed Georgia location, appears to be hosted on a UK Eventbrite domain suggesting international scope, and the missing location field creates uncertainty about accessibility to the Georgia-focused client audience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>10th Marketing AI Pulse</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>3</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D292" s="3" t="n">
+        <v>46338</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>1:30 PM</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Atlanta Tech Park</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/10th-marketing-ai-pulse-tickets-2003106787323?aff=ebdsoporgprofile</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="inlineStr">
+        <is>
+          <t>Join 150+ marketers to learn, connect, and grow intellectually and professionally as marketing leaders discuss how AI is shaping the future of marketing. Network with fellow marketers actively transforming the industry.</t>
+        </is>
+      </c>
+      <c r="K292" s="2" t="inlineStr">
+        <is>
+          <t>In-person Atlanta event with clear AI content (marketing leaders discussing how AI is shaping marketing's future) and good attendance scale, but lacks the hands-on builder/demo focus and Georgia community tie that would elevate it to 4-5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr"/>
+      <c r="C293" t="inlineStr"/>
+      <c r="D293" s="3" t="inlineStr"/>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr"/>
+      <c r="G293" t="inlineStr"/>
+      <c r="H293" t="inlineStr"/>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="inlineStr"/>
+      <c r="K293" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13420,7 +13900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K422"/>
+  <dimension ref="A1:K433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -31821,7 +32301,6 @@
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="G378" t="inlineStr"/>
       <c r="H378" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/ZRFWY64HgCeC2</t>
@@ -31915,7 +32394,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G380" t="inlineStr"/>
       <c r="H380" t="inlineStr">
         <is>
           <t>https://www.meetup.com/blackhack-society-atlanta/events/314101555/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
@@ -31960,7 +32438,6 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
-      <c r="G381" t="inlineStr"/>
       <c r="H381" t="inlineStr">
         <is>
           <t>https://www.meetup.com/freeside-atlanta/events/312398748/?recId=487620f9-b776-4c03-badb-1d4972f3be9f&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=3de92dcd-4ca8-4c6b-a13d-cdb72cea4f77&amp;eventOrigin=find_page%24all</t>
@@ -32009,7 +32486,6 @@
           <t>10:00 AM PDT</t>
         </is>
       </c>
-      <c r="G382" t="inlineStr"/>
       <c r="H382" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-mastery-with-armand-morin-tickets-2002955088588?aff=ebdssbdestsearch</t>
@@ -32058,7 +32534,6 @@
           <t>10:00 AM EDT</t>
         </is>
       </c>
-      <c r="G383" t="inlineStr"/>
       <c r="H383" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/start-your-cybersecurity-career-free-3-hour-live-training-career-roadmap-tickets-2001641954970?aff=ebdssbdestsearch</t>
@@ -32846,7 +33321,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G399" t="inlineStr"/>
       <c r="H399" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/launch-your-cybersecurity-career-cyber-work-role-pathways-with-uofl-dtc-tickets-2002439958821?aff=ebdssbdestsearch</t>
@@ -33630,7 +34104,6 @@
           <t>10:00 AM EDT</t>
         </is>
       </c>
-      <c r="G415" t="inlineStr"/>
       <c r="H415" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/start-your-devops-career-free-3-hour-live-training-career-roadmap-tickets-2001700803989?aff=ebdssbdestsearch</t>
@@ -33985,7 +34458,6 @@
           <t>12:00 PM - 1:00 PM</t>
         </is>
       </c>
-      <c r="G422" t="inlineStr"/>
       <c r="H422" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/2002457508312?aff=oddtdtcreator</t>
@@ -34000,6 +34472,535 @@
       <c r="K422" s="2" t="inlineStr">
         <is>
           <t>The event title and available details make no mention of AI, machine learning, or automation, triggering the automatic-1 rule for events with zero AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Women of GMA Virtual Networking Event 10/20/26</t>
+        </is>
+      </c>
+      <c r="B423" t="n">
+        <v>1</v>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D423" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>3:30 PM</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr"/>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/women-of-gma-virtual-networking-event-10326</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J423" s="2" t="inlineStr"/>
+      <c r="K423" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, and is a networking event rather than an educational or builder-focused AI event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>FREE Data Science Bootcamp | USA Only | Live Training | Join WhatsApp Group</t>
+        </is>
+      </c>
+      <c r="B424" t="n">
+        <v>1</v>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D424" s="3" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>10:30 AM EDT</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr"/>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-data-science-bootcamp-usa-only-live-training-join-whatsapp-group-tickets-2002085679161?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J424" s="2" t="inlineStr">
+        <is>
+          <t>FREE 10-Day Live Data Science Bootcamp with hands-on training in Python, SQL, Data Analysis, Statistics, Visualization, and Machine Learning. Designed for students, beginners, recent graduates, career switchers, data analysts, and IT professionals in the USA. Learn NumPy, Pandas, Matplotlib, Seaborn, Scikit-learn, and build real-world Data Science projects.</t>
+        </is>
+      </c>
+      <c r="K424" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event (explicitly states 'Live Training' and WhatsApp group format) with no Georgia host or tie, and while it has machine learning content, it is a national USA-only bootcamp with no Georgia connection, scoring it as a national corporate/training webinar without local relevance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>ACS Georgia Section: Herty Medal Award Dinner</t>
+        </is>
+      </c>
+      <c r="B425" t="n">
+        <v>1</v>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D425" s="3" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>Midtown · Georgia Tech Hotel and Conference Center</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/acs-georgia-section-herty-medal-award-dinner-tickets-2001710612326?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J425" s="2" t="inlineStr"/>
+      <c r="K425" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is an awards dinner for the American Chemical Society, not an AI event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>STEM on the Green Halloween</t>
+        </is>
+      </c>
+      <c r="B426" t="n">
+        <v>1</v>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D426" s="3" t="n">
+        <v>46326</v>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>Jamestown · College Park Golf Course</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/stem-on-the-green-halloween-tickets-2003067062505?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J426" s="2" t="inlineStr"/>
+      <c r="K426" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; it appears to be a general STEM outreach activity rather than an AI-focused event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B427" t="n">
+        <v>1</v>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D427" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>Linwood Heights · East Point Library</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J427" s="2" t="inlineStr"/>
+      <c r="K427" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics outreach event focused on hardware and building smart machines for ages 8-16, which falls under the robotics-competition/build-a-bot category that scores 1 regardless of AI mentions in the title, as it centers on robotics activities rather than genuine AI content like machine perception or autonomy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B428" t="n">
+        <v>1</v>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D428" s="3" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>Georgia · Browns Mill Recreation Center</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J428" s="2" t="inlineStr"/>
+      <c r="K428" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of location or host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>AI, SPAM and Medicare Fraud</t>
+        </is>
+      </c>
+      <c r="B429" t="n">
+        <v>1</v>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D429" s="3" t="n">
+        <v>46323</v>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>1:00 PM</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>Riverdale · G. Cecil Pruett Community Center Family YMCA</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-spam-and-medicare-fraud-tickets-2003199892804?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J429" s="2" t="inlineStr">
+        <is>
+          <t>Learn how to identify, prevent and report Medicare fraud.</t>
+        </is>
+      </c>
+      <c r="K429" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description mention AI only as a label but focus entirely on Medicare fraud identification and prevention with no genuine AI-focused component, session, speaker, or technical content about machine learning or automation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>NGS Seminar at Emory: Higher-Accuracy Sequencing at Lower Cost</t>
+        </is>
+      </c>
+      <c r="B430" t="n">
+        <v>1</v>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D430" s="3" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>Clifton Community · 1750 Haygood Dr NE</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ngs-seminar-at-emory-higher-accuracy-sequencing-at-lower-cost-tickets-2003023739926?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J430" s="2" t="inlineStr"/>
+      <c r="K430" s="2" t="inlineStr">
+        <is>
+          <t>The event title and available description contain zero mention of AI, machine learning, or automation—it is about sequencing technology in a genomics/biology context with no stated AI component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Blockchain Economics</t>
+        </is>
+      </c>
+      <c r="B431" t="n">
+        <v>1</v>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D431" s="3" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>Castleberry Hill · 504 Fair St SW</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/blockchain-economics-tickets-2003272159957?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J431" s="2" t="inlineStr"/>
+      <c r="K431" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule; blockchain economics is a distinct topic from AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Cybersecurity: Ethical Hacking, Blue Team &amp; Red Team | FREE Live Online</t>
+        </is>
+      </c>
+      <c r="B432" t="n">
+        <v>1</v>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D432" s="3" t="inlineStr"/>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr"/>
+      <c r="G432" t="inlineStr"/>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/cybersecurity-ethical-hacking-blue-team-red-team-free-live-online-tickets-2003205772390?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J432" s="2" t="inlineStr"/>
+      <c r="K432" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description mention only cybersecurity, ethical hacking, and red/blue team concepts with no mention of AI, machine learning, or automation, triggering the automatic-1 rule for events with zero AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Private, Event Members-Only Mixer!</t>
+        </is>
+      </c>
+      <c r="B433" t="n">
+        <v>1</v>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D433" s="3" t="n">
+        <v>46337</v>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>October 12, 2026</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>5:30 pm</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr"/>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/private-event-members-only-happy-hour/</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J433" s="2" t="inlineStr">
+        <is>
+          <t>Sponsorship opportunities are available. Event Membership info is available. Members-only mixer.</t>
+        </is>
+      </c>
+      <c r="K433" s="2" t="inlineStr">
+        <is>
+          <t>This is a members-only mixer with no AI content mentioned in the title or description, making it ineligible regardless of host or location.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-10-19
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K293" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K306" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K433" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K445" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K293"/>
+  <dimension ref="A1:K306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -13409,7 +13409,6 @@
           <t>5:15 PM - 8:00 PM</t>
         </is>
       </c>
-      <c r="G282" t="inlineStr"/>
       <c r="H282" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/dxFKQdzfoC0Cv</t>
@@ -13437,17 +13436,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr"/>
-      <c r="C283" t="inlineStr"/>
       <c r="D283" s="3" t="inlineStr"/>
       <c r="E283" t="inlineStr">
         <is>
           <t>October 12, 2026</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
-      <c r="G283" t="inlineStr"/>
-      <c r="H283" t="inlineStr"/>
       <c r="I283" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -13462,17 +13456,12 @@
           <t>https://www.meetup.com/find/?source=EVENTS&amp;categoryId=546&amp;location=us--georgia</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr"/>
-      <c r="C284" t="inlineStr"/>
       <c r="D284" s="3" t="inlineStr"/>
       <c r="E284" t="inlineStr">
         <is>
           <t>October 12, 2026</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr"/>
-      <c r="G284" t="inlineStr"/>
-      <c r="H284" t="inlineStr"/>
       <c r="I284" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -13487,17 +13476,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr"/>
-      <c r="C285" t="inlineStr"/>
       <c r="D285" s="3" t="inlineStr"/>
       <c r="E285" t="inlineStr">
         <is>
           <t>October 12, 2026</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr"/>
-      <c r="G285" t="inlineStr"/>
-      <c r="H285" t="inlineStr"/>
       <c r="I285" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -13533,7 +13517,6 @@
           <t>9:00 AM EDT</t>
         </is>
       </c>
-      <c r="G286" t="inlineStr"/>
       <c r="H286" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-builders-global-conference-2026-tickets-2002917814099?aff=ebdssbdestsearch</t>
@@ -13582,7 +13565,6 @@
           <t>10:00 AM CDT</t>
         </is>
       </c>
-      <c r="G287" t="inlineStr"/>
       <c r="H287" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/ai-can-build-your-edc-but-it-cant-shape-your-culture-tickets-2003032338645?aff=ebdssbdestsearch</t>
@@ -13631,7 +13613,6 @@
           <t>12:00 PM PDT</t>
         </is>
       </c>
-      <c r="G288" t="inlineStr"/>
       <c r="H288" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/mentorshop-using-claude-ai-to-build-a-saas-site-in-about-a-week-tickets-2003024863286?aff=ebdssbdestsearch</t>
@@ -13786,7 +13767,6 @@
           <t>9:00 AM EDT</t>
         </is>
       </c>
-      <c r="G291" t="inlineStr"/>
       <c r="H291" t="inlineStr">
         <is>
           <t>https://www.eventbrite.co.uk/e/agentic-ai-for-fpa-forecasting-variance-analysis-decision-support-tickets-2001140331601?aff=ebdssbdestsearch</t>
@@ -13867,17 +13847,12 @@
           <t>https://atlanta.aitinkerers.org/</t>
         </is>
       </c>
-      <c r="B293" t="inlineStr"/>
-      <c r="C293" t="inlineStr"/>
       <c r="D293" s="3" t="inlineStr"/>
       <c r="E293" t="inlineStr">
         <is>
           <t>October 12, 2026</t>
         </is>
       </c>
-      <c r="F293" t="inlineStr"/>
-      <c r="G293" t="inlineStr"/>
-      <c r="H293" t="inlineStr"/>
       <c r="I293" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -13885,6 +13860,615 @@
       </c>
       <c r="J293" s="2" t="inlineStr"/>
       <c r="K293" s="2" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>AI in Healthcare: Clinical Judgement, Governance &amp; Accountability presented by TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>5</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="n">
+        <v>46330</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr"/>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/EqFMN30tgC6C9</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a timely conversation on AI in Healthcare: Clinical Judgement, Governance &amp; Accountability.</t>
+        </is>
+      </c>
+      <c r="K294" s="2" t="inlineStr">
+        <is>
+          <t>TAG Data Science &amp; AI Society event with explicit AI content (AI in Healthcare) hosted by a Georgia organization with clear Georgia tie, meeting the criteria for automatic 5 on TAG events with genuine AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Data After Dark / Analytically Yours: Where the Data &amp; AI Community Connects After presented by TAG Data Science &amp; AI Society</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>4</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="n">
+        <v>46338</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>5:30 PM</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr"/>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/WqFjkzjuaCJCE</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="inlineStr">
+        <is>
+          <t>An evening designed to bring Atlanta's data, analytics, and AI community together for meaningful connections and conversations. Network with professionals, exchange ideas, expand your network, and participate in nominations for Innovator of the Year Awards.</t>
+        </is>
+      </c>
+      <c r="K295" s="2" t="inlineStr">
+        <is>
+          <t>TAG Data Science &amp; AI Society event with clear AI community focus and networking purpose, hosted by Georgia's most valued source, but scored 4 rather than 5 because it is primarily a networking/social event rather than an in-person AI builder/demo event with technical content and project presentations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>TAG AI Summit: The AI-Powered Enterprise</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>5</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D296" s="3" t="n">
+        <v>46343</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>8:00 AM</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/OOFvaqjSaCqCD</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="inlineStr">
+        <is>
+          <t>The TAG Data Science &amp; AI Summit 2026 is a full-day Atlanta experience connecting executive strategy with applied implementation.</t>
+        </is>
+      </c>
+      <c r="K296" s="2" t="inlineStr">
+        <is>
+          <t>This is a TAG Data Science &amp; AI Summit with explicit AI content (executive strategy and applied implementation), hosted by TAG (the client's most valued source), in-person in Atlanta, which qualifies for the automatic 5-point TAG uplift for events with genuine AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>https://www.aimanufacturingconference.com/</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr"/>
+      <c r="C297" t="inlineStr"/>
+      <c r="D297" s="3" t="inlineStr"/>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr"/>
+      <c r="G297" t="inlineStr"/>
+      <c r="H297" t="inlineStr"/>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J297" s="2" t="inlineStr"/>
+      <c r="K297" s="2" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>FREE REMOTE | LADIES IN AI + AI GROWTH CIRCLE (AN OPEN AI FORUM FOR ALL)</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>2</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D298" s="3" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/315939829/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-online&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J298" s="2" t="inlineStr">
+        <is>
+          <t>A collaborative community where members of all backgrounds and experience levels learn and share about AI. Topics include basic AI concepts, advanced tools, automation, prompting, business applications, productivity, and emerging technologies. Members bring questions, tools, use cases, and lessons to help each other grow in AI.</t>
+        </is>
+      </c>
+      <c r="K298" s="2" t="inlineStr">
+        <is>
+          <t>Virtual-only event with genuine AI content (basic concepts, tools, automation, prompting, business applications) hosted by AI Growth Circle, but no clear Georgia organizational tie, so it caps at 2 per the virtual-event rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>AI COMMUNITY NIGHT - Tuesdays @7pm (FREE|Remote) - a group-led event</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>2</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ai-growth-circle/events/317016310/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-online&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>A casual, community-led space to connect, share ideas, and help each other move forward with AI. Bring something you're working on, a question, a tool to demo, or just yourself. Conversations include AI show-and-tell, project feedback, troubleshooting, job opportunities, and catching up with community members. Self-organized with no designated facilitator or set agenda. All experience levels welco</t>
+        </is>
+      </c>
+      <c r="K299" s="2" t="inlineStr">
+        <is>
+          <t>This is a virtual-only AI community event with genuine AI content (show-and-tell, project feedback, tool demos), but it lacks a clear Georgia organizational tie and scores at the virtual-only cap of 2-3 without additional Georgia context to elevate it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Monthly Meetup + Demo Night: October 2026</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>5</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D300" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>7:00 PM EDT</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr"/>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atl-ai/events/314482325/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J300" s="2" t="inlineStr"/>
+      <c r="K300" s="2" t="inlineStr">
+        <is>
+          <t>This is an in-person AI builder event (demo night) hosted by Atlanta AI Tinkerers, a Georgia-based organization, which scores 5 per the criteria even with minimal description details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Delta Airlines - AI in Action</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>4</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D301" s="3" t="n">
+        <v>46338</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>10:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr"/>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/317012340/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="inlineStr">
+        <is>
+          <t>Delta Air Lines showcases how AI is being applied across the enterprise to enhance customer and employee experiences, enable airline operations, and deliver business value. Through presentations and demonstrations from business leaders, attendees will gain insight into real-world AI use cases and Delta's approach to responsible adoption, governance, and stewardship of technology innovation.</t>
+        </is>
+      </c>
+      <c r="K301" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (enterprise AI applications, real-world use cases, governance) hosted by Georgia AI Alliance (Georgia tie), in-person format, but missing venue details and no indication this is a recurring builder-focused community event that would warrant a 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Changing Landscape of UX: AI in Practice</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>4</v>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D302" s="3" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr"/>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/ixdaatlanta/events/316575374/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr">
+        <is>
+          <t>A practical conversation about how UX, product, research, design and technology professionals are using AI in their work today. Panelists will share how they're incorporating AI into workflows, what's working, what's changing, and where human judgment still matters most. Includes moderated panel, audience Q&amp;A, and networking.</t>
+        </is>
+      </c>
+      <c r="K302" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta-based UX/design meetup with genuine AI content (practical panel discussion on AI in professional workflows), in-person format, and networking component, but not a builder-focused event so scores 4 rather than 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr"/>
+      <c r="C303" t="inlineStr"/>
+      <c r="D303" s="3" t="inlineStr"/>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr"/>
+      <c r="G303" t="inlineStr"/>
+      <c r="H303" t="inlineStr"/>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="inlineStr"/>
+      <c r="K303" s="2" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>AI. Content. Vibes.</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>4</v>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D304" s="3" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Georgia · 3565 GA-20 suite d</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-content-vibes-tickets-2003402994286?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>A one-day content creation experience for entrepreneurs and business owners. Attendees will create and capture professional content while learning AI automation. Leave with 5 edited videos, 5 professional photos, a content calendar, and one free business automation setup.</t>
+        </is>
+      </c>
+      <c r="K304" s="2" t="inlineStr">
+        <is>
+          <t>In-person Georgia event with genuine AI content (learning AI automation, business automation setup) focused on practical application for entrepreneurs, though not a pure builder community event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>AI Tinkerers Atlanta — Community Demos (Oct 29)</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>5</v>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D305" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>4:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>https://atlanta.aitinkerers.org/p/ai-tinkerers-atlanta-community-demos-oct-29</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="inlineStr">
+        <is>
+          <t>AI Tinkerers Atlanta will showcase live, code-first AI implementations. Attendees will see working agents, retrieval engines, and performance optimizations.</t>
+        </is>
+      </c>
+      <c r="K305" s="2" t="inlineStr">
+        <is>
+          <t>This is an in-person AI builder event in Georgia hosted by Atlanta AI Tinkerers (a recognized Georgia organization) featuring live code-first AI implementations and community demos, which matches the client's highest-priority event type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>From AI Idea to Executable Use Case Workshop</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>4</v>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D306" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>10:00 a.m.</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>https://ai.georgia.gov/events/2026-10-29/ai-idea-executable-use-case</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>An interactive 90-minute workshop for public-sector leaders to move from AI ideas toward actionable use cases. Participants will learn to identify, evaluate, and prioritize AI opportunities, covering value, feasibility, risk, data readiness, responsible AI, and governance through facilitated discussion and applied activities.</t>
+        </is>
+      </c>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>A genuine AI-focused educational workshop hosted by ai.georgia.gov (Georgia state organization with clear AI content: identifying, evaluating, and prioritizing AI use cases), in-person in Atlanta, though not a builder/demo event so does not reach the 5-point ceiling for those.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13900,7 +14484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K433"/>
+  <dimension ref="A1:K445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -34502,7 +35086,6 @@
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="G423" t="inlineStr"/>
       <c r="H423" t="inlineStr">
         <is>
           <t>https://www.georgiamanufacturingalliance.com/events/women-of-gma-virtual-networking-event-10326</t>
@@ -34547,7 +35130,6 @@
           <t>10:30 AM EDT</t>
         </is>
       </c>
-      <c r="G424" t="inlineStr"/>
       <c r="H424" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-data-science-bootcamp-usa-only-live-training-join-whatsapp-group-tickets-2002085679161?aff=ebdssbdestsearch</t>
@@ -34936,8 +35518,6 @@
           <t>October 12, 2026</t>
         </is>
       </c>
-      <c r="F432" t="inlineStr"/>
-      <c r="G432" t="inlineStr"/>
       <c r="H432" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/cybersecurity-ethical-hacking-blue-team-red-team-free-live-online-tickets-2003205772390?aff=ebdssbdestsearch</t>
@@ -34982,7 +35562,6 @@
           <t>5:30 pm</t>
         </is>
       </c>
-      <c r="G433" t="inlineStr"/>
       <c r="H433" t="inlineStr">
         <is>
           <t>https://technorthatlanta.org/event/private-event-members-only-happy-hour/</t>
@@ -35001,6 +35580,590 @@
       <c r="K433" s="2" t="inlineStr">
         <is>
           <t>This is a members-only mixer with no AI content mentioned in the title or description, making it ineligible regardless of host or location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>TAGit 2027 Golf Tournament</t>
+        </is>
+      </c>
+      <c r="B434" t="n">
+        <v>1</v>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D434" s="3" t="n">
+        <v>46552</v>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>7:00 AM</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr"/>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/calendar/Details/tagit-2027-golf-tournament-1960549?sourceTypeId=Website</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J434" s="2" t="inlineStr">
+        <is>
+          <t>TAG's 2026 Southern Company TAGit Global Innovation Cup Golf Tournament sponsored by Softensity is the state's most prestigious golf tournament for technology stakeholders. The day is filled with networking, fun, prizes and awards.</t>
+        </is>
+      </c>
+      <c r="K434" s="2" t="inlineStr">
+        <is>
+          <t>This event has zero mention of AI, machine learning, or automation in its title or description—it is a golf tournament focused on networking and socializing, not an AI-focused component or educational session, triggering the automatic-1 rule regardless of TAG's hosting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026 Bar-B-Que and Bowling Party - Dacula</t>
+        </is>
+      </c>
+      <c r="B435" t="n">
+        <v>1</v>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D435" s="3" t="n">
+        <v>46385</v>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>6:00 PM EST</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>Dacula, Georgia</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/2026-bar-b-que-and-bowling-party---dacula</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J435" s="2" t="inlineStr"/>
+      <c r="K435" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule; it is a social gathering (bar-b-que and bowling) with no stated AI content component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Bytes &amp; Bites @ Krog St Market</t>
+        </is>
+      </c>
+      <c r="B436" t="n">
+        <v>1</v>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D436" s="3" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>11:45 AM EDT</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>Krog St Market</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/refactr-tech/events/315803183/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J436" s="2" t="inlineStr">
+        <is>
+          <t>A casual, community-driven monthly lunch where technologists of all backgrounds connect, swap ideas, and build relationships over good food. No agenda—just lunch and conversation for tech folks at any career level.</t>
+        </is>
+      </c>
+      <c r="K436" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, automation, or any technical topic beyond a generic "tech folks" networking lunch, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Open House!</t>
+        </is>
+      </c>
+      <c r="B437" t="n">
+        <v>1</v>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D437" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>7:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr"/>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/freeside-atlanta/events/312398750/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J437" s="2" t="inlineStr">
+        <is>
+          <t>A 501(c)(3) non-profit meetup for engineers, programmers, inventors, artists to collaborate. Features a quick introduction meeting with project updates and occasional guest lectures, followed by an informal open house with tours and networking.</t>
+        </is>
+      </c>
+      <c r="K437" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it describes a general engineering and maker meetup with no AI-focused component, session, speaker, or theme stated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Atlanta Tech Meet-Up</t>
+        </is>
+      </c>
+      <c r="B438" t="n">
+        <v>1</v>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D438" s="3" t="n">
+        <v>46329</v>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>6:00 PM EST</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr"/>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atl-tech-meetup/events/316377764/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J438" s="2" t="inlineStr"/>
+      <c r="K438" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of the meetup's general focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>FREE Cybersecurity: Ethical Hacking, Blue Team &amp; Red Team | Live Online-UK</t>
+        </is>
+      </c>
+      <c r="B439" t="n">
+        <v>1</v>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D439" s="3" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>2:30 AM GMT+0</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr"/>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/free-cybersecurity-ethical-hacking-blue-team-red-team-live-online-uk-tickets-2003619988321?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J439" s="2" t="inlineStr"/>
+      <c r="K439" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, covering only cybersecurity and ethical hacking topics, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Music of the Spheres II: An Immersive Experience with Live Choral Music</t>
+        </is>
+      </c>
+      <c r="B440" t="n">
+        <v>1</v>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D440" s="3" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>8:00 PM</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>Young Harris · O. Wayne Rollins Planetarium</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/music-of-the-spheres-ii-an-immersive-experience-with-live-choral-music-tickets-1998990016952?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J440" s="2" t="inlineStr"/>
+      <c r="K440" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is an immersive choral music experience at a planetarium with no stated AI component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>PMP Certification Training in Augusta, GA | PMI Exam Prep</t>
+        </is>
+      </c>
+      <c r="B441" t="n">
+        <v>1</v>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D441" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>Greene Street Historic District · 823 Broad St</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/pmp-certification-training-in-augusta-ga-pmi-exam-prep-tickets-1973124928777?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J441" s="2" t="inlineStr"/>
+      <c r="K441" s="2" t="inlineStr">
+        <is>
+          <t>The event is PMP certification training with no mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>PMP Certification Training in Atlanta, GA | PMI Exam Prep</t>
+        </is>
+      </c>
+      <c r="B442" t="n">
+        <v>1</v>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D442" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>Downtown · 260 Peachtree St suite 2200</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/pmp-certification-training-in-atlanta-ga-pmi-exam-prep-tickets-1973135226578?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J442" s="2" t="inlineStr"/>
+      <c r="K442" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description—it is PMP certification training, a project management credential with no AI component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B443" t="n">
+        <v>1</v>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D443" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>Linwood Heights · East Point Library</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J443" s="2" t="inlineStr"/>
+      <c r="K443" s="2" t="inlineStr">
+        <is>
+          <t>This is a youth robotics outreach and build program focused on hardware and STEM instruction rather than AI content, which per the criteria scores 1 regardless of the AI mention in the title.</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B444" t="n">
+        <v>1</v>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D444" s="3" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>Georgia · Browns Mill Recreation Center</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J444" s="2" t="inlineStr"/>
+      <c r="K444" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule regardless of location or other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Tech Women of ATL CoWork</t>
+        </is>
+      </c>
+      <c r="B445" t="n">
+        <v>1</v>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D445" s="3" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>October 19, 2026</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>Grant Park · Condesa Coffee</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tech-women-of-atl-cowork-tickets-2003545310959?aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J445" s="2" t="inlineStr"/>
+      <c r="K445" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rule regardless of other factors.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update state - 2026-10-26
</commit_message>
<xml_diff>
--- a/events_master.xlsx
+++ b/events_master.xlsx
@@ -134,7 +134,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K306" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EventsTable" displayName="EventsTable" ref="A1:K316" headerRowCount="1">
   <autoFilter ref="A1:K53"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K445" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RejectedEventsTable" displayName="RejectedEventsTable" ref="A1:K458" headerRowCount="1">
   <autoFilter ref="A1:K132"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Event Title"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K306"/>
+  <dimension ref="A1:K316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -13888,7 +13888,6 @@
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="G294" t="inlineStr"/>
       <c r="H294" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/EqFMN30tgC6C9</t>
@@ -13937,7 +13936,6 @@
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="G295" t="inlineStr"/>
       <c r="H295" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/ap/Events/Register/WqFjkzjuaCJCE</t>
@@ -14018,17 +14016,12 @@
           <t>https://www.aimanufacturingconference.com/</t>
         </is>
       </c>
-      <c r="B297" t="inlineStr"/>
-      <c r="C297" t="inlineStr"/>
       <c r="D297" s="3" t="inlineStr"/>
       <c r="E297" t="inlineStr">
         <is>
           <t>October 19, 2026</t>
         </is>
       </c>
-      <c r="F297" t="inlineStr"/>
-      <c r="G297" t="inlineStr"/>
-      <c r="H297" t="inlineStr"/>
       <c r="I297" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -14170,7 +14163,6 @@
           <t>7:00 PM EDT</t>
         </is>
       </c>
-      <c r="G300" t="inlineStr"/>
       <c r="H300" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atl-ai/events/314482325/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
@@ -14215,7 +14207,6 @@
           <t>10:00 AM EST</t>
         </is>
       </c>
-      <c r="G301" t="inlineStr"/>
       <c r="H301" t="inlineStr">
         <is>
           <t>https://www.meetup.com/georgia-ai-alliance-meetup-group/events/317012340/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
@@ -14264,7 +14255,6 @@
           <t>6:30 PM EDT</t>
         </is>
       </c>
-      <c r="G302" t="inlineStr"/>
       <c r="H302" t="inlineStr">
         <is>
           <t>https://www.meetup.com/ixdaatlanta/events/316575374/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
@@ -14292,17 +14282,12 @@
           <t>https://luma.com/genai-collective</t>
         </is>
       </c>
-      <c r="B303" t="inlineStr"/>
-      <c r="C303" t="inlineStr"/>
       <c r="D303" s="3" t="inlineStr"/>
       <c r="E303" t="inlineStr">
         <is>
           <t>October 19, 2026</t>
         </is>
       </c>
-      <c r="F303" t="inlineStr"/>
-      <c r="G303" t="inlineStr"/>
-      <c r="H303" t="inlineStr"/>
       <c r="I303" t="inlineStr">
         <is>
           <t>no_events</t>
@@ -14467,6 +14452,490 @@
       <c r="K306" s="2" t="inlineStr">
         <is>
           <t>A genuine AI-focused educational workshop hosted by ai.georgia.gov (Georgia state organization with clear AI content: identifying, evaluating, and prioritizing AI use cases), in-person in Atlanta, though not a builder/demo event so does not reach the 5-point ceiling for those.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>AIMST 2027 Atlanta</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>4</v>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D307" s="3" t="inlineStr">
+        <is>
+          <t>August 30 - September 1, 2027</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Renaissance Atlanta Waverly Hotel &amp; Convention Center, 2450 Galleria Pkwy, Atlanta, GA 30339</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>https://twstevents.meetmax.com/AIMST_attendee</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>North America's #1 conference in Industrial AI, focused on providing in-depth discussions and solutions for heads of manufacturing, advanced technology managers, ICS, IT/OT, SCADA, and cybersecurity professionals to accelerate their digital transformation and transform their operational and automation systems.</t>
+        </is>
+      </c>
+      <c r="K307" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI conference in Atlanta with clear industrial AI focus, strong relevance to automation and digital transformation, multi-day format, and established event series, though not a builder-focused hands-on event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>We're Gonna Need a Bigger Lab: AI-Assisted CVE Hunting from Repo to Real World</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>4</v>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D308" s="3" t="n">
+        <v>46345</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>6:00 PM EST</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/owasp-atlanta/events/316997081/?recId=2f1a3733-0527-4693-8a9a-7ad088930890&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=1a83f45e-702b-492a-adf4-b83dc139dbf9&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>Two researchers share practical approaches to finding CVEs using AI as a working partner. One covers open-source vulnerability research using AI-assisted code review, while the other discusses reverse engineering closed-source targets from a real penetration test. Learn where AI accelerates research, where it fails, and how to maintain human validation throughout the process.</t>
+        </is>
+      </c>
+      <c r="K308" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI content (AI-assisted security research with practical applications) hosted by OWASP Atlanta, in-person in Georgia, but not a builder/hands-on demo event which would score 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Mastering ChatGPT</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>4</v>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="n">
+        <v>46340</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>10:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr"/>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlanta-ai-builders/events/317059963/?recId=2f1a3733-0527-4693-8a9a-7ad088930890&amp;recSource=ml-popular-events-nearby-online&amp;searchId=1a83f45e-702b-492a-adf4-b83dc139dbf9&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>A live, hands-on online workshop exploring Dots, Agents, Astra 6, Skills, and Codex. Learn to use AI for productivity, research, content creation, and business tasks through guided demonstrations, practical examples, and exercises. Topics include better prompting, reusable workflows, and coding with Codex. Designed for professionals, business owners, creators, and curious learners with no coding b</t>
+        </is>
+      </c>
+      <c r="K309" s="2" t="inlineStr">
+        <is>
+          <t>Atlanta AI Builders is a Georgia-based AI builder community hosting a hands-on ChatGPT workshop with practical AI applications, which qualifies as an in-person builder event despite the virtual-only format, and scores 4 rather than 5 only because it is virtual rather than in-person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>https://luma.com/genai-collective</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr"/>
+      <c r="C310" t="inlineStr"/>
+      <c r="D310" s="3" t="inlineStr"/>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr"/>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr"/>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>no_events</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr"/>
+      <c r="K310" s="2" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Create AI-Powered Online Course Curriculums That People Want to Buy</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>2</v>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>10:00 AM PDT</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr"/>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/create-ai-powered-online-course-curriculums-that-people-want-to-buy-tickets-2001869092344?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=2001869092344&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>Learn to design powerful online courses using AI and human expertise that deliver results, keep clients engaged, and drive sales. Explore balancing your unique human connection with AI tools to create engaging course content, clear instructions, and step-by-step structures that clients will be excited to buy.</t>
+        </is>
+      </c>
+      <c r="K311" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (using AI tools to create course curriculums) but is virtual-only (PDT time zone, no Georgia host, no Georgia tie mentioned), lacks a specific location, and appears to be a sales-focused workshop rather than an educational or builder-focused event, which caps it at 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>AI SAFETY LAB - SILICON VALLEY</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>4</v>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D312" s="3" t="n">
+        <v>46321</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>3:00 PM</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Atlanta · Atlanta Convention Center at AmericasMart</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-safety-lab-silicon-valley-tickets-1985762152052?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=1985762480033&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>A live online AI safety workshop where participants learn how to use AI safely, minimize privacy and security risks, and responsibly use AI. Topics include core AI safety principles, common implementation risks, real-world AI failures, and risk mitigation strategies. Features live Q&amp;A with an AI safety expert.</t>
+        </is>
+      </c>
+      <c r="K312" s="2" t="inlineStr">
+        <is>
+          <t>Strong AI safety content in Atlanta in-person, but the contradictory 'live online' language in the description creates ambiguity about the actual format that prevents a higher score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>AI &amp; Robotics for Youth and Teens: The Smart Machines Program (ages 8 - 16)</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>4</v>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D313" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>East Point · East Point Library</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/ai-robotics-for-youth-and-teens-the-smart-machines-program-ages-8-16-tickets-1999165834828?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=1999165863915&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J313" s="2" t="inlineStr">
+        <is>
+          <t>A weekly hands-on program introducing youth and teens to robotics, artificial intelligence, engineering thinking, and creative problem-solving. Students explore real robots, virtual robotics environments, and beginner-friendly AI tools while completing challenges that build confidence and technical skills.</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI and robotics hands-on program for youth in East Point (outside metro Atlanta), with genuine AI content including AI tools and machine learning concepts, though the youth/educational focus and robotics-heavy framing prevent a perfect score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Build Production-Ready Agents with Claude Code</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>2</v>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D314" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>10:00 AM EDT</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.co.uk/e/build-production-ready-agents-with-claude-code-tickets-1998636083327?dsrp_sid=5172cc76-8f21-492e-a2bc-fad0bcd19f2f&amp;dsrp_item_id=1998636083327&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J314" s="2" t="inlineStr">
+        <is>
+          <t>Build and evaluate Claude agents, add production controls, test failure modes, and leave with an evidence-based deployment assessment. Learn to define correct agent behavior before coding, redesign agents into specialized subagents, and measure cost and quality differences to prove agent reliability.</t>
+        </is>
+      </c>
+      <c r="K314" s="2" t="inlineStr">
+        <is>
+          <t>The event has genuine AI content (Claude agents, production deployment) but lacks location information and shows no Georgia tie, and the signup link suggests a UK Eventbrite domain which may indicate a non-Georgia or virtual event, making it impossible to confirm in-person Georgia attendance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>BitPlebs Bitcoin Meetup @ ATL BitLab</t>
+        </is>
+      </c>
+      <c r="B315" t="n">
+        <v>5</v>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="n">
+        <v>46337</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>6:00 PM EST</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>684 John Wesley Dobbs Ave NE suite a1, Atlanta, GA, US</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/atlbitlab/events/317134789/?eventOrigin=group_events_list</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="inlineStr">
+        <is>
+          <t>Join us at ATL BitLab for another fun BitPlebs meetup. Sovereign Cinema: Making AI Films on Your Own Hardware. We'll screen an AI storybook video of 'The Sovereign Cross,' generated with local image and voice models on two DGX Sparks, then open the floor: How was it made? What does self-hosted AI mean for creators? Bring your questions.</t>
+        </is>
+      </c>
+      <c r="K315" s="2" t="inlineStr">
+        <is>
+          <t>In-person AI builder event in Georgia (ATL BitLab) featuring a hands-on demonstration of self-hosted AI for creative applications with Q&amp;A and networking, hosted by a Georgia-based organization that the client values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>AI Builders Meetup</t>
+        </is>
+      </c>
+      <c r="B316" t="n">
+        <v>5</v>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D316" s="3" t="n">
+        <v>46364</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr"/>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/1998165965191?aff=oddtdtcreator</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="inlineStr">
+        <is>
+          <t>Join us for a live show-and-tell where 5-7 AI builders share what they're building, how they're building it (approach, tools and tech stacks), and real lessons learned along the way. Come for the demos - stay for the conversations!</t>
+        </is>
+      </c>
+      <c r="K316" s="2" t="inlineStr">
+        <is>
+          <t>This is an in-person AI builder meetup in Georgia (based on the Eventbrite link pattern and event type) featuring 5-7 builders presenting their own AI projects with tools, tech stacks, and lessons learned, followed by networking—exactly matching the client's highest-priority event type.</t>
         </is>
       </c>
     </row>
@@ -14484,7 +14953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K445"/>
+  <dimension ref="A1:K458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -35610,7 +36079,6 @@
           <t>7:00 AM</t>
         </is>
       </c>
-      <c r="G434" t="inlineStr"/>
       <c r="H434" t="inlineStr">
         <is>
           <t>https://members.tagonline.org/calendar/Details/tagit-2027-golf-tournament-1960549?sourceTypeId=Website</t>
@@ -35761,7 +36229,6 @@
           <t>7:30 PM EDT</t>
         </is>
       </c>
-      <c r="G437" t="inlineStr"/>
       <c r="H437" t="inlineStr">
         <is>
           <t>https://www.meetup.com/freeside-atlanta/events/312398750/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
@@ -35810,7 +36277,6 @@
           <t>6:00 PM EST</t>
         </is>
       </c>
-      <c r="G438" t="inlineStr"/>
       <c r="H438" t="inlineStr">
         <is>
           <t>https://www.meetup.com/atl-tech-meetup/events/316377764/?recId=148a871b-5701-4562-950f-af3268cc9595&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=da848962-7fea-437b-817a-1481c89c24ef&amp;eventOrigin=find_page%24all</t>
@@ -35855,7 +36321,6 @@
           <t>2:30 AM GMT+0</t>
         </is>
       </c>
-      <c r="G439" t="inlineStr"/>
       <c r="H439" t="inlineStr">
         <is>
           <t>https://www.eventbrite.com/e/free-cybersecurity-ethical-hacking-blue-team-red-team-live-online-uk-tickets-2003619988321?aff=ebdssbdestsearch</t>
@@ -36164,6 +36629,635 @@
       <c r="K445" s="2" t="inlineStr">
         <is>
           <t>The event has zero mention of AI, machine learning, or automation in its title or description, triggering the automatic 1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Georgia Rural Health Transformation presented by TAG Digital Health Society</t>
+        </is>
+      </c>
+      <c r="B446" t="n">
+        <v>1</v>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D446" s="3" t="n">
+        <v>46335</v>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>5:30 PM - 7:30 PM</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr"/>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/eZF9dANTYCWCq</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J446" s="2" t="inlineStr">
+        <is>
+          <t>As Georgia's Department of Community Health advances the Georgia Rural Enhancement and Transformation of Health (GREAT) Program and directs funding, this panel will explore what these investments could mean for rural communities.</t>
+        </is>
+      </c>
+      <c r="K446" s="2" t="inlineStr">
+        <is>
+          <t>The event description contains zero mention of AI, machine learning, or automation—it is exclusively about rural health policy and funding, and despite being hosted by TAG Digital Health Society, the event's own title and description lack any genuine AI-focused component, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>2026 TAG Society Holiday Party</t>
+        </is>
+      </c>
+      <c r="B447" t="n">
+        <v>1</v>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D447" s="3" t="n">
+        <v>46336</v>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>6:00 PM - 8:00 PM</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr"/>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>https://members.tagonline.org/ap/Events/Register/DgFZozoF1CQCW</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J447" s="2" t="inlineStr">
+        <is>
+          <t>Where Innovation Meets Celebration.</t>
+        </is>
+      </c>
+      <c r="K447" s="2" t="inlineStr">
+        <is>
+          <t>This is a TAG holiday party with no mention of AI, machine learning, or automation in the title or description, making it an automatic 1 regardless of the host organization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>EP American Footwear, McPherson Manufacturing Corporation, South Georgia Cotton Gin and Mary Hill Dumpling Shoppe Plant Tours - Hazlehurst</t>
+        </is>
+      </c>
+      <c r="B448" t="n">
+        <v>1</v>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D448" s="3" t="n">
+        <v>46401</v>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>10:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>Hazlehurst</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/mcpherson-manufacturing-corporation-south-georgia-cotton-gin-and-mary-hill-dumpling-shoppe-plant-tours--hazlehurst</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J448" s="2" t="inlineStr"/>
+      <c r="K448" s="2" t="inlineStr">
+        <is>
+          <t>The event is plant tours of manufacturing facilities with no mention of AI, machine learning, or automation in the title or description, triggering the automatic-1 rule despite being hosted by the Georgia Manufacturing Alliance in Hazlehurst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>WGMA Collins Manufacturing Plant Tour- Macon</t>
+        </is>
+      </c>
+      <c r="B449" t="n">
+        <v>1</v>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D449" s="3" t="n">
+        <v>46406</v>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>10:00 AM EST</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>Macon</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>https://www.georgiamanufacturingalliance.com/events/wgma-collins-manufacturing-plant-tour--macon</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J449" s="2" t="inlineStr"/>
+      <c r="K449" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a manufacturing plant tour with no stated AI-focused component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Ethical Hacker Tactics, CTF &amp; Tech Talks Monthly by BlackHack Society</t>
+        </is>
+      </c>
+      <c r="B450" t="n">
+        <v>1</v>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D450" s="3" t="n">
+        <v>46331</v>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>6:30 PM EST</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/blackhack-society-atlanta/events/316426916/?recId=2f1a3733-0527-4693-8a9a-7ad088930890&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=1a83f45e-702b-492a-adf4-b83dc139dbf9&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J450" s="2" t="inlineStr"/>
+      <c r="K450" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain no mention of AI, machine learning, or automation—it is about ethical hacking, CTF (Capture The Flag) competitions, and general tech talks, which do not constitute genuine AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>BHS X Sandbox Atlanta Present: CTF Training for First-timers</t>
+        </is>
+      </c>
+      <c r="B451" t="n">
+        <v>1</v>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D451" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/blackhack-society-atlanta/events/317060515/?recId=2f1a3733-0527-4693-8a9a-7ad088930890&amp;recSource=ml-popular-events-nearby-offline&amp;searchId=1a83f45e-702b-492a-adf4-b83dc139dbf9&amp;eventOrigin=find_page%24all</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J451" s="2" t="inlineStr">
+        <is>
+          <t>Learn basic concepts and strategies for capture-the-flag contests and Network King of the Hill events. This training covers recon and post-exploitation techniques for beginners. Bring a computer with Kali Linux installed.</t>
+        </is>
+      </c>
+      <c r="K451" s="2" t="inlineStr">
+        <is>
+          <t>This is a cybersecurity/CTF (capture-the-flag) training event with zero mention of AI, machine learning, or automation in its title or description, making it an automatic 1 regardless of location or host.</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Launch Your Career in AI &amp; Emerging Tech-Cyber Work Roles at UofL DTC</t>
+        </is>
+      </c>
+      <c r="B452" t="n">
+        <v>1</v>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D452" s="3" t="n">
+        <v>46324</v>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>6:30 PM EDT</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>University of Louisville</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/launch-your-career-in-ai-emerging-tech-cyber-work-roles-at-uofl-dtc-tickets-2002449837368?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=2002449837368&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J452" s="2" t="inlineStr"/>
+      <c r="K452" s="2" t="inlineStr">
+        <is>
+          <t>The event is hosted by University of Louisville, which is in Kentucky, not Georgia, and no event description is provided to verify AI content exists beyond the title's mention of 'AI &amp; Emerging Tech,' making it impossible to assess the event's genuine AI focus and placing it outside the client's geographic scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>PMP Certification Training in Augusta, GA | PMI Exam Prep</t>
+        </is>
+      </c>
+      <c r="B453" t="n">
+        <v>1</v>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D453" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>Augusta · 823 Broad St</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/pmp-certification-training-in-augusta-ga-pmi-exam-prep-tickets-1973124928777?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=2002756608930&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J453" s="2" t="inlineStr"/>
+      <c r="K453" s="2" t="inlineStr">
+        <is>
+          <t>The event is PMP certification training with no mention of AI, machine learning, or automation in its title or description, triggering the automatic-1 rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>PMP Certification Training in Atlanta, GA | PMI Exam Prep</t>
+        </is>
+      </c>
+      <c r="B454" t="n">
+        <v>1</v>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D454" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>Atlanta · 260 Peachtree St suite 2200</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/pmp-certification-training-in-atlanta-ga-pmi-exam-prep-tickets-1973135226578?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=2002958916036&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J454" s="2" t="inlineStr"/>
+      <c r="K454" s="2" t="inlineStr">
+        <is>
+          <t>The event is PMP (Project Management Professional) certification training with no mention of AI, machine learning, or automation in the title or description, triggering the automatic-1 rule for events with zero AI content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>"STARTUP-INVESTOR PITCH LUNCH" - FUNDRAISING PROGRAM IN SILICON VALLEY</t>
+        </is>
+      </c>
+      <c r="B455" t="n">
+        <v>1</v>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D455" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>10:00 AM</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr"/>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/startup-investor-pitch-lunch-fundraising-program-in-silicon-valley-tickets-1992323518275?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=1992323654683&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J455" s="2" t="inlineStr"/>
+      <c r="K455" s="2" t="inlineStr">
+        <is>
+          <t>Event has zero mention of AI, machine learning, or automation in its title or description, and is located in Silicon Valley (California), not Georgia, making it ineligible for the digest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Tap Into Tech with Seniors</t>
+        </is>
+      </c>
+      <c r="B456" t="n">
+        <v>1</v>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D456" s="3" t="n">
+        <v>46322</v>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>9:30 AM</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>Stonecrest · Browns Mill Recreation Center</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/tap-into-tech-with-seniors-tickets-1984059620735?dsrp_sid=b64e283e-37ff-43a7-ae99-b4473c723129&amp;dsrp_item_id=1984059772188&amp;aff=ebdssbdestsearch</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J456" s="2" t="inlineStr"/>
+      <c r="K456" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule regardless of other factors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Startup Workshop: Startup Operational Benchmarks &amp; Best Practices</t>
+        </is>
+      </c>
+      <c r="B457" t="n">
+        <v>1</v>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D457" s="3" t="n">
+        <v>46345</v>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>12:00 PM - 1:00 PM</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr"/>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>https://www.eventbrite.com/e/2003771229688?aff=oddtdtcreator</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J457" s="2" t="inlineStr"/>
+      <c r="K457" s="2" t="inlineStr">
+        <is>
+          <t>The event title and description contain zero mention of AI, machine learning, or automation, triggering the automatic-1 rule; it is a general startup operational workshop with no stated AI-focused component, session, panel, or speaker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Holiday Mixer</t>
+        </is>
+      </c>
+      <c r="B458" t="n">
+        <v>1</v>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D458" s="3" t="n">
+        <v>46365</v>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>October 26, 2026</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>5:30 PM - 8:30 PM</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr"/>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>https://technorthatlanta.org/event/holiday-mixer-2/</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="J458" s="2" t="inlineStr"/>
+      <c r="K458" s="2" t="inlineStr">
+        <is>
+          <t>The event has zero mention of AI, machine learning, or automation in its title or description—it is a holiday mixer with no stated AI content, triggering the automatic-1 rule.</t>
         </is>
       </c>
     </row>

</xml_diff>